<commit_message>
Append 2026h1 PDF and Word outlines to cumulative course database
</commit_message>
<xml_diff>
--- a/course-outline-database/UCR_Course_Outline_Database.xlsx
+++ b/course-outline-database/UCR_Course_Outline_Database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="1" r:id="R509d54b91d414040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="1" r:id="R566cc85d65a942de"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2475,6 +2475,2236 @@
       </x:c>
       <x:c r="L64"/>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>BENBUSI211</x:v>
+      </x:c>
+      <x:c r="C65" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>Business &amp; Economy in the Age of AI</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>Examines AI's business, economic and societal implications without requiring a technical background. AI foundations and limitations lead into applications across enterprise functions and industries, labour-market change, productivity, innovation, market structure and inequality. Governance, corporate responsibility, regulation and future scenarios connect technological developments to institutional choices. Students analyze business cases and competing scholarly arguments, then investigate a country's AI readiness, workforce, regulation and industrial policy.</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>Business studies; Economics; Technology governance</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>AI capabilities and limitations; AI in business functions and industries; Agentic AI; Market structure and business models; Automation and augmentation; Labour markets and productivity; Innovation and economic growth; Inequality; Techno-economic paradigms and economic narratives; AI ethics and societal impacts; Corporate governance and AI regulation; National AI readiness and industrial policy; Future AI scenarios</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>Business-case analysis; Comparative analysis of economic arguments; Evidence-based policy argumentation; Comparative country AI-readiness analysis</x:v>
+      </x:c>
+      <x:c r="I65" t="str">
+        <x:v>BENBUSI211.pdf</x:v>
+      </x:c>
+      <x:c r="J65" t="str">
+        <x:v>a6e7fef5481d1bbcc8be694343d7b3ebe83b51486b2a8836b36a057dd55f8ffd</x:v>
+      </x:c>
+      <x:c r="K65"/>
+      <x:c r="L65"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B66" t="str">
+        <x:v>BENBUSI311</x:v>
+      </x:c>
+      <x:c r="C66" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D66" t="str">
+        <x:v>Transnational Business Law</x:v>
+      </x:c>
+      <x:c r="E66" t="str">
+        <x:v>Studies legal frameworks governing cross-border business transactions, combining comparative and international perspectives with practical legal problem-solving. Topics include trade regulation, contracts and international sales, transport and documentary transactions, finance, services, intellectual property, foreign investment and digital commerce. Advisory assignments assess contractual outcomes, risk allocation, intellectual-property protection and e-commerce compliance. A simulated arbitration develops written legal argument and oral advocacy.</x:v>
+      </x:c>
+      <x:c r="F66" t="str">
+        <x:v>International business law; Comparative law; Commercial law</x:v>
+      </x:c>
+      <x:c r="G66" t="str">
+        <x:v>International trade regulation; Comparative and international contract law; International sales; Transport of goods and Incoterms; Documentary transactions; International trade finance; Employment and sale of services; Intellectual-property protection; International commercial dispute resolution; Foreign direct investment; E-commerce and digital economy regulation</x:v>
+      </x:c>
+      <x:c r="H66" t="str">
+        <x:v>Comparative legal analysis; Application of legal rules to commercial scenarios; Transport-risk allocation analysis; Intellectual-property strategy assessment; E-commerce legal-compliance analysis; Arbitration memorandum drafting and simulated advocacy</x:v>
+      </x:c>
+      <x:c r="I66" t="str">
+        <x:v>BENBUSI311.pdf</x:v>
+      </x:c>
+      <x:c r="J66" t="str">
+        <x:v>f31d461ec0ceefc930dd96059e9d91b881e5596a53dcc0f9809ce2ab47ded01a</x:v>
+      </x:c>
+      <x:c r="K66"/>
+      <x:c r="L66"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B67" t="str">
+        <x:v>BENECON212</x:v>
+      </x:c>
+      <x:c r="C67" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D67" t="str">
+        <x:v>Microeconomics</x:v>
+      </x:c>
+      <x:c r="E67" t="str">
+        <x:v>Develops microeconomic theory through consumer behaviour, imperfectly competitive markets and economy-wide allocation. Students examine choice under uncertainty, non-egoistic preferences and cognitive limitations, then monopoly, strategic behaviour and labour and capital markets. General equilibrium, efficiency, externalities and government complete the analysis. Algebraic problem-solving and graphical analysis are connected to the interpretation and evaluation of research papers.</x:v>
+      </x:c>
+      <x:c r="F67" t="str">
+        <x:v>Microeconomics; Behavioural economics</x:v>
+      </x:c>
+      <x:c r="G67" t="str">
+        <x:v>Choice under uncertainty; Non-egoistic preferences; Cognitive limitations; Monopoly; Imperfect competition and strategic behaviour; Labour markets; Capital markets; General equilibrium; Market efficiency; Externalities; Government intervention</x:v>
+      </x:c>
+      <x:c r="H67" t="str">
+        <x:v>Algebraic microeconomic analysis; Graphical economic analysis; Critical evaluation of economic research</x:v>
+      </x:c>
+      <x:c r="I67" t="str">
+        <x:v>BENECON212.pdf</x:v>
+      </x:c>
+      <x:c r="J67" t="str">
+        <x:v>698f75bfea6eeae09f5313c207a6ceae6754af223de4146e76464ca3dfbee2ae</x:v>
+      </x:c>
+      <x:c r="K67"/>
+      <x:c r="L67"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B68" t="str">
+        <x:v>BENECON311</x:v>
+      </x:c>
+      <x:c r="C68" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D68" t="str">
+        <x:v>Public Economics</x:v>
+      </x:c>
+      <x:c r="E68" t="str">
+        <x:v>Examines government intervention through the efficiency and equity effects of public policy. Market failure, public goods and externalities provide foundations for studying public production, collective choice, spending and taxation. Health, education, welfare and social insurance illustrate expenditure and redistribution questions. Students apply economic models, interpret data and graphs, evaluate research and develop a research proposal and paper.</x:v>
+      </x:c>
+      <x:c r="F68" t="str">
+        <x:v>Public economics; Political economy</x:v>
+      </x:c>
+      <x:c r="G68" t="str">
+        <x:v>Role and size of government; Market efficiency and failure; Public goods; Externalities; Efficiency and equity; Public production; Public choice; Public expenditure; Health and education policy; Welfare programs; Social insurance; Taxation and redistribution</x:v>
+      </x:c>
+      <x:c r="H68" t="str">
+        <x:v>Economic model-based policy analysis; Efficiency and equity assessment; Interpretation of economic data and graphs; Critical evaluation of public-economics research</x:v>
+      </x:c>
+      <x:c r="I68" t="str">
+        <x:v>BENECON311.pdf</x:v>
+      </x:c>
+      <x:c r="J68" t="str">
+        <x:v>0033a6a37127ce7ba2c3df19a887537dfcd601286cf9b112ff2fe1ede2470a02</x:v>
+      </x:c>
+      <x:c r="K68"/>
+      <x:c r="L68"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B69" t="str">
+        <x:v>BENENTR111</x:v>
+      </x:c>
+      <x:c r="C69" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D69" t="str">
+        <x:v>Consumer Product Design</x:v>
+      </x:c>
+      <x:c r="E69" t="str">
+        <x:v>Teaches consumer-product design through a sequence from investigating existing products to developing an original product. Students assess customer needs, develop concepts, devise fabrication approaches and consider production at laboratory and industrial scales. Practical work includes interviewing, experimentation, quantitative modelling and prototyping, with economic and environmental appraisal. Sustainability, including materials, lifespan, repairability and circularity, informs the design process.</x:v>
+      </x:c>
+      <x:c r="F69" t="str">
+        <x:v>Product design; Product development; Sustainable design</x:v>
+      </x:c>
+      <x:c r="G69" t="str">
+        <x:v>Customer needs and product concepts; Product mechanisms; Fabrication and prototyping; Laboratory-to-industrial scaling; Environmental impact; Costs and revenues; Materials and product lifespan; Repairability and circularity; Intellectual-property protection; Product marketing</x:v>
+      </x:c>
+      <x:c r="H69" t="str">
+        <x:v>Customer interviewing; Existing-product analysis; Laboratory experimentation; Quantitative product modelling; Prototype construction; Fabrication-process development; Cost and revenue estimation; Environmental-impact assessment</x:v>
+      </x:c>
+      <x:c r="I69" t="str">
+        <x:v>BENENTR111.pdf</x:v>
+      </x:c>
+      <x:c r="J69" t="str">
+        <x:v>54c2e1718f15e3bb60cd6b9b35cf69a4f2d725a7c392c5cbd3ab5801d7f7a300</x:v>
+      </x:c>
+      <x:c r="K69" t="str">
+        <x:v>The heading and filename identify BENENTR111, while running footers and the course-manual reference retain ENGPROJ103.</x:v>
+      </x:c>
+      <x:c r="L69"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>BENENTR211</x:v>
+      </x:c>
+      <x:c r="C70" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>Marketing &amp; Consumer Engagement</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Connects marketing strategy and consumer psychology to responsible brand development and customer engagement. Students study strategic planning, customer experience, qualitative and quantitative insights, brand identity, digital marketing and behavioural framing. Applied projects analyze a company's strategy and response to disruption, design a brand, and investigate a consumer phenomenon using academic literature and primary and secondary evidence. Customer-journey mapping translates findings into recommendations.</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>Marketing; Consumer psychology; Brand management</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Strategic marketing planning; Marketing mix; Customer centricity and experience; Consumer journeys; Market research and augmented insights; Brand identity and image; Brand partnerships; Digital and social marketing; Responsible marketing; Consumer psychology; Nudging and framing; Emerging technologies and marketing agility</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>Marketing-strategy case analysis; Advertising-campaign analysis; Kapferer brand-identity prism; Brand design; Primary and secondary consumer research; Consumer-journey mapping; Disruption-response planning</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>BENENTR211.pdf</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>b63a16f400eff3cf608269ce8e05f4e370952ec13f6fc752376bac39657fb80d</x:v>
+      </x:c>
+      <x:c r="K70"/>
+      <x:c r="L70" t="str">
+        <x:v>The consumer project permits a choice of primary research methods; the outline does not establish that every student practices each listed example.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>BENGATE102</x:v>
+      </x:c>
+      <x:c r="C71" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>Research Methods &amp; Statistics</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>Introduces empirical research design and statistical analysis, followed by a substantial student research project. Students study operationalization, measurement quality, sampling, surveys and experimental and nonexperimental designs, then descriptive statistics, estimation, hypothesis testing and introductory regression. R and R Commander support data display and analysis. Project teams develop instruments and a research plan, collect and analyze data, and report results under explicit research-ethics and privacy requirements.</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>Research methodology; Applied statistics</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>Scientific inquiry and hypotheses; Operationalization and measurement; Reliability and validity; Survey construction and sampling; Randomized and quasi-experimental designs; Nonexperimental and qualitative research; Descriptive statistics; Sampling distributions and estimation; Hypothesis testing and confidence intervals; Association and regression; Research ethics and anonymous data collection</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>Survey design; Probability and nonprobability sampling; Experimental and nonexperimental research design; R and R Commander data analysis; Descriptive statistics and visualization; Scale-reliability analysis; One- and two-sample mean tests; ANOVA; Chi-square tests; Correlation and regression; Empirical data collection and analysis</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>BENGATE102.docx</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>a7449c15eb1e37aaaed7d43b49f67b3492fe6b3f9163275197f62c4450a8485e</x:v>
+      </x:c>
+      <x:c r="K71"/>
+      <x:c r="L71"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>BENLEAD112</x:v>
+      </x:c>
+      <x:c r="C72" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>Leadership Communication (Theory and Practice)</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>Studies leadership communication through leadership theory, persuasion and practical rhetorical work. Students compare contemporary leadership approaches and examine emotional intelligence, gender, culture and ethics. Literary characters, film and speeches provide material for analyzing effective and ineffective leadership. Students interview a real leader, analyze the leader's communication challenge in an advisory report, and develop a public address presenting their own ethical leadership vision.</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>Leadership studies; Communication studies; Rhetoric</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>Leadership models and approaches; Transformational, authentic and adaptive leadership; Servant leadership and followership; Emotional intelligence; Leadership ethics; Gender and culture in leadership; Persuasion and organizational communication; Leadership in literature and film; Storytelling and public speaking; Personal leadership vision</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>Leadership-theory application; Literary and film-based leadership analysis; Professional interviewing and note collection; Leadership-discourse analysis; Communication-advisory report development; Rhetorical speechwriting and storytelling</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>BENLEAD112.docx</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>1c68ecf16bed5882efb0632a24aafaaf060c5da403870fd44aba5682ac087172</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>The opening heading says Spring 2026, while running headers and footers retain Spring 2025.</x:v>
+      </x:c>
+      <x:c r="L72"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>BENLEAD312</x:v>
+      </x:c>
+      <x:c r="C73" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>Negotiation and Strategic Thinking (in Business and Beyond)</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>Develops negotiation as an analytical practice and interpersonal skill. Students learn interest-based bargaining, BATNA and ZOPA, value creation, framing, concessions and strategies for handling power, emotions and difficult counterparts. Social-psychological and communication perspectives connect negotiation to trust, ethics, culture and relationships. Frequent simulations and narrative analysis lead to an annotated negotiation film and the design, teaching and evaluation of a negotiation scenario grounded in Delta Climate Center themes.</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>Negotiation studies; Strategic management; Social psychology; Communication studies</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>Interests versus positions; BATNA and ZOPA; Mutual gains and objective criteria; Dual-concern model; Anchoring, framing and concessions; Trade-offs and logrolling; Cognitive biases and influence; Power and emotions; Trust, reputation and ethics; Cross-cultural and organizational negotiation; Negotiation implementation and withdrawal; Stakeholder interests</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>BATNA and ZOPA analysis; Stakeholder-interest mapping; Interest-based negotiation; Negotiation simulations; Narrative and film analysis of bargaining; Negotiation-scene scripting and annotation; Scenario design and reflective evaluation</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>BENLEAD312.docx</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>002e9603ebc48e416d74e4150484f949c5feea7495c2c4cfe3f557d3ba919e47</x:v>
+      </x:c>
+      <x:c r="K73"/>
+      <x:c r="L73"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>DISARIN111</x:v>
+      </x:c>
+      <x:c r="C74" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>AI, Ethics &amp; Psychology</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Examines AI through ethical theory and psychological accounts of human behaviour and interaction. Ethical debates address fairness, privacy, responsibility, alignment, moral status and political or existential risks. Psychological perspectives consider development, clinical care, social and organizational relationships, forensic applications and cognitive neuroscience. Students synthesize literature and apply ethical frameworks in an analytical psychology project and a research-grounded podcast, with a creative communication component.</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>AI ethics; Philosophy; Psychology</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>Algorithmic fairness and bias; Privacy and surveillance; Responsibility and accountability; Human-value alignment; Moral status of AI; Existential risk and democratic implications; Trust and agency in human-AI interaction; AI in clinical care; Child development and AI; Social and organizational effects of AI; AI in forensic psychology; Cognitive and socioemotional development; AI consciousness and sentience</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>Ethical-framework application; Philosophical argument evaluation; Psychological-literature synthesis; Theory-based analysis of AI applications; Research podcast scripting, recording and editing</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>DISARIN111.pdf</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>d14871e6a13652bae8f9fa423360ec39b8c9804c70fc19d4b77f305b16dea799</x:v>
+      </x:c>
+      <x:c r="K74"/>
+      <x:c r="L74" t="str">
+        <x:v>The psychology project is literature-based with a choice of creative outputs; empirical data collection and technical AI development are not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>DISARIN311</x:v>
+      </x:c>
+      <x:c r="C75" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>Optimization Methods in AI</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>Studies search and optimization for rational agents in known, complex and adversarial environments. Students move from uninformed and heuristic search to local and global optimization, first- and second-order methods and population approaches. Adversarial search, constraint satisfaction, linear programming and discrete optimization extend the toolkit. Laboratories and projects require algorithm tracing, implementation and evaluation and experimental investigation of small intelligent systems.</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>Artificial intelligence; Mathematical optimization; Computer science</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>Intelligent and rational agents; Uninformed and informed search; Heuristic functions; Search in complex environments; Local and global optimization; First- and second-order optimization; Population methods; Adversarial games; Constraint satisfaction; Linear programming; Discrete optimization</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>Uninformed and heuristic search; Local and global search; First- and second-order optimization; Population-based optimization; Adversarial search; Monte Carlo tree search; Constraint-satisfaction algorithms; Linear programming; Discrete optimization; Algorithm implementation and experimental evaluation</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>DISARIN311.pdf</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>9abd4ca16ad834aebc1b3d6a55b5133c96f8ef0b56d0428156722730b48d9dea</x:v>
+      </x:c>
+      <x:c r="K75"/>
+      <x:c r="L75"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>DISCOMP213</x:v>
+      </x:c>
+      <x:c r="C76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>Software Development</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>Develops software-construction skills through C++ and functional programming in Haskell, alongside software design and quality assurance. C++ work addresses classes, inheritance, polymorphism and memory management; Haskell introduces functions, recursion, types and input/output. Laboratories apply version control, code review, debugging, testing, documentation and design patterns. Projects require students to build and explain programs in both languages.</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Computer science; Software engineering; Programming</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>C++ classes and operator overloading; Inheritance and polymorphism; Dynamic memory and smart pointers; Copy construction; Functional programming and immutability; Haskell functions, recursion and types; Higher-order functions; Software development lifecycle; Version control; Debugging and testing; Documentation; Design patterns</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>C++ programming; Haskell functional programming; Git and GitLab version control; Code review; Systematic debugging; Unit and integration testing; White-box and black-box testing; Static testing; Design-pattern implementation; Software documentation</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>DISCOMP213.pdf</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>80d6a774ba5afdec9beee32bf301e111036e96b121702d4bb0a436dd0a3a5abd</x:v>
+      </x:c>
+      <x:c r="K76"/>
+      <x:c r="L76"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>DISCOMP312</x:v>
+      </x:c>
+      <x:c r="C77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>Advanced Algorithms</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>Studies algebraic algorithms and advanced optimization methods through mathematical reasoning, implementation and experimental analysis. Fast and exact arithmetic, number-theoretic algorithms, matrix multiplication and Fourier transformation lead into hashing, greedy methods, dynamic programming and network flows. Laboratories develop algorithmic understanding, while projects investigate exact computing and optimization, including hypotheses, measured performance and sensitivity analysis.</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Computer science; Algorithm design and analysis; Computational mathematics</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>Asymptotic time complexity; Fast integer arithmetic; Greatest common divisors and modular arithmetic; Chinese remainder theorem; Arbitrary-precision integers; Primality and factorization; Fast matrix multiplication; Polynomials and Fourier transformation; Hashing and Bloom filters; Greedy algorithms and coding; Dynamic programming; Flow networks; Network science</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>Asymptotic and empirical complexity analysis; Euclidean algorithm; Primality testing and factorization; Fast arithmetic and matrix algorithms; Fast Fourier transformation; Hashing; Greedy optimization; Dynamic programming; Maximum-flow algorithms; Algorithmic experimental design; Sensitivity analysis</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>DISCOMP312.pdf</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>9e6765b092585a19e53f8537598f2da6828893169e9ce9dd10afa83806319aea</x:v>
+      </x:c>
+      <x:c r="K77"/>
+      <x:c r="L77"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>DISDATA111</x:v>
+      </x:c>
+      <x:c r="C78" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>Introduction to Data Science</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>Introduces data visualization, exploration and manipulation in R using tabular, textual and spatial data. Students learn tidy-data principles, data import and joins, web scraping, functions and the grammar of graphics. Group and individual projects apply data integration and visualization to an assigned administrative dataset and an independently chosen question, emphasizing data interpretation, clear code and informative graphics.</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>Data science</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>Data visualization and exploratory analysis; Tidy data; Data transformation and integration; Dates and times; Web data; Text data; Geospatial data; Programming functions; Data quality and interpretation; Visualization-based empirical inquiry</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>R and tidyverse programming; ggplot visualization; Data cleaning, tidying and transformation; Data import and joins; Web scraping; Text-data analysis; Geospatial-data analysis; Exploratory analysis of administrative datasets</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>DISDATA111.pdf</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>d952cc9390df33764d2a2319da681453fb3a74fa0b2dca9305b51564656a4120</x:v>
+      </x:c>
+      <x:c r="K78"/>
+      <x:c r="L78"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>DISDATA311</x:v>
+      </x:c>
+      <x:c r="C79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Neural Networks and Deep Learning</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>Develops neural-network theory and practical implementation in Python, Keras and TensorFlow. Students build and train simple networks before studying multilayer architectures, backpropagation, regularization and model evaluation. Later work applies deep learning to computer vision, time series and text, including transformers. Projects construct predictors for tabular data and investigate an independently chosen image- or text-based prediction problem, with experimental results reported in a paper.</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Machine learning; Deep learning; Data science</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>Perceptrons and ADALINE; Multilayer neural networks; Gradient descent and backpropagation; Bias-variance trade-off and regularization; Computation graphs; Network architectures and interpretation; Computer vision; Time-series learning; Text classification and generation; Transformers and large language models; Feature engineering; Predictive performance</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>Python programming; Keras and TensorFlow network implementation; Gradient-descent training; Backpropagation implementation; Neural-network performance evaluation; Tabular prediction; Image classification; Text classification and generation; Deep-learning experimental design</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>DISDATA311.pdf</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>ce82215edc42a5562f8e67af87bbc4a12ea4e0b4c20ca84442c83deddc14950a</x:v>
+      </x:c>
+      <x:c r="K79"/>
+      <x:c r="L79" t="str">
+        <x:v>Image-generation models are mentioned only as a possible brief addition if time permits; they are not treated as established course coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>DISDATA312</x:v>
+      </x:c>
+      <x:c r="C80" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Robotics</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Studies computational problems in robot motion and manipulation, supported by linear algebra, calculus and geometric modelling. Students analyze forward and inverse kinematics, configuration spaces, collision-free motion planning and grasping, with shorter introductions to sensing and control. Practical work programs a robot arm and gripper; research investigates inverse kinematics for an articulated structure. A smaller component examines a chosen legal, ethical, safety or human-robot issue.</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>Robotics; Computer science; Applied mathematics; Engineering</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>Robot architecture and industrial automation; Rotations, orientations and rigid transformations; Forward and inverse kinematics; Trajectory generation; Configuration spaces and obstacles; Exact, approximate and sampling-based motion planning; Collision detection; Sensing and control; Form and force closure; Caging; Non-prehensile manipulation; Social and ethical aspects of robotics</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Coordinate-frame modelling of articulated structures; Analytic and iterative inverse kinematics; Mathematica computation; Configuration-space modelling; Motion-planning analysis; Collision-detection analysis; Instantaneous-motion and wrench analysis; Robot-arm and gripper programming; Modelling of physical manipulation</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>DISDATA312.pdf</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>6745ea87b45725e23b123e23ee15d99329ba7e7bd4ef4a571afade109c801018</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>The cover identifies DISDATA312 and June 2026; an internal heading retains ENGDATA302 and Spring 2025. The authoritative container semester remains 2026h1.</x:v>
+      </x:c>
+      <x:c r="L80"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>DISMATH213</x:v>
+      </x:c>
+      <x:c r="C81" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>Computational and Numerical Methods</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>Develops numerical solutions to mathematical problems that lack convenient analytical solutions, emphasizing when algorithms work and how to validate their output. Students study numerical root finding, interpolation, differentiation, quadrature, ordinary differential equations, and linear and nonlinear systems. Mathematica notebooks apply and compare textbook algorithms with built-in routines, with attention to roundoff, convergence, error, stability and sensitivity.</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>Numerical analysis; Computational mathematics; Scientific computing</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>Computer arithmetic and roundoff; Algorithm convergence and error; Scalar root finding; Polynomial interpolation and splines; Parametric curves; Numerical differentiation and integration; Initial-value problems; Multistep and adaptive differential-equation methods; Stability and stiff equations; Linear systems and matrix factorization; Nonlinear systems; Numerical-result validation</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>Mathematica numerical computation; Bisection, fixed-point, Newton and secant methods; Polynomial and spline interpolation; Numerical differentiation and Richardson extrapolation; Simpson, Romberg and Gaussian quadrature; Adaptive quadrature; Euler and Runge-Kutta methods; Multistep predictor-corrector methods; Gaussian elimination and pivoting; Matrix factorizations; Newton and quasi-Newton methods for systems; Steepest descent; Continuation methods</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>DISMATH213.pdf</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>b67d8077fd5b789845d7efc73e302aa6092ef42448893e357bfc3b8aec64aadb</x:v>
+      </x:c>
+      <x:c r="K81"/>
+      <x:c r="L81"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>DISMATH312</x:v>
+      </x:c>
+      <x:c r="C82" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>Linear Systems</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>Analyzes continuous- and discrete-time signals and linear time-invariant systems through differential or difference equations, impulse responses and frequency-domain representations. Convolution, Fourier series and transforms lead into sampling and reconstruction, filtering, communication systems, Laplace and Z-transforms, and linear feedback. Mathematica laboratories and an applied project connect mathematical properties to signal processing and system behaviour.</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Applied mathematics; Signal processing; Systems and control</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>Continuous- and discrete-time signals; System linearity, causality and stability; Impulse and frequency responses; Convolution; Fourier series and transforms; Time-frequency representations; Sampling, reconstruction and aliasing; Digital filtering; Modulation and multiplexing; Laplace and Z-transforms; Regions of convergence and pole-zero representations; Linear feedback and stability</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>Convolution sums and integrals; Fourier-series and Fourier-transform analysis; Bode-plot analysis; Sampling and signal reconstruction; Filter analysis; Modulation and demodulation; Laplace and Z-transform analysis; Block-diagram system analysis; Root-locus analysis; Mathematica signal and system computation</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>DISMATH312.pdf</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>42d2ebd985ff5832b7f838ea1d426815b470667bebee89fb17893151f2195208</x:v>
+      </x:c>
+      <x:c r="K82" t="str">
+        <x:v>The communication-systems learning-objective narrative says the focus is frequency modulation, whereas the detailed schedule specifies amplitude-modulation topics.</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>The applied-project subjects are examples students may select; quantum mechanics, image processing and additional transforms are not established common coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>DISMATH313</x:v>
+      </x:c>
+      <x:c r="C83" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>Advanced Physics</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>Develops a mathematical treatment of classical mechanics centered on the principle of least action and Lagrangian formalism. Oscillations, central forces, angular momentum, rigid-body rotation and accelerating frames connect abstract principles to mechanical systems. Students derive and solve equations of motion and use Mathematica for calculations. An independent literature-based paper extends an assigned physics article and reproduces key calculations in an accompanying notebook.</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>Theoretical physics; Classical mechanics; Mathematical physics</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>Principle of least action; Lagrangian mechanics and generalized coordinates; Calculus of variations; Harmonic and coupled oscillators; Central forces and orbital motion; Angular momentum and torque; Moments of inertia and inertia tensors; Rigid-body dynamics; Conservation laws and collisions; Rotating frames and fictitious forces</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>Variational derivation of Euler-Lagrange equations; Newtonian and Lagrangian modelling; Differential-equation solution; Normal-mode analysis; Central-force orbital analysis; Inertia-tensor calculation; Conservation-law analysis; Rotating-frame transformations; Mathematica symbolic and numerical computation; Literature-based reproduction and extension of physics calculations</x:v>
+      </x:c>
+      <x:c r="I83" t="str">
+        <x:v>DISMATH313.pdf</x:v>
+      </x:c>
+      <x:c r="J83" t="str">
+        <x:v>be33ddf46f10c84ad4b6b89b12c2d858726017876c6b0056d4a5154e88797186</x:v>
+      </x:c>
+      <x:c r="K83"/>
+      <x:c r="L83" t="str">
+        <x:v>Some later sessions and individual paper topics are unspecified; their narrower subject matter cannot be established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>ENSDELT211</x:v>
+      </x:c>
+      <x:c r="C84" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>Living with Water</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>Examines how delta societies manage water risks and opportunities, using Zeeland as a central case. Physical and ecological challenges such as flooding, salinization, freshwater scarcity, subsidence and pollution are connected to infrastructure, history, governance, law and justice. Students evaluate engineered and nature-based responses, considering trade-offs and long-term consequences. Site-based inquiry and a project apply these concepts to context-sensitive adaptation in a delta region.</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>Water management; Environmental governance; Delta sustainability</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>Delta environments; Flood risk and protection; Drainage and freshwater management; Sea-level rise and subsidence; Salinization; Water infrastructure and ecological consequences; Water governance, law and justice; Contaminants and pollution; EU Water Framework Directive; Nature-based adaptation; Urban ecology and water; Long-term delta resilience</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>Site-based water-management case analysis; Comparative appraisal of engineered and nature-based solutions; Context-sensitive adaptation-strategy development</x:v>
+      </x:c>
+      <x:c r="I84" t="str">
+        <x:v>ENSDELT211.pdf</x:v>
+      </x:c>
+      <x:c r="J84" t="str">
+        <x:v>6bb326cf0652c24583cecb7bc13dd206fc629c227944e8dd4fec37374b4ade9a</x:v>
+      </x:c>
+      <x:c r="K84"/>
+      <x:c r="L84" t="str">
+        <x:v>Detailed project and site-visit instructions are deferred to Moodle; the outline does not specify hydrological measurement, modelling or other technical field methods.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>ENSDELT312</x:v>
+      </x:c>
+      <x:c r="C85" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>Governance of Sustainability</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>Analyzes sustainability as a problem of collective decision-making involving governments, markets and civil society. Concepts of institutions, power, participation, justice and problem complexity frame competing technological and systemic responses. Structured cases examine food, freshwater, energy and climate mitigation. Students apply governance frameworks to a Zeeland issue, consult relevant organizations or experts, and produce policy advice or an evaluation assessing effectiveness, feasibility and stakeholder interests.</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>Environmental governance; Public policy; Political science</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Institutions, actors and power; Collective action and common-pool resources; Governance modes and networks; Techno-optimism and ecological limits; Climate justice; Populism and environmental politics; Wicked and long-term problems; Public participation; Food, water and energy governance; Markets, public goods and externalities; Adaptive and global governance; Climate mitigation; Policy effectiveness and feasibility</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>Governance-framework application; Problem diagnosis and causal analysis; Stakeholder and policy-option matrices; Policy evaluation; Policy-advice memo development; Stakeholder and expert interviewing; Comparative analysis of normative policy perspectives</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>ENSDELT312.docx</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>aa60b30832d0031c1fcbf3d32adbc4a9b519b4223078a145688b52aace058c01</x:v>
+      </x:c>
+      <x:c r="K85"/>
+      <x:c r="L85"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>ENSECOL112</x:v>
+      </x:c>
+      <x:c r="C86" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>Protecting Nature: The Science of Conservation</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Introduces conservation biology through biodiversity loss, its human causes and possible responses. Students examine habitat destruction and fragmentation, overharvesting, invasive species, climate change, disasters and extinction, followed by conservation planning, species management and conservation in altered landscapes. A local threatened-species project investigates conservation status and protection measures and develops a public-awareness flyer.</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>Conservation biology; Ecology</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>Biodiversity and ecosystems; Anthropogenic extinction; Habitat loss and fragmentation; Overharvesting; Invasive species; Climate impacts; Natural and human-caused disasters; Conservation priorities; Endangered-species management; Human-modified landscapes; People and conservation; Conservation-study design and evaluation</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>Threatened-species conservation-status analysis; Assessment of species-protection measures; Evidence-based conservation communication</x:v>
+      </x:c>
+      <x:c r="I86" t="str">
+        <x:v>ENSECOL112.docx</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>1ed9acec492bd694d577ed350e7e008eb7b5f45ee54623e9f19219b1fde897e6</x:v>
+      </x:c>
+      <x:c r="K86"/>
+      <x:c r="L86" t="str">
+        <x:v>The outline does not specify field sampling or population-estimation techniques for the species project.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>ENSECOL212</x:v>
+      </x:c>
+      <x:c r="C87" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>Ecosystems Uncovered: How Nature Works</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Develops ecological principles from organisms and populations to communities and ecosystems. Environmental conditions, resources and life cycles frame competition, feeding relationships, selection, population dynamics and biodiversity. Energy and matter cycles connect ecological processes to conservation and human impacts. Dedicated practical sessions teach simple ecological modelling in R, and a small research project communicates findings through a poster.</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Ecology; Ecosystem science</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>Ecology and evolution; Environmental conditions and resources; Climate and life cycles; Ecological niches; Competition and cohabitation; Predation and food webs; Natural selection; Population dynamics; Biodiversity patterns; Ecological succession; Ecosystem energy and matter fluxes; Global cycles; Conservation and human impacts; Ecosystem value</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>Ecological modelling in R; Population-dynamics calculations; Ecosystem energy and matter-flux calculations; Ecological research-project design and analysis</x:v>
+      </x:c>
+      <x:c r="I87" t="str">
+        <x:v>ENSECOL212.docx</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>2353fd7c9724839667650fabfe4a29ff7d1244f2566c21d4e1893dba036351b3</x:v>
+      </x:c>
+      <x:c r="K87"/>
+      <x:c r="L87" t="str">
+        <x:v>The ecological research project's specific sampling and measurement procedures are not supplied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>ENSECOL312</x:v>
+      </x:c>
+      <x:c r="C88" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>Sustainable Farming &amp; Innovation</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>Examines how food production can balance human needs with environmental impacts. Students assess current agriculture, horticulture and animal husbandry, their effects on biodiversity and ecosystems, and alternative practices and innovations. Aquaculture, alternative animal-protein sources and farming for other industries extend the comparison. A literature-based project critically investigates a chosen sustainable-farming question and reports the evidence without prescribing a single preferred approach.</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>Sustainable agriculture; Agroecology; Food-system sustainability</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>Agricultural and horticultural systems; Environmental impacts of farming; Wildlife and biodiversity; Modification of current farming practices; Alternative agricultural approaches; Animal husbandry; Aquaculture; Alternative protein sources; Farming for non-food industries; Sustainable-farming innovation</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>Scientific-literature review; Comparative appraisal of farming practices and innovations</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>ENSECOL312.docx</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>cd23c7fca1ca10b003ec0b5e00a1925654e963dfa3619fa45bcb57b1f3c1c02a</x:v>
+      </x:c>
+      <x:c r="K88"/>
+      <x:c r="L88" t="str">
+        <x:v>Alternative systems are not individually named in the outline, and hands-on farming or experimental agronomy is not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>ENSENVI211</x:v>
+      </x:c>
+      <x:c r="C89" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>Earth Observation</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>Develops geospatial analysis for investigating environmental change and designing responses to Earth-system problems. Hands-on ArcGIS Pro work covers spatial data models, georeferencing, projections, visualization, queries, transformations and surface analysis. Remote-sensing foundations extend into spectral signatures, acquisition systems, preprocessing and image processing. A collaborative case study applies geospatial methods to an environmental research question.</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Geographic information science; Remote sensing; Environmental science</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>Spatial concepts and data models; Geospatial databases; Georeferencing and map projections; Spatial visualization; Spatial queries and transformations; Surface analysis; Earth-observation tools; Spectral signatures; Remote-sensing acquisition systems; Image preprocessing and processing; Environmental geospatial applications</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>ArcGIS Pro spatial analysis; Spatial-data collection and database management; Georeferencing and coordinate transformation; Geospatial visualization and queries; Surface analysis; Remote-sensing preprocessing; Image processing; Geospatial case-study design</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>ENSENVI211.pdf</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>933c6839c355f31884087a9b59e2a6e1c5dac6bcfe4e95e7c1af92f6b158b880</x:v>
+      </x:c>
+      <x:c r="K89"/>
+      <x:c r="L89"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>ENSGATE201</x:v>
+      </x:c>
+      <x:c r="C90" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>Sustainability Essentials II</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>Connects wave physics, chemistry and materials science to sustainability questions. Students study wave behaviour and observation methods, chemical analysis, microscopic material structure and macroscopic stress and strain. Practical sessions include wave applications and chemistry laboratory work. Reflective inquiries and a final project critically assess sustainability campaigns, identify greenwashing and communicate evidence-based improvements to a public audience.</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>Physics; Chemistry; Materials science; Sustainability studies</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>Electromagnetic and mechanical waves; Wave composition and interference; Optical spectroscopy; Electron microscopy; Inorganic and organic chemistry; Chemical testing; Material structure and crystallography; Stress and strain; Sustainable material design; Geological wave applications; Nuclear power and waste; Greenwashing</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>Oscilloscope wave visualization; Optical-spectroscopy interpretation; Fourier wave analysis; Copper dissolution and chemical analysis; Laboratory logbook documentation; Stress-strain analysis; Mohr's-circle application; Evidence-based greenwashing case analysis; Public sustainability-communication design</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>ENSGATE201.pdf</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>dc9ace82b93250d969939ce5f8c0893cf399adb06f1b0ac97a1b45126931a9d0</x:v>
+      </x:c>
+      <x:c r="K90" t="str">
+        <x:v>The cover omits the title's 'II', while the course-title field and running headings say Sustainability Essentials II. The chemistry learning-outcomes table describes observing mycelium growth under contaminants, whereas the detailed schedule specifies copper-penny analysis and chemical testing.</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>The extraction follows the scheduled chemistry activities; specific mycelium methods and hands-on electron-microscopy training are not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>ENSSUST113</x:v>
+      </x:c>
+      <x:c r="C91" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>Calling Bullshit</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>Examines misinformation through philosophy, history, psychology and practical information evaluation. Students distinguish misleading discourse from related concepts, investigate cognitive and social vulnerabilities, and analyze pseudoscience, statistical misrepresentation and reasoning errors. Fact-checking, deepfake production and response exercises develop recognition and intervention skills. Projects map a misinformation narrative's actors and circulation and produce a research-grounded myth-debunking video with an external interview.</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Misinformation studies; Psychology; Applied epistemology; Science communication</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Bullshit, lying and misinformation; Historical hoaxes and propaganda; Cognitive bias and motivated reasoning; Social identity and information overload; Scientific credibility and pseudoscience; Publication bias and misconduct; Misleading statistics and data displays; Reasoning fallacies; Deepfakes; Misinformation diffusion; Debunking and counter-narratives; Medical and climate misinformation</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>Source-credibility evaluation; Fact-checking protocols; Reasoning-fallacy detection; Critical analysis of statistical claims; Misinformation-network mapping; Deepfake video construction and analysis; Debunking-message design; Expert interviewing; Documentary-style explanatory video production</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>ENSSUST113.docx</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>cb604ad4e33d3e0619df15847cf21b4b322e46c96e1624112b63ce2fc4fdf6fc</x:v>
+      </x:c>
+      <x:c r="K91"/>
+      <x:c r="L91"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>ENSSUST313</x:v>
+      </x:c>
+      <x:c r="C92" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>Research in a Sustainable Delta</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Provides an applied research setting for sustainability problems proposed by regional institutions and companies. Small teams work with an external advisor to review literature, formulate a research question, plan and execute an investigation, and develop a final product, design or report. Projects connect academic inquiry to the Zeeland delta, while their substantive questions and practical activities vary with the external partner.</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Sustainability research</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>Applied sustainability problems in the Zeeland delta; Partner-defined research questions; Academic evidence for sustainability interventions; External stakeholder collaboration</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>Literature review; Applied research design</x:v>
+      </x:c>
+      <x:c r="I92" t="str">
+        <x:v>ENSSUST313.pdf</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>d0e099ffaea3f971b03ab68c180247ca99964782b60814d8ae794f54a5248197</x:v>
+      </x:c>
+      <x:c r="K92" t="str">
+        <x:v>The PDF identifies ENSUST313, while the authoritative filename identifies ENSSUST313.</x:v>
+      </x:c>
+      <x:c r="L92" t="str">
+        <x:v>No specific project subjects or practical techniques are supplied; these depend on the external partner and cannot be specified from the outline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>ENSSUST314</x:v>
+      </x:c>
+      <x:c r="C93" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>Thermodynamics &amp; Molecular Statistics</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>Introduces chemical thermodynamics before concentrating on the statistical derivation of macroscopic behaviour from molecular properties. Thermodynamic laws, potentials and chemical and electrochemical equilibrium provide the foundation. Boltzmann distributions, partition functions and ensemble theory are applied to gases, adsorption, interacting particles, electrons and electrolyte solutions. Mathematical derivations and structured problem-solving connect formal expressions to physical meaning.</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Physical chemistry; Thermodynamics; Statistical mechanics</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>Thermodynamic laws and equilibrium; Internal energy, enthalpy and entropy; Helmholtz and Gibbs energies; Chemical potential; Chemical and electrochemical equilibria; Boltzmann distribution; Molecular partition functions; Fermi-Dirac, Bose-Einstein and Maxwell-Boltzmann statistics; Canonical, microcanonical and grand-canonical ensembles; Fluctuations and intermolecular interactions; Adsorption and lattice models; Electrons in metals and semiconductors; Electrical double layers and electrolyte solutions</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>Thermodynamic-potential and equilibrium calculation; Legendre transformations; Partition-function analysis; Ensemble-statistical derivation; Mean-field approximation; Langmuir adsorption modelling; Debye-Hückel electrolyte modelling</x:v>
+      </x:c>
+      <x:c r="I93" t="str">
+        <x:v>ENSSUST314.pdf</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>578ac398a88078299bfaf009bbead593f097cd97458c6ea4d84341260c804999</x:v>
+      </x:c>
+      <x:c r="K93" t="str">
+        <x:v>The PDF identifies ENSUST314, while the authoritative filename identifies ENSSUST314.</x:v>
+      </x:c>
+      <x:c r="L93" t="str">
+        <x:v>The content list is explicitly incomplete and provisional; the outline warns that the planned coverage may not all fit within the semester.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>GOSHIST213</x:v>
+      </x:c>
+      <x:c r="C94" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>Western Way of War</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Surveys Western warfare from antiquity to the present and examines the contested claim that a distinctive military trajectory helped produce Western global dominance. Weapons, technology, strategy, tactics, institutions and soldiers' experience are studied across land, sea and air warfare. Research analyzes a strategic text, a commander's performance or a battle from the individual soldier's perspective, using primary sources and historical scholarship.</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Military history; Strategic studies; Historiography</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>Western warfare and global power; Ancient infantry and Roman warfare; Medieval warfare; Gunpowder and naval warfare; Overseas conquest; Dynastic and national warfare; Industrialization of war; World wars; Cold War and nuclear strategy; Guerrilla warfare and terrorism; Military leadership; Soldiers' experience, morale and cohesion; Future warfare</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>Primary- and secondary-source analysis; Historiographical critique of strategic texts; Historical analysis of military command; Soldier-centered battle analysis; Analysis of diaries, memoirs and combat accounts</x:v>
+      </x:c>
+      <x:c r="I94" t="str">
+        <x:v>GOSHIST213.docx</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>4ff7ce4c761e45585343beaec4dafdf8dda9ea398cc43cdb61026a6d4c4304a2</x:v>
+      </x:c>
+      <x:c r="K94" t="str">
+        <x:v>The heading identifies GOSHIS213, while the filename identifies GOSHIST213; the learning-outcomes mapping also retains AH-HIST210.</x:v>
+      </x:c>
+      <x:c r="L94"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>GOSHIST311</x:v>
+      </x:c>
+      <x:c r="C95" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>Native American Histories</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>Studies Native American social and cultural histories from the nineteenth century to the present through Indigenous perspectives and collaborative inquiry. Boarding schools, institutional violence, family separation and intergenerational trauma are connected to contemporary resistance, resurgence, food sovereignty and cultural expression. Storytelling, relational accountability and reciprocity inform work with Indigenous peers and knowledge holders. Arts-based collaborations and a public-history project develop respectful, accessible accounts of historical and contemporary issues.</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Indigenous studies; Social and cultural history; Public history</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>Indigenous histories and ways of knowing; Colonialism and white saviourism; Indian wars; Boarding schools and childhood trauma; Institutional confinement; Adoption and blood quantum; Gendered violence and missing Indigenous people; Traditional ecological knowledge; Food sovereignty; Decolonization and Indigenization; Cultural resistance and resurgence; Indigenous storytelling and public history</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>Indigenous storywork and relational historical inquiry; Primary-source and oral-history analysis; Arts-based collaborative inquiry; Photo/Voice photography and audio narratives; Historical contextualization of contemporary issues; Public-history multimedia production</x:v>
+      </x:c>
+      <x:c r="I95" t="str">
+        <x:v>GOSHIST311.docx</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>bae68811a6f3b2677acff8fdb6cd22a6d89cca11133d14366bca7909acfc5eae</x:v>
+      </x:c>
+      <x:c r="K95" t="str">
+        <x:v>The document heading identifies GOSHIST313, while the authoritative filename identifies GOSHIST311.</x:v>
+      </x:c>
+      <x:c r="L95" t="str">
+        <x:v>The current-events and public-history projects offer a choice of topics and media; not every listed topic or production format is required of every student.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>GOSHIST312</x:v>
+      </x:c>
+      <x:c r="C96" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>The Walcheren Expedition, 1809 History Research Seminar</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>Uses the British expedition to Walcheren in 1809 as a setting for sustained primary-source research. Introductory study places the campaign in Napoleonic warfare, the Netherlands and Zeeland. Students then locate, read and critically analyze a selected contemporary source, supported by additional primary and secondary material. Research papers investigate military, civilian, political, cultural or medical perspectives on the campaign and its consequences.</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>History; Military history; Historical research</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Napoleonic Europe and warfare; The Netherlands and Zeeland under Napoleon; Walcheren and Scheldt expedition of 1809; British, Dutch and French perspectives; Siege and bombardment of Vlissingen; Military and civilian experience; Walcheren fever; Historical testimony and source perspective</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>Primary-source discovery and selection; Contextual analysis of diaries, letters, memoirs and official reports; Historical source criticism; Comparison of primary and secondary evidence; Independent historical research</x:v>
+      </x:c>
+      <x:c r="I96" t="str">
+        <x:v>GOSHIST312.docx</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>a1859a171a3e3934984b4f96ab45fabd5a4daefab3ffed77b0cbd106ad6641e9</x:v>
+      </x:c>
+      <x:c r="K96" t="str">
+        <x:v>The opening heading identifies GOSHIS312, while the authoritative filename and learning-outcomes mapping identify GOSHIST312.</x:v>
+      </x:c>
+      <x:c r="L96" t="str">
+        <x:v>The extensive source list offers alternative research subjects; individual students study selected sources rather than every listed perspective.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>GOSLAWJ212</x:v>
+      </x:c>
+      <x:c r="C97" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>Introduction to Public International Law</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Introduces public international law through its sources, theories, institutions and relationship to domestic legal systems. Legal principles are applied to responsibility, force, armed conflict, international crime, human rights, economic relations and environmental protection. The later course examines self-determination, Third World approaches, soft law, compliance and treaty politics. Case exercises develop legal reasoning, while a research podcast critically investigates a political dimension of international law.</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Public international law; Socio-legal studies</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Sources and theories of international law; Treaty law; International legal subjects; Jurisdiction and immunities; Domestic courts and international law; State responsibility; Use of force; UN reform; Armed conflict and international criminal law; International human rights and economic law; Environmental law; Self-determination; Third World Approaches to International Law; Soft law, compliance and effectiveness; Global environmental treaties</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Identification and interpretation of international legal instruments; Judgment and case-law analysis; Application of legal principles to factual scenarios; Legal, empirical and normative critique; Research podcast development</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>GOSLAWJ212.pdf</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>b229b0b5f1fa795d1d10fe39a86c75d9cbd946b3db604f8d70889344596c07d6</x:v>
+      </x:c>
+      <x:c r="K97"/>
+      <x:c r="L97" t="str">
+        <x:v>The description names refugee law, but the detailed schedule does not identify a separate refugee-law component; its depth cannot be established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>GOSLAWJ213</x:v>
+      </x:c>
+      <x:c r="C98" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>Comparative Constitutional Law</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>Compares constitutional structures, institutions and rights across legal systems and introduces administrative law. Students examine constitutional features, federalism, legislatures, executive relationships, courts, judicial review and human rights. The administrative component addresses public participation, remedies and procedural fairness. A staged booklet compares two constitutions, supported by legal interpretation, case-law analysis and application of principles to hypothetical facts.</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>Comparative constitutional law; Administrative law</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Constitutional origins and fundamental features; Federalism and decentralization; Parliaments and lawmaking; Governments and heads of state; Court systems and judicial review; Constitutional rights; EU constitutional order; Administrative-law functions; Public participation; Administrative remedies; Procedural fairness, discretion and legitimate expectations</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>Comparative constitutional analysis; Constitutional and legislative interpretation; Case-law analysis; Application of legal principles to hypothetical facts; Structured comparative legal writing</x:v>
+      </x:c>
+      <x:c r="I98" t="str">
+        <x:v>GOSLAWJ213.pdf</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>774d5e9db0b95d4a9eb10e52080e31fb243d786c4407a2d6a343c47aba23bf41</x:v>
+      </x:c>
+      <x:c r="K98" t="str">
+        <x:v>The revised assessment section explicitly omits the administrative-law research paper, while the learning outcomes still describe independent administrative research and investigation.</x:v>
+      </x:c>
+      <x:c r="L98" t="str">
+        <x:v>The extraction reflects the retained comparative booklet and scheduled administrative-law material, without treating the omitted research paper as required work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>GOSLAWJ312</x:v>
+      </x:c>
+      <x:c r="C99" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>Foundations of EU Law</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>Introduces the EU legal order through its institutions, sources, competences and relationship to member-state law. Students study supremacy, legal effect, liability and judicial remedies before applying citizenship and free-movement law to concrete problems. Structured legal cases and research into current judgments develop interpretation and comparison across EU and domestic settings. Digital regulation and the green transition provide a contemporary application.</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>European Union law; Public law</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>European integration and institutions; EU legal sources and fundamental rights; Competences, subsidiarity and proportionality; Supremacy; Direct and indirect effect; State liability; Preliminary rulings; Review of EU acts and enforcement; EU citizenship; Free movement of persons, workers and goods; Establishment and services; Digital-market regulation and green transition</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>EU legal-source research; Case-law analysis; Comparative interpretation of EU and national law; Application of free-movement principles to factual scenarios; Structured legal problem analysis</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>GOSLAWJ312.docx</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>316d83161b69ac1e1e118c7ad1f1ab65dafcff461adb109db31d360eec9e81b1</x:v>
+      </x:c>
+      <x:c r="K99"/>
+      <x:c r="L99"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>GOSPHIL212</x:v>
+      </x:c>
+      <x:c r="C100" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>Ethics</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>Studies moral reasoning through historical and contemporary ethical theories and close philosophical reading. Utilitarianism, consequentialism, Kantian ethics, virtue ethics, contractarianism and feminist ethics lead into Nietzsche's genealogy, Murdoch's account of goodness and Nagel's treatments of value, perspective, death and meaning. Reflection and research essays require interpretation, argument evaluation and an independent position on ethical theory or a practical ethical problem.</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Moral philosophy; Metaethics; Practical ethics</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>Divine command and human nature; Moral relativism and universalism; Utilitarianism and consequentialism; Kantian ethics; Virtue ethics; Social contract and intuitionism; Feminist and care ethics; Nietzschean genealogy and nihilism; Murdoch's sovereignty of good; Moral value and perspective; Death, absurdity and meaning; Ethical theory and practical judgment</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>Close philosophical text analysis; Reconstruction and critical evaluation of moral arguments; Comparison of ethical theories; Conceptual analysis; Independent philosophical argument development</x:v>
+      </x:c>
+      <x:c r="I100" t="str">
+        <x:v>GOSPHIL212.pdf</x:v>
+      </x:c>
+      <x:c r="J100" t="str">
+        <x:v>c9d998071717b41e6f22eccc928229b14aee720759d703b906832bebf1852a1e</x:v>
+      </x:c>
+      <x:c r="K100" t="str">
+        <x:v>The description and later learning outcomes emphasize practical issues such as poverty, climate justice and historical injustice, while the detailed second-half schedule instead centers Nietzsche, Murdoch and Nagel.</x:v>
+      </x:c>
+      <x:c r="L100" t="str">
+        <x:v>The scheduled philosophical readings determine the main profile and topics; the extent of classroom coverage of the additional practical-ethics issues is uncertain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>GOSPHIL214</x:v>
+      </x:c>
+      <x:c r="C101" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>Philosophy of Mind</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>Examines minds, selves and conscious experience through historical and contemporary philosophy. Personal identity and self-knowledge are considered alongside Buddhist accounts and neuropsychological cases. Behaviourism, physicalism, functionalism and their critics frame the mind-body problem. Later inquiries address machine consciousness, virtual worlds, dreaming, perception, transformative experience and the value of experience. Essays develop independent philosophical interpretations and arguments.</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>Philosophy of mind; Metaphysics; Philosophy of cognitive science</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Persons and personal identity; Psychological and narrative theories of identity; Buddhist non-self; Split-brain cases and self-knowledge; Behaviourism; Physicalism and functionalism; Mind-body problem; Content externalism and internalism; AI intelligence and consciousness; Virtual reality; Dreaming and perception; Transformative experience; Value of conscious experience; Animal minds</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>Close philosophical reading; Conceptual analysis; Reconstruction and evaluation of arguments; Comparison of theories of mind; Literature-based philosophical research</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>GOSPHIL214.pdf</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>696658fcb99397616164f39ac292f3076d6ba1d189fd76530074fec0d368fc24</x:v>
+      </x:c>
+      <x:c r="K101"/>
+      <x:c r="L101"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>GOSPHIL312</x:v>
+      </x:c>
+      <x:c r="C102" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>Religion: Ethics and Philosophy</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>Compares religious ethics and investigates philosophical questions about religion's moral and political roles. Students examine sacredness, violence and moral doubt through ancient narrative, Socratic ethics and Hindu, Buddhist, Jewish, Christian and Islamic traditions. The course considers internal ethical debates, inequality, peace and religiously motivated social action. The second half emphasizes developing and revising an independently argued research paper on a course-related question.</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Philosophy of religion; Comparative religious ethics; Religious studies</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Sacred and holy; Religion and violence; Ethical doubt; Gilgamesh and ancient religious narrative; Socratic ethics; Hindu ethics; Buddhist ethics; Jewish ethics; Christian ethics; Islamic ethics; Religion, gender and justice; Peace and interfaith dialogue; Religious contributions to political and personal life</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>Comparative analysis of religious ethical systems; Philosophical text and argument analysis; Literature-based research; Argumentative research-paper development</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>GOSPHIL312.docx</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>820b3a0e0b106e6047332efc80278c6e452b08fd50e2ca6d36117e895ad96b3e</x:v>
+      </x:c>
+      <x:c r="K102"/>
+      <x:c r="L102"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>GOSPOLI212</x:v>
+      </x:c>
+      <x:c r="C103" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>Introduction to International Relations</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>Introduces international relations and geopolitics through competing theoretical approaches and historical and contemporary cases. Students study realism, liberalism, Marxism, constructivism, critical theory and foreign-policy analysis. Case research connects theories to conflicts, colonial relationships, economic competition and climate politics. A UN Security Council simulation requires country-position research, strategy and position papers, negotiation and collaborative resolution drafting.</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>International relations; Geopolitics; Political science</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>International state system and non-state actors; Classical and contemporary geopolitics; Realism and neorealism; Liberalism and neoliberalism; Marxism and world-systems theory; Constructivism and critical theory; Foreign-policy decision-making; War and great-power competition; Colonialism and economic relations; Climate politics; UN Security Council diplomacy</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>Theory-guided international case analysis; Historical-source analysis; Comparative foreign-policy analysis; Country-position and strategy research; Diplomatic negotiation simulation; Position-paper and resolution drafting</x:v>
+      </x:c>
+      <x:c r="I103" t="str">
+        <x:v>GOSPOLI212.docx</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>67ef7104081d8a54afa8c506f23f2ca4124aefa111199cec652a765cc8855987</x:v>
+      </x:c>
+      <x:c r="K103"/>
+      <x:c r="L103"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>GOSPOLI313</x:v>
+      </x:c>
+      <x:c r="C104" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>Peace and Conflict</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>Examines causes and dynamics of conflict and approaches to peace through legal, sociological, political and historical perspectives. Structural inequality, identity and colonial legacies are connected to international security, humanitarian law, human rights, peacebuilding and transitional justice. Students compare travelling concepts across disciplines, produce an interdisciplinary podcast, and develop an evidence-based policy brief with a research dossier. Positionality reflection addresses how assumptions shape inquiry.</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>Peace and conflict studies; International relations; Sociology; International law</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>Conflict theories and structural violence; Identity and historical grievances; Colonialism and forced migration; International peace and security; Humanitarian law and human rights; Positive, negative and hybrid peace; Local peacebuilding; Frozen conflicts; Counterterrorism and rule of law; Transitional justice; Gender and conflict; Development and peacebuilding; Reconciliation, arts and religion; Global South perspectives; Travelling concepts and researcher positionality</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>Interdisciplinary Research Process; Cross-disciplinary travelling-concept analysis; Conflict case analysis; Context and stakeholder mapping; Annotated bibliography and evidence synthesis; Policy-option appraisal; Policy-brief and background-dossier development; Researcher positionality analysis; Comparative research podcast production</x:v>
+      </x:c>
+      <x:c r="I104" t="str">
+        <x:v>GOSPOLI313.pdf</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>9b18d6d13ad9734de7883f7ce91095b135b60862161c027b117facd604e4e71e</x:v>
+      </x:c>
+      <x:c r="K104"/>
+      <x:c r="L104"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>GOSSOCI212</x:v>
+      </x:c>
+      <x:c r="C105" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>Qualitative Research Methodology</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>Develops qualitative inquiry from research design and preparation through data collection, management, analysis and dissemination. Students examine methodological foundations, ethics, positionality and reflexivity alongside interviews, focus groups, ethnography, documentary and visual approaches. Coding, thematic interpretation and NVivo support analysis. Research teams formulate a question, collect and analyze qualitative evidence, and report their methodological decisions, findings and limitations in staged assignments.</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>Qualitative research methodology; Social research</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Qualitative knowledge and research design; Ethics, positionality and reflexivity; Mixed methods; Participatory research; Interview and focus-group approaches; Ethnography and participant observation; Documentary and archival sources; Visual and participatory media; Coding and thematic interpretation; Qualitative research dissemination</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>Qualitative research design; Interviews; Focus groups; Ethnography and participant observation; Documentary and archival analysis; Visual-data analysis; Participatory video and drawing; Transcription; Qualitative coding; Thematic analysis; NVivo-supported analysis; Reflexive methodological evaluation</x:v>
+      </x:c>
+      <x:c r="I105" t="str">
+        <x:v>GOSSOCI212.docx</x:v>
+      </x:c>
+      <x:c r="J105" t="str">
+        <x:v>ea39e5374f2b280c8104221a7010299994b281b74507a6272793ba256eb83422</x:v>
+      </x:c>
+      <x:c r="K105"/>
+      <x:c r="L105"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>HCBBIOM211</x:v>
+      </x:c>
+      <x:c r="C106" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>Functional Anatomy</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>Studies human anatomical structure in relation to function through regional and body-system blocks. Skeletal, thoracic, cardiovascular, respiratory, abdominal, reproductive and lower urinary anatomy are developed through spatial reasoning, medical images, anatomical drawing and human-specimen material. Guided practicals and dissection-room observation connect three-dimensional relationships to variation. Historical, ethical and societal questions about human remains, representation and sex accompany the anatomical study; activities are framed as academic learning rather than clinical qualification.</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>Human anatomy; Functional anatomy; Biomedical ethics</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>Anatomical terminology and body planes; Medical imaging; Skeletal system and vertebral column; Thorax and pelvis; Respiratory and cardiovascular systems; Abdominal organs and vascular supply; Reproductive and lower urinary systems; Anatomical variation and intersex presentations; Human remains and dissection ethics; History and representation of the body</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>Surface-anatomy observation; Anatomical image interpretation; Scientific anatomical drawing; Three-dimensional anatomical reasoning; Guided study of human skeletal remains and anatomical specimens; Ethical reflection on anatomical practice</x:v>
+      </x:c>
+      <x:c r="I106" t="str">
+        <x:v>HCBBIOM211.docx</x:v>
+      </x:c>
+      <x:c r="J106" t="str">
+        <x:v>f52b60b33990c6eb0786bf07231aafb857ba317674baf83caa9a236975b15faf</x:v>
+      </x:c>
+      <x:c r="K106"/>
+      <x:c r="L106" t="str">
+        <x:v>Auscultation, ECG, resuscitation and defibrillation appear as guided practicals or demonstrations; the outline explicitly distinguishes these experiences from clinical skills training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>HCBBIOM312</x:v>
+      </x:c>
+      <x:c r="C107" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>Infection and Immunity</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>Examines host-microbe interactions and the immune mechanisms that protect against infection or cause disease. Microbiology and innate defence lead into antibodies, antigen recognition, lymphocyte development and memory, effector responses and mucosal immunity. Vaccination, allergy, immunodeficiency and autoimmunity connect mechanisms to clinical problems. Students analyze lymphocyte phenotypes using original flow-cytometry data and synthesize recent research in an extended and graphical abstract.</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Immunology; Medical microbiology; Infectious-disease biology</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>Infectious agents and microbial virulence; Host defence and immune evasion; Immune cells, organs and cytokines; Innate immunity and complement; Antibodies and antigen recognition; MHC and lymphocyte receptors; Lymphocyte activation, development and memory; Cell- and antibody-mediated immunity; Mucosal immunity; Vaccination and viral infections; Hypersensitivity and allergy; Immunodeficiency; Autoimmune disease; Outbreak management</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>Flow-cytometry data analysis and lymphocyte phenotyping; Clinical symptom and mechanism analysis; Medline/PubMed literature searching; Critical analysis of immunological research; Graphical synthesis of scientific findings</x:v>
+      </x:c>
+      <x:c r="I107" t="str">
+        <x:v>HCBBIOM312.pdf</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>c08f5e38dc54510386837ae1fa791204186af5bc8bc70fa980481ffb38a2bd11</x:v>
+      </x:c>
+      <x:c r="K107"/>
+      <x:c r="L107" t="str">
+        <x:v>Flow cytometry is established as analysis of supplied laboratory data; sample preparation and instrument operation are not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B108" t="str">
+        <x:v>HCBBIOM313</x:v>
+      </x:c>
+      <x:c r="C108" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D108" t="str">
+        <x:v>Mechanisms of Disease</x:v>
+      </x:c>
+      <x:c r="E108" t="str">
+        <x:v>Connects normal organ function to pathophysiology across digestive, cardiovascular, respiratory, renal, endocrine and nervous systems. Students integrate anatomy and physiology to explain symptoms, disease mechanisms, diagnostic findings, treatment and prognosis. Published clinical cases develop differential reasoning and appraisal of diagnostic procedures. A creative assignment constructs an imaginary disease whose symptoms, mechanism and proposed treatment must form a coherent pathophysiological account.</x:v>
+      </x:c>
+      <x:c r="F108" t="str">
+        <x:v>Pathophysiology; Clinical biomedical science</x:v>
+      </x:c>
+      <x:c r="G108" t="str">
+        <x:v>Organ-system disease mechanisms; Nutrition and digestive disease; Hematological and cardiovascular disease; Respiratory disease; Renal failure, dialysis and transplantation; Endocrine disorders; Neurological disease; Etiology and pathogenesis; Diagnosis, treatment and prognosis; Medical ethics; Rheumatic disease</x:v>
+      </x:c>
+      <x:c r="H108" t="str">
+        <x:v>Clinical case analysis; Differential diagnosis reasoning; Critical appraisal of diagnostic and laboratory procedures; Integration of anatomy, physiology and clinical evidence; Mechanistic modelling of an imaginary disease; Biomedical literature comparison</x:v>
+      </x:c>
+      <x:c r="I108" t="str">
+        <x:v>HCBBIOM313.docx</x:v>
+      </x:c>
+      <x:c r="J108" t="str">
+        <x:v>559a7419db8b53361aad9c25a690502009fb3eee498b6e26f4d5f40895c3c670</x:v>
+      </x:c>
+      <x:c r="K108"/>
+      <x:c r="L108" t="str">
+        <x:v>Some responsive sessions are unspecified. Clinical and laboratory procedures are analyzed through cases; hands-on diagnostic or treatment competence is not established. Optional extra research groups are outside the assessed core.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B109" t="str">
+        <x:v>HCBCOGN112</x:v>
+      </x:c>
+      <x:c r="C109" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D109" t="str">
+        <x:v>Neurobiology</x:v>
+      </x:c>
+      <x:c r="E109" t="str">
+        <x:v>Studies nervous systems and behaviour from comparative, evolutionary and physiological perspectives. Brain anatomy and laboratory introductions support analysis of animal behaviour, research models and welfare. The second part connects regulatory behaviour and biological rhythms to sleep, lifestyle drugs, mood and eating disorders. Comparative-anatomy work and a literature-based disorder report apply neurobiological concepts while animal-research assignments examine reduction, refinement and replacement.</x:v>
+      </x:c>
+      <x:c r="F109" t="str">
+        <x:v>Neurobiology; Behavioural biology; Comparative neuroscience</x:v>
+      </x:c>
+      <x:c r="G109" t="str">
+        <x:v>Nervous-system evolution and comparative anatomy; Brain cells and morphology; Cerebral circulation and nerves; Animal behaviour and welfare; Sentience and research ethics; Reduction, refinement and replacement; Enrichment and brain development; Regulatory and sexual behaviour; Lifestyle drugs; Circadian rhythms and sleep; Sleeping and eating disorders; Depression and anxiety; Gut-brain axis; Hypothalamus and pineal gland; Dying brain and consciousness</x:v>
+      </x:c>
+      <x:c r="H109" t="str">
+        <x:v>Comparative brain-anatomy analysis; Introductory microscopy and cell staining; Brain-model comparison; Ethical appraisal of animal research and the 3Rs; Literature-based analysis of neurobiological disorders</x:v>
+      </x:c>
+      <x:c r="I109" t="str">
+        <x:v>HCBCOGN112.pdf</x:v>
+      </x:c>
+      <x:c r="J109" t="str">
+        <x:v>9ee66e128e3fbc236d4ae53e58c158160b784ee8b820d16ade0dded0c5d05f8e</x:v>
+      </x:c>
+      <x:c r="K109" t="str">
+        <x:v>The PDF covers both groups 1 and 2; this record uses group 1 under the user's explicit convention for the unsuffixed filenames.</x:v>
+      </x:c>
+      <x:c r="L109"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B110" t="str">
+        <x:v>HCBGATE102</x:v>
+      </x:c>
+      <x:c r="C110" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D110" t="str">
+        <x:v>Introduction to Brain &amp; Behavior</x:v>
+      </x:c>
+      <x:c r="E110" t="str">
+        <x:v>Introduces psychological and neuroscientific explanations of behaviour and mental processes. Students study learning, intelligence, personality, self-concepts and social influence alongside neural communication, functional anatomy, development and hemispheric specialization. Later sessions introduce mental disorders, diagnostic classification, treatment and neuroscience research tools. Article and interdisciplinary case analysis connect psychological concepts to brain mechanisms and clinical questions.</x:v>
+      </x:c>
+      <x:c r="F110" t="str">
+        <x:v>Psychology; Cognitive neuroscience; Clinical psychology</x:v>
+      </x:c>
+      <x:c r="G110" t="str">
+        <x:v>History and scientific scope of psychology and neuroscience; Learning and conditioning; Intelligence; Neural signalling and action potentials; Functional brain anatomy; Brain development and neurogenesis; Personality and self-concepts; Social influence; Hemispheric specialization; Mental disorders and DSM-5-TR; Psychological treatment; Neuroimaging and electrophysiology; Computational and converging neuroscience methods</x:v>
+      </x:c>
+      <x:c r="H110" t="str">
+        <x:v>Critical analysis of psychological and neuroscientific research articles; Interdisciplinary case-study analysis; Appraisal of research approaches</x:v>
+      </x:c>
+      <x:c r="I110" t="str">
+        <x:v>HCBGATE102.pdf</x:v>
+      </x:c>
+      <x:c r="J110" t="str">
+        <x:v>a6f41bf81d59545fd4f13a097031f036f295628e82f8ca106c6b81b3a7531a72</x:v>
+      </x:c>
+      <x:c r="K110"/>
+      <x:c r="L110" t="str">
+        <x:v>Neuroscience imaging, recording and stimulation techniques are introduced; the outline does not establish hands-on acquisition or clinical treatment training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B111" t="str">
+        <x:v>HCBLIFE214</x:v>
+      </x:c>
+      <x:c r="C111" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D111" t="str">
+        <x:v>Life Science Laboratory</x:v>
+      </x:c>
+      <x:c r="E111" t="str">
+        <x:v>Provides hands-on training in biochemical, microbiological and molecular laboratory methods. Blood analysis, microbial culture and hygiene lead into bacterial transformation, green fluorescent protein production and purification, DNA isolation and analysis, and introductory bioinformatics. Students follow and sometimes adapt protocols, interpret experimental results, maintain reproducible laboratory records and communicate findings in scientific reports and figures.</x:v>
+      </x:c>
+      <x:c r="F111" t="str">
+        <x:v>Molecular biology; Biochemistry; Microbiology; Laboratory life sciences; Bioinformatics</x:v>
+      </x:c>
+      <x:c r="G111" t="str">
+        <x:v>Blood cells and proteins; Blood groups and hemograms; Aseptic culture and bacterial identification; Disinfection and sterilization; Antibiotic susceptibility; Genetically modified bacteria; GFP production and purification; DNA and plasmid analysis; PCR and restriction digestion; Protein and DNA databases; Genotype and population-genetic interpretation; Experimental reproducibility</x:v>
+      </x:c>
+      <x:c r="H111" t="str">
+        <x:v>Pipetting and workflow planning; Microscopy and blood-smear examination; Blood cell counting and hemogram measurement; ELISA; Aseptic culture and purity streaking; Bacterial identification and inhibition-zone testing; Sterilization and disinfection testing; pGLO bacterial transformation; Protein extraction and chromatographic purification; SDS-PAGE; DNA and plasmid isolation; PCR; Restriction digestion and agarose-gel electrophoresis; DNA and protein database searching; Laboratory notebook and scientific-report preparation</x:v>
+      </x:c>
+      <x:c r="I111" t="str">
+        <x:v>HCBLIFE214.pdf</x:v>
+      </x:c>
+      <x:c r="J111" t="str">
+        <x:v>aeed53713f07f1e4ba1e69eb52cc1d7f48acec576c744ad2e406b97e549ced4d</x:v>
+      </x:c>
+      <x:c r="K111"/>
+      <x:c r="L111"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B112" t="str">
+        <x:v>HCBLIFE311</x:v>
+      </x:c>
+      <x:c r="C112" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D112" t="str">
+        <x:v>Molecular Pathology and Genetics</x:v>
+      </x:c>
+      <x:c r="E112" t="str">
+        <x:v>Connects cellular pathology with molecular and genetic mechanisms of human disease. Cell injury, inflammation, repair, neoplasia and pulmonary pathology lead into inheritance, genetic variation, epigenetics, diagnosis and treatment. Students examine ethical and legal questions in genetic testing and manipulation. A two-year biomedical research proposal integrates literature, hypotheses, method selection, controls, feasibility, ethics and budgeting, and a stakeholder debate develops reasoned positions on a fictitious policy issue.</x:v>
+      </x:c>
+      <x:c r="F112" t="str">
+        <x:v>Molecular pathology; Human genetics; Molecular medicine</x:v>
+      </x:c>
+      <x:c r="G112" t="str">
+        <x:v>Cell injury and death; Acute and chronic inflammation; Tissue repair, regeneration and fibrosis; Neoplasia; Pulmonary pathology; Genes and genomes; Inheritance and chromosome abnormalities; Genetic variation; Gene regulation and epigenetics; Genotype-phenotype relationships; DNA technologies and genetic testing; Genetic therapies and cell manipulation; Genetic ethics and law</x:v>
+      </x:c>
+      <x:c r="H112" t="str">
+        <x:v>Biomedical literature retrieval and review; Research-proposal design; Hypothesis and experimental-control formulation; Research-method selection and feasibility assessment; Research timeline and resource planning; Stakeholder-based ethical argument analysis</x:v>
+      </x:c>
+      <x:c r="I112" t="str">
+        <x:v>HCBLIFE311.pdf</x:v>
+      </x:c>
+      <x:c r="J112" t="str">
+        <x:v>8530671af2a2aee4a7590f93ed855e89014bfba65f2c1eb770faff68acd181c6</x:v>
+      </x:c>
+      <x:c r="K112"/>
+      <x:c r="L112" t="str">
+        <x:v>Laboratory methods are selected and justified for proposed research; the outline does not establish hands-on laboratory training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B113" t="str">
+        <x:v>HCBPSYC212</x:v>
+      </x:c>
+      <x:c r="C113" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D113" t="str">
+        <x:v>Abnormal Psychology</x:v>
+      </x:c>
+      <x:c r="E113" t="str">
+        <x:v>Examines mental health and psychopathology across the lifespan using a biopsychosocial perspective. Historical views, classification and assessment frame biological, psychological, cultural and social explanations of disorders and treatment. Case-based work applies diagnostic concepts to varied presentations. A structured literature-based essay investigates a focused mental-health question through explicit searching, source selection, evidence appraisal and synthesis, with optional use of PRISMA reporting tools.</x:v>
+      </x:c>
+      <x:c r="F113" t="str">
+        <x:v>Abnormal psychology; Clinical psychology; Psychopathology</x:v>
+      </x:c>
+      <x:c r="G113" t="str">
+        <x:v>Mental-disorder concepts and stigma; Historical and contemporary psychopathology; Biopsychosocial causation; Clinical assessment and diagnostic classification; Stress and health; Anxiety and obsessive-compulsive disorders; Mood disorders; Somatic and dissociative disorders; Psychotic disorders; Eating and personality disorders; Substance-related and neurocognitive disorders; Sexuality and mental health; Childhood and adolescent disorders; Forensic psychology; Culture and emotion regulation</x:v>
+      </x:c>
+      <x:c r="H113" t="str">
+        <x:v>Diagnostic case analysis; Application and critique of DSM criteria; Biopsychosocial case formulation; Structured literature searching and screening; Source-quality appraisal; Evidence synthesis; Critical evaluation of etiological and intervention models</x:v>
+      </x:c>
+      <x:c r="I113" t="str">
+        <x:v>HCBPSYC212.pdf</x:v>
+      </x:c>
+      <x:c r="J113" t="str">
+        <x:v>34712883e06713d7a4bfb72b9404358665fd8bcd1033b8c92d9dcbc97fa31f6b</x:v>
+      </x:c>
+      <x:c r="K113"/>
+      <x:c r="L113" t="str">
+        <x:v>The research essay uses published literature; original clinical data collection and treatment delivery are not established. PRISMA is optional rather than a mandatory method.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="A114" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B114" t="str">
+        <x:v>HCBPSYC312</x:v>
+      </x:c>
+      <x:c r="C114" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D114" t="str">
+        <x:v>Psychodiagnostics &amp; Psychotherapies</x:v>
+      </x:c>
+      <x:c r="E114" t="str">
+        <x:v>Introduces clinical psychological assessment and major psychotherapeutic approaches across the lifespan. Students study ethics, diagnostic systems, test reliability and validity, interviews, personality and cognitive assessment, then psychodynamic, behavioural, cognitive, humanistic, systemic and integrative treatments. Training sessions develop introductory administration, scoring and interpretation skills. A psychodiagnostic case report integrates findings and treatment recommendations, while self-monitoring examines developing clinical skills.</x:v>
+      </x:c>
+      <x:c r="F114" t="str">
+        <x:v>Clinical psychology; Psychological assessment; Psychotherapy</x:v>
+      </x:c>
+      <x:c r="G114" t="str">
+        <x:v>Clinical attitude and ethics; Diagnostic classification; Reliability and validity; Clinical interviews; Personality inventories and projective techniques; Cognitive and neuropsychological assessment; Behavioural and biological assessment; Psychological reporting; Psychodynamic and behavioural therapies; Cognitive therapy and CBT; Person-centered and family therapies; Integrative psychotherapy; Treatment outcomes and evidence; Child and adolescent clinical psychology</x:v>
+      </x:c>
+      <x:c r="H114" t="str">
+        <x:v>Clinical interviewing practice; Introductory psychological-test administration, scoring and interpretation; Psychometric appraisal; Behavioural observation; Integration of assessment data; Psychodiagnostic report writing; Clinical case and therapy-session analysis; Reflective monitoring of clinical skills</x:v>
+      </x:c>
+      <x:c r="I114" t="str">
+        <x:v>HCBPSYC312.pdf</x:v>
+      </x:c>
+      <x:c r="J114" t="str">
+        <x:v>c130121d25ab405cf898452fdc02c1d0b50175a0b8354d3ff567a67165feada4</x:v>
+      </x:c>
+      <x:c r="K114"/>
+      <x:c r="L114"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="A115" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B115" t="str">
+        <x:v>HCBPSYC313</x:v>
+      </x:c>
+      <x:c r="C115" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D115" t="str">
+        <x:v>Advanced Research Seminar: Statistical Synthesis of Evidence in Medical and Behavioral Sciences</x:v>
+      </x:c>
+      <x:c r="E115" t="str">
+        <x:v>Teaches systematic review and meta-analysis for synthesizing evidence in medical, behavioural and related research. Students define review questions, search and select studies, extract and code findings, assess bias and compute effect sizes. Hands-on R work fits fixed- and random-effects models, examines heterogeneity and moderators, conducts meta-regression and investigates publication bias. A group project completes a small meta-analysis and presents its methods and results in a research poster.</x:v>
+      </x:c>
+      <x:c r="F115" t="str">
+        <x:v>Evidence synthesis; Meta-analysis; Applied statistics; Research methodology</x:v>
+      </x:c>
+      <x:c r="G115" t="str">
+        <x:v>Systematic-review purpose and limitations; Review protocols and scope; Literature searching and inclusion criteria; Data extraction and study coding; Risk of bias; Effect-size types and transformations; Fixed- and random-effects models; Effect heterogeneity; Moderators and subgroup differences; Meta-regression; Publication bias; Research synthesis and reporting</x:v>
+      </x:c>
+      <x:c r="H115" t="str">
+        <x:v>Systematic literature review; Database searching and study screening; Study-data extraction and coding; Critical risk-of-bias appraisal; R programming and data management; Effect-size calculation and conversion; Fixed- and random-effects meta-analysis; Moderator and subgroup analysis; Meta-regression; Publication-bias analysis; Meta-analytic visualization and reporting</x:v>
+      </x:c>
+      <x:c r="I115" t="str">
+        <x:v>HCBPSYC313.docx</x:v>
+      </x:c>
+      <x:c r="J115" t="str">
+        <x:v>3145c5e8b975e5c1b783ef3d740feb983e1bf86580e9f1d25ee2bef84479abc4</x:v>
+      </x:c>
+      <x:c r="K115" t="str">
+        <x:v>The heading says Fall 2026, while the detailed schedule runs from January to May 2026. The authoritative ZIP semester is 2026h1.</x:v>
+      </x:c>
+      <x:c r="L115"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>HCBPSYC314</x:v>
+      </x:c>
+      <x:c r="C116" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>Lifespan Developmental Psychology</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>Examines physical, cognitive, emotional, social and personality development from prenatal life through old age and death. Biological and environmental influences are considered alongside attachment, education, relationships, cultural differences and developmental psychopathology. Students connect theoretical perspectives to case studies, assessment and interventions at different life stages. A life-story interview with an adult over fifty applies developmental concepts through interviewing, analysis and a written report.</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>Developmental psychology; Lifespan psychology</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>Developmental theories; Genetics and environment; Prenatal development and birth; Infancy and attachment; Cognitive and psychomotor development; Early and middle childhood; Play and education; Adolescence and psychopathology; Emerging and early adulthood; Middle and late adulthood; Relationships and personality development; Care and developmental interventions; Death, dying, grief and bereavement</x:v>
+      </x:c>
+      <x:c r="H116" t="str">
+        <x:v>Life-story interviewing; Theory-guided lifespan interview analysis; Developmental case-study analysis; Critical appraisal of developmental research and assessment reports</x:v>
+      </x:c>
+      <x:c r="I116" t="str">
+        <x:v>HCBPSYC314.pdf</x:v>
+      </x:c>
+      <x:c r="J116" t="str">
+        <x:v>df78b331ab8e4b9d39f3fa7e314aaca2ed3729ee3f806ff033bd8acbcf81b14a</x:v>
+      </x:c>
+      <x:c r="K116"/>
+      <x:c r="L116"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>MCCCOMM211</x:v>
+      </x:c>
+      <x:c r="C117" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>Style and Meaning</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>Studies how linguistic choices produce meaning and interpretive effects, principally in literary texts but also in nonfiction. Students connect linguistic description to interpretation across grammar, discourse and cognition. Stylistic frameworks address foregrounding, dialogue, narration, modality, transitivity, deixis, schemas, construal and text worlds. Frequent analysis exercises lead to an original, research-supported stylistic analysis of a selected text.</x:v>
+      </x:c>
+      <x:c r="F117" t="str">
+        <x:v>Stylistics; Linguistics; Literary studies; Cognitive poetics</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>Foregrounding and deviation; Morphology, syntax and lexical semantics; Register and cohesion; Dialogue and turn-taking; Cooperative principle; Speech and thought presentation; Modality and point of view; Transitivity and ideology; Narrative urgency; Figure and ground; Deixis and deictic shift; Schemas, scripts and prototypes; Cognitive grammar and construal; Text-world theory; Negation and lacuna</x:v>
+      </x:c>
+      <x:c r="H117" t="str">
+        <x:v>Linguistic stylistic analysis; Close textual analysis; Discourse and conversation analysis; Speech and thought presentation analysis; Modality and transitivity analysis; Deictic and cognitive-grammar analysis; Text-world analysis; Framework-based interpretation supported by retrievable textual evidence</x:v>
+      </x:c>
+      <x:c r="I117" t="str">
+        <x:v>MCCCOMM211.docx</x:v>
+      </x:c>
+      <x:c r="J117" t="str">
+        <x:v>0b62aeabc122cba3c36f65f323796f08929a5560bb0b7fa289d3f2830154a535</x:v>
+      </x:c>
+      <x:c r="K117"/>
+      <x:c r="L117"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="A118" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B118" t="str">
+        <x:v>MCCCOMM213</x:v>
+      </x:c>
+      <x:c r="C118" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Rhetoric in Action</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>Applies rhetoric through community-engaged work with local primary-school children. Students develop their own public-speaking, debating and storytelling skills, then design and iteratively refine age-appropriate teaching activities with school partners. On-site coaching and a final public-speaking event connect rhetorical education to civic participation and confidence. Structured reflection examines reciprocity, cultural sensitivity, personal development and the practical challenges of community-engaged teaching.</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>Rhetoric; Communication education; Community-engaged pedagogy</x:v>
+      </x:c>
+      <x:c r="G118" t="str">
+        <x:v>Public work of rhetoric; Community-engaged learning and reciprocity; Public speaking and debate; Storytelling; Children's rhetorical confidence and civic participation; Rhetorical teaching and coaching; Cultural sensitivity; Collaboration with community partners; Experiential and reflective learning</x:v>
+      </x:c>
+      <x:c r="H118" t="str">
+        <x:v>Public-speaking and debate coaching; Storytelling exercises; Iterative design and revision of teaching materials; Practice-based rhetorical instruction; Gibbs reflective-cycle analysis; Public-speaking event design and evaluation</x:v>
+      </x:c>
+      <x:c r="I118" t="str">
+        <x:v>MCCCOMM213.docx</x:v>
+      </x:c>
+      <x:c r="J118" t="str">
+        <x:v>b29d6d99f724856e6da49f999a3850d576e9369c6d2bb9fb46660c6b8b0b9e66</x:v>
+      </x:c>
+      <x:c r="K118"/>
+      <x:c r="L118"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B119" t="str">
+        <x:v>MCCCOMM312</x:v>
+      </x:c>
+      <x:c r="C119" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>Creative Communication Laboratory</x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>Studies and develops creative communication through poetry, performance and critically articulated artistic practice. Students move from lyric foundations to constrained and experimental forms, attending to sound, rhythm, imagery, voice and embodiment. Close reading and creative workshops lead into an independent traditional or hybrid project grounded in scholarship and aesthetic traditions. Revision and reflection require students to justify formal, conceptual and procedural choices.</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>Creative writing; Poetics; Performance studies</x:v>
+      </x:c>
+      <x:c r="G119" t="str">
+        <x:v>Meaning and formal experimentation; Lyric poetry; Poetic sound and rhythm; Imagery and voice; Embodiment and performance; Constraint and formal deviation; Experimental poetry; Hybrid and digitally mediated forms; Creative process and revision; Aesthetic traditions and conceptual coherence</x:v>
+      </x:c>
+      <x:c r="H119" t="str">
+        <x:v>Close poetic reading and listening; Constraint-based composition; Poetic and performative experimentation; Structured drafting and revision; Critical analysis of creative decisions; Independent practice-based creative inquiry</x:v>
+      </x:c>
+      <x:c r="I119" t="str">
+        <x:v>MCCCOMM312.pdf</x:v>
+      </x:c>
+      <x:c r="J119" t="str">
+        <x:v>feb6d6e6af4fdbe78c724ef139c9e135fbe38aa5b1c6e203fe1b7a7c0fcdbd02</x:v>
+      </x:c>
+      <x:c r="K119"/>
+      <x:c r="L119" t="str">
+        <x:v>Final-project media are chosen individually. Singing, songwriting and music performance are explicitly excluded; sound work must function as poetic, linguistic or conceptual material.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>MCCHEAM112</x:v>
+      </x:c>
+      <x:c r="C120" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Introduction to World Archaeology: Craft, technology and community identity</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>Examines how making objects shaped communities and identities from the Neolithic through antiquity across Europe, Asia and Africa. Artefacts, production technologies and craft organization are interpreted in relation to social status, religion, gender, exchange and environmental settings. Students produce an archaeological catalogue description and technical drawings, research a craft-related question and design a hands-on educational game. A small contemporary-archaeology project collects local material evidence and proposes a testable interpretation.</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>Archaeology; Material culture studies; Ancient social history</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>Materiality, craft and cognition; Settlement and landscape; Neolithic and Bronze Age communities; Craft production and social hierarchy; Trade and exchange; Pottery and iconography; Seals, textiles and elite identities; Domestic and urban craft spaces; Archaeological interpretation; Ancient technology and community identity; Contemporary archaeology</x:v>
+      </x:c>
+      <x:c r="H120" t="str">
+        <x:v>Artefact observation, measurement and cataloguing; Archaeological technical drawing; Visual and stylistic analysis; Comparative material-culture analysis; Archaeological database and literature research; Material-evidence-based argumentation; Archaeological educational-game design; Contemporary archaeological data collection and hypothesis development</x:v>
+      </x:c>
+      <x:c r="I120" t="str">
+        <x:v>MCCHEAM112.docx</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>b0fb78688764073e1a2ea37cd115e02546d204fb5dbf9a85f91becb344a79691</x:v>
+      </x:c>
+      <x:c r="K120"/>
+      <x:c r="L120" t="str">
+        <x:v>The contemporary project proposes how to test an interpretation in future research; students are not required to carry out that subsequent test. Field excavation training is not established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B121" t="str">
+        <x:v>MCCHEAM211</x:v>
+      </x:c>
+      <x:c r="C121" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>African Art and Heritage</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>Introduces African art and heritage with particular attention to western African visual traditions and their cultural, religious and social meanings. Students study sculpture, masks and other forms across regional contexts before tracing African art's role in European modernism, the Harlem Renaissance and African artistic renewal. Colonial dispossession, museum collecting and restitution form a major later strand. An independent paper develops a research question supported by scholarly evidence.</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>African art history; Cultural heritage studies; Museum studies</x:v>
+      </x:c>
+      <x:c r="G121" t="str">
+        <x:v>Western African artistic traditions; Sculpture, masks and visual languages; Art, religion and social authority; Regional traditions in Nigeria, the Niger region, Atlantic forests and Congo; African influences on European modernism; Harlem Renaissance and diaspora; Art Nègre and the Ecole de Dakar; Colonial looting; Universal museums; Museum acquisition and display; Restitution and repatriation</x:v>
+      </x:c>
+      <x:c r="H121" t="str">
+        <x:v>Visual and contextual art-historical analysis; Comparative interpretation of artistic traditions; Analysis of primary artistic and critical texts; Heritage-restitution case analysis; Scholarly literature review and annotated bibliography; Independent art-historical research</x:v>
+      </x:c>
+      <x:c r="I121" t="str">
+        <x:v>MCCHEAM211.docx</x:v>
+      </x:c>
+      <x:c r="J121" t="str">
+        <x:v>277bf41797d207507eda599b018e4a69b9e64ff1c418fd0e0301534980cbfedf</x:v>
+      </x:c>
+      <x:c r="K121"/>
+      <x:c r="L121"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B122" t="str">
+        <x:v>MCCHEAM313</x:v>
+      </x:c>
+      <x:c r="C122" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Greek Art &amp; Archaeology Research Seminar: Art, Cult &amp; Gender in the Ancient Greek World</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>Investigates how Greek art, craft and ritual shaped identities, especially gendered identities. An archaeological chronology provides foundations for studying dedications, burial, cult, religious iconography, law, medicine and magic. Students combine material evidence with texts and scholarship in an independent research paper based on primary archaeological data. A contextualized artefact animation or storyboard and a research dialogue extend interpretation and communication of the findings.</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>Greek archaeology; Ancient art history; Ancient religion; Gender studies</x:v>
+      </x:c>
+      <x:c r="G122" t="str">
+        <x:v>Greek material culture and stylistic chronology; Art, craft and ritual; Gendered identities and social status; Votives and funerary objects; Cult and cognition; Women and religious practice; Law, courts and religion; Magic, medicine and agency; Curse tablets and amulets; Ritual continuity and change; Ancient art in modern interpretation</x:v>
+      </x:c>
+      <x:c r="H122" t="str">
+        <x:v>Archaeological stylistic and iconographic analysis; Primary archaeological dataset compilation and interpretation; Comparative analysis of material and textual evidence; Theory-guided study of gender and ritual; Critical evaluation of archaeological interpretations; Historically contextualized artefact storytelling and storyboarding</x:v>
+      </x:c>
+      <x:c r="I122" t="str">
+        <x:v>MCCHEAM313.docx</x:v>
+      </x:c>
+      <x:c r="J122" t="str">
+        <x:v>db8dbab35ed5e9571053790ef34c465cf635e209c9ac8dca1549a164b616394b</x:v>
+      </x:c>
+      <x:c r="K122"/>
+      <x:c r="L122" t="str">
+        <x:v>Research datasets and analytical techniques vary by paper; quantitative analysis is offered as a possible approach rather than a universal requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B123" t="str">
+        <x:v>MCCLITR112</x:v>
+      </x:c>
+      <x:c r="C123" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Great Literary Works</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>Surveys major literary works from ancient epic to modern and later fiction, connecting literary form to questions of humanity, mortality, gender, freedom, community and civilization. Students compare genres and recurring motifs through works including Gilgamesh, Greek tragedy, confessional writing, framed tales, philosophical satire, colonial narratives and modernist fiction. Text-focused analysis and engagement with criticism develop interpretation of theme, technique and cultural context.</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>Literary studies; Comparative literature; Literary criticism</x:v>
+      </x:c>
+      <x:c r="G123" t="str">
+        <x:v>Literature, canon and world literature; Epic and heroism; Tragedy, fate and identity; Autobiography and memory; Framed storytelling and narrative power; Gender and agency; Essay and philosophical tale; Satire and irony; Colonialism and its critique; Modernist narration and subjectivity; Alienation and family; Art, sexuality and civilization; Magical realism</x:v>
+      </x:c>
+      <x:c r="H123" t="str">
+        <x:v>Close literary reading; Formalist analysis of genre, theme and technique; Comparative textual interpretation; Narrative analysis; Critical-source interpretation and integration</x:v>
+      </x:c>
+      <x:c r="I123" t="str">
+        <x:v>MCCLITR112.docx</x:v>
+      </x:c>
+      <x:c r="J123" t="str">
+        <x:v>18588f6a8311d3dca836a08a123446be141db6f4ac2e78c6b3e3729f34d382a8</x:v>
+      </x:c>
+      <x:c r="K123"/>
+      <x:c r="L123"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B124" t="str">
+        <x:v>MCCLITR212</x:v>
+      </x:c>
+      <x:c r="C124" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Life and Travel Writing</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>Studies life narrative in literature and popular culture, including memoir, autobiography, diary, personal essay, travel writing and digital self-presentation. Memory, experience, identity, embodiment and agency frame debates about autobiographical truth, fiction, ethics, trauma and cultural positioning. Close readings connect popular, intellectual and migrant memoirs to theory. Students apply analytical concepts in a personal writing portfolio and an independent comparative or focused life-narrative project.</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>Life-writing studies; Literary studies; Autobiographical criticism</x:v>
+      </x:c>
+      <x:c r="G124" t="str">
+        <x:v>Autobiography and memoir culture; Fact, fiction and autobiographical truth; Autobiographical pact; Self and multiple identities; Individual and collective memory; Experience, embodiment and agency; Ethics and traumatic memory; Grief and disability narratives; Popular memoir and narrative technique; Digital self-presentation; Travel and spiritual self-fashioning; Migration, language and cultural identity</x:v>
+      </x:c>
+      <x:c r="H124" t="str">
+        <x:v>Close life-narrative analysis; Smith and Watson's strategies for reading life narratives; Theory-guided analysis of memory, identity, embodiment and agency; Comparative textual and contextual interpretation; Structured autobiographical creative writing</x:v>
+      </x:c>
+      <x:c r="I124" t="str">
+        <x:v>MCCLITR212.docx</x:v>
+      </x:c>
+      <x:c r="J124" t="str">
+        <x:v>21e144b10f08588bae7f92cc94ff911b36e6152fa74b618d1a488a834f770f2d</x:v>
+      </x:c>
+      <x:c r="K124"/>
+      <x:c r="L124" t="str">
+        <x:v>The extensive annotated appendix suggests alternative texts for final projects; these are not all confirmed shared readings or independent course topics.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B125" t="str">
+        <x:v>MCCMEDI211</x:v>
+      </x:c>
+      <x:c r="C125" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>From T.V. to TikTok: Mainstream Media</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>Examines American social history and everyday life from the mid-twentieth century through contemporary media. Storytelling, power and representation connect television, film and digital forms to conformity, identity and imagined futures. Students analyze 1950s media, compare dominant portrayals with Indigenous self-representation, and investigate disability representation. Futures-oriented projects create a speculative television-episode proposal and imagine possibilities that center disabled people.</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>Media studies; Social and cultural history; Disability studies; Futures studies</x:v>
+      </x:c>
+      <x:c r="G125" t="str">
+        <x:v>Media storytelling and power; American everyday life; 1950s television and conformity; Science fiction and social anxieties; Media futures and marginalization; Indigenous representation and self-representation; Disability stereotypes and visibility; Authentic voice and cultural agency; Future foresight and inclusive scenarios</x:v>
+      </x:c>
+      <x:c r="H125" t="str">
+        <x:v>Historical analysis of primary media sources; Comparative representation analysis; Future-foresight scenario development; Theory-based speculative narrative design; Disability-centered futures inquiry</x:v>
+      </x:c>
+      <x:c r="I125" t="str">
+        <x:v>MCCMEDI211.docx</x:v>
+      </x:c>
+      <x:c r="J125" t="str">
+        <x:v>9285b3093540b0d9fcbc8dfb809c0dad90c65d83e52de6300f85a65feb7b4995</x:v>
+      </x:c>
+      <x:c r="K125" t="str">
+        <x:v>The learning-outcomes activities retain references to projects and visits absent from the detailed assessment and schedule, including a disability blog, a banned-books broadcast and archive or museum research.</x:v>
+      </x:c>
+      <x:c r="L125" t="str">
+        <x:v>The outline is a working draft for Summer 2026, with June dates and many session details marked TBA. The extraction follows the specified television, speculative-episode and disability-futures projects.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B126" t="str">
+        <x:v>MCCMEDI212</x:v>
+      </x:c>
+      <x:c r="C126" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D126" t="str">
+        <x:v>Media &amp; the Environment</x:v>
+      </x:c>
+      <x:c r="E126" t="str">
+        <x:v>Examines how visual, audiovisual, sound and digital media shape understanding of ecological problems and human-nonhuman relations. Environmental-humanities concepts guide close analysis of images, narratives and aesthetic strategies across cultural and historical contexts. Students investigate how scientific knowledge, risk and lived experience become representations that influence ethics, public debate and sustainability. A final analytical paper or media-based project develops an argument grounded in course theory.</x:v>
+      </x:c>
+      <x:c r="F126" t="str">
+        <x:v>Environmental humanities; Media studies; Ecocriticism</x:v>
+      </x:c>
+      <x:c r="G126" t="str">
+        <x:v>Environmental representation; Anthropocene; Animal representation and human-nonhuman relations; Deep time and ecological temporality; Biocentrism and environmental justice; Contested ideas of nature; Indigenous and postcolonial media; Ecological risk and scientific knowledge; Environmental affect and perception; Agency, scale and responsibility; Sustainability discourse</x:v>
+      </x:c>
+      <x:c r="H126" t="str">
+        <x:v>Close film, image and sound analysis; Comparative analysis of media forms and representational strategies; Ecocritical interpretation; Theory-based analytical or creative media inquiry</x:v>
+      </x:c>
+      <x:c r="I126" t="str">
+        <x:v>MCCMEDI212.pdf</x:v>
+      </x:c>
+      <x:c r="J126" t="str">
+        <x:v>ff2c8223c683e2dd1ee8d2c3e078781f18392d25fbf5a7226d95c52de6362c0d</x:v>
+      </x:c>
+      <x:c r="K126"/>
+      <x:c r="L126" t="str">
+        <x:v>The outline provides phases rather than a detailed reading schedule, and final-project media are individually chosen; specific production techniques cannot be established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="A127" t="str">
+        <x:v>2026h1</x:v>
+      </x:c>
+      <x:c r="B127" t="str">
+        <x:v>MCCMEDI312</x:v>
+      </x:c>
+      <x:c r="C127" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D127" t="str">
+        <x:v>The Documentary</x:v>
+      </x:c>
+      <x:c r="E127" t="str">
+        <x:v>Studies documentary history, modes and styles alongside practical documentary production. Students analyze nonfiction representation in historical, social, ethical and aesthetic contexts, from early and Soviet filmmaking through direct cinema and contemporary forms. Topics include propaganda, advocacy, ethnography, history, nature, audio and interactive documentary. Production workshops guide a short film through preproduction, filming and postproduction, with reflection on interviewing and representational choices.</x:v>
+      </x:c>
+      <x:c r="F127" t="str">
+        <x:v>Documentary studies; Film studies; Media production</x:v>
+      </x:c>
+      <x:c r="G127" t="str">
+        <x:v>Documentary definition, modes and ethics; Early documentary and city symphonies; Soviet filmmaking; European documentary traditions; Direct cinema and cinéma vérité; Audio and public-affairs documentary; Propaganda and advocacy; Historical and ethnographic documentary; Nature documentary; Mockumentary; Interactive and autobiographical documentary; Documentary aesthetics</x:v>
+      </x:c>
+      <x:c r="H127" t="str">
+        <x:v>Critical documentary analysis; Historical and contextual film comparison; Documentary research and interviewing; Script, storyboard and shot-list development; Preproduction planning; Documentary filming and postproduction; Reflective evaluation of production practice</x:v>
+      </x:c>
+      <x:c r="I127" t="str">
+        <x:v>MCCMEDI312.docx</x:v>
+      </x:c>
+      <x:c r="J127" t="str">
+        <x:v>7c826bfcf158f3050d161a8f6e78dcec4f30e62d38bc15fec051e6d6b8fed526</x:v>
+      </x:c>
+      <x:c r="K127"/>
+      <x:c r="L127"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Append 2025h2 PDF and Word outlines to cumulative course database
</commit_message>
<xml_diff>
--- a/course-outline-database/UCR_Course_Outline_Database.xlsx
+++ b/course-outline-database/UCR_Course_Outline_Database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="1" r:id="R566cc85d65a942de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="1" r:id="R98640de413aa4c2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4705,6 +4705,2432 @@
       <x:c r="K127"/>
       <x:c r="L127"/>
     </x:row>
+    <x:row r="128">
+      <x:c r="A128" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B128" t="str">
+        <x:v>ACCPPDE101</x:v>
+      </x:c>
+      <x:c r="C128" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D128" t="str">
+        <x:v>Personal and professional development</x:v>
+      </x:c>
+      <x:c r="E128" t="str">
+        <x:v>Develops academic communication, reflective learning and civic engagement through connected individual and community projects. Students learn to locate and evaluate academic sources, construct arguments and write a literature review, while examining responsible use of AI. A personal development plan sets learning goals and documents reflection. Work with societal partners applies these skills to a collaboratively designed response to a local issue.</x:v>
+      </x:c>
+      <x:c r="F128" t="str">
+        <x:v>Academic communication; Personal and professional development; Civic engagement</x:v>
+      </x:c>
+      <x:c r="G128" t="str">
+        <x:v>Academic source evaluation; Research questions and thesis statements; Argumentation; Literature reviews; Paraphrasing and referencing; Responsible academic use of AI; Reflective learning; Self-efficacy; Stress and time management; Community engagement and knowledge diversity</x:v>
+      </x:c>
+      <x:c r="H128" t="str">
+        <x:v>Academic literature searching; Critical literature review; Argument analysis; Reflective writing; Community-engaged project design</x:v>
+      </x:c>
+      <x:c r="I128" t="str">
+        <x:v>ACCPPDE101.docx</x:v>
+      </x:c>
+      <x:c r="J128" t="str">
+        <x:v>cdfda2aa4808cf1d9d45b00e2997fddcea2b8ff6c382a433eec05d14354a84e7</x:v>
+      </x:c>
+      <x:c r="K128"/>
+      <x:c r="L128" t="str">
+        <x:v>Community-project subjects depend on the societal partners and are not specified in the outline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B129" t="str">
+        <x:v>BENBUSI111</x:v>
+      </x:c>
+      <x:c r="C129" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D129" t="str">
+        <x:v>Foundations of Business and Management</x:v>
+      </x:c>
+      <x:c r="E129" t="str">
+        <x:v>Introduces how businesses operate, make decisions and create economic and social value. Management theory, organizational structure and competitive positioning lead into responsible and sustainable business, digital and AI transformation, globalization and resilience. Students investigate a real company's response to these challenges and use a business simulation to examine how finance, human resources, operations, marketing and sales interact in managerial decision-making.</x:v>
+      </x:c>
+      <x:c r="F129" t="str">
+        <x:v>Business administration; Management; Business economics</x:v>
+      </x:c>
+      <x:c r="G129" t="str">
+        <x:v>Economic activity and capitalism; Firm ownership and entrepreneurship; Management and leadership; Organizational structure; Competitive positioning; Management theories; Corporate social responsibility; Business sustainability; Digital and AI transformation; Globalization; Organizational resilience; Finance and accounting; Human resource management; Operations management; Marketing and sales</x:v>
+      </x:c>
+      <x:c r="H129" t="str">
+        <x:v>Strategic business analysis; Company case analysis; Business simulation; Interpretation of company performance data</x:v>
+      </x:c>
+      <x:c r="I129" t="str">
+        <x:v>BENBUSI111.pdf</x:v>
+      </x:c>
+      <x:c r="J129" t="str">
+        <x:v>a467540cd6c0da888dc76f15b79b1c76db04875539602e8605232a0c97517f9a</x:v>
+      </x:c>
+      <x:c r="K129"/>
+      <x:c r="L129"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B130" t="str">
+        <x:v>BENECON111</x:v>
+      </x:c>
+      <x:c r="C130" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D130" t="str">
+        <x:v>Introduction to Economics</x:v>
+      </x:c>
+      <x:c r="E130" t="str">
+        <x:v>Introduces microeconomic principles and short-run macroeconomic analysis. Students study supply and demand, strategic interaction, consumer choice, production, costs and perfect competition before examining aggregate output, unemployment, inflation, goods and financial markets. Algebraic exercises and graphical analysis connect individual decisions and market outcomes to the IS–LM account of the economy.</x:v>
+      </x:c>
+      <x:c r="F130" t="str">
+        <x:v>Economics; Microeconomics; Macroeconomics</x:v>
+      </x:c>
+      <x:c r="G130" t="str">
+        <x:v>Supply and demand; Game theory; Rational consumer choice; Individual and market demand; Production; Costs; Perfect competition; Aggregate output; Unemployment and inflation; Goods markets; Financial markets; IS–LM model</x:v>
+      </x:c>
+      <x:c r="H130" t="str">
+        <x:v>Algebraic economic modelling; Graphical economic analysis; Game-theoretic analysis</x:v>
+      </x:c>
+      <x:c r="I130" t="str">
+        <x:v>BENECON111.pdf</x:v>
+      </x:c>
+      <x:c r="J130" t="str">
+        <x:v>eb8fa90c582d83f975bd9c1f8af153aa371219b932b72ef242823ec667f8dc77</x:v>
+      </x:c>
+      <x:c r="K130" t="str">
+        <x:v>The outline identifies the course as SSCECON104; the authoritative filename code is BENECON111.</x:v>
+      </x:c>
+      <x:c r="L130"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>BENECON211</x:v>
+      </x:c>
+      <x:c r="C131" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>International Macroeconomics</x:v>
+      </x:c>
+      <x:c r="E131" t="str">
+        <x:v>Examines how economies function in the short, medium and long run. Goods, financial and labour markets are connected through IS–LM and Phillips-curve models, followed by growth, capital accumulation and technological change. Students study expectations, open-economy relationships and policy, using algebra, graphs and macroeconomic data to interpret economic outcomes and evaluate fiscal and monetary decisions.</x:v>
+      </x:c>
+      <x:c r="F131" t="str">
+        <x:v>Economics; Macroeconomics; International economics</x:v>
+      </x:c>
+      <x:c r="G131" t="str">
+        <x:v>Goods and financial markets; IS–LM model; Labour markets; Inflation and unemployment; Phillips curve; IS–LM–PC model; Economic growth; Saving and capital accumulation; Technological change; Expectations; Open-economy macroeconomics; Fiscal and monetary policy</x:v>
+      </x:c>
+      <x:c r="H131" t="str">
+        <x:v>Algebraic macroeconomic modelling; Graphical macroeconomic analysis; Macroeconomic data analysis</x:v>
+      </x:c>
+      <x:c r="I131" t="str">
+        <x:v>BENECON211.pdf</x:v>
+      </x:c>
+      <x:c r="J131" t="str">
+        <x:v>54dedf164dd75b905123ecacbd46ab709d8a0c8da10fca6bb4a0502a4698b3a6</x:v>
+      </x:c>
+      <x:c r="K131" t="str">
+        <x:v>The outline identifies the course as SSCECON208; the authoritative filename code is BENECON211.</x:v>
+      </x:c>
+      <x:c r="L131"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>BENGATE101</x:v>
+      </x:c>
+      <x:c r="C132" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>Entrepreneurship and New Venture Creation</x:v>
+      </x:c>
+      <x:c r="E132" t="str">
+        <x:v>Introduces entrepreneurship by developing a new venture from an initial problem to a business plan and investor pitch. Students apply design thinking to frame opportunities, generate and test solutions, validate markets and refine a value proposition. Business models, marketing, financial planning, resourcing and funding connect commercial and social aims to venture feasibility, while entrepreneur case analysis and reflection examine the entrepreneurial process.</x:v>
+      </x:c>
+      <x:c r="F132" t="str">
+        <x:v>Entrepreneurship; Business administration</x:v>
+      </x:c>
+      <x:c r="G132" t="str">
+        <x:v>Entrepreneurial mindset; Commercial and social entrepreneurship; Opportunity and problem framing; Value propositions; Market validation; Business models; Go-to-market strategy; Revenue and cost structures; Pricing and margins; Venture finance and funding; Resource mobilization; Venture growth and scaling</x:v>
+      </x:c>
+      <x:c r="H132" t="str">
+        <x:v>Design thinking; Divergent and convergent ideation; Prototyping and concept testing; Market analysis; Business Model Canvas; Financial planning; Business-plan development; Entrepreneur case analysis</x:v>
+      </x:c>
+      <x:c r="I132" t="str">
+        <x:v>BENGATE101.pdf</x:v>
+      </x:c>
+      <x:c r="J132" t="str">
+        <x:v>b3b0e1829f0d95288724a4f90bfe6d565b258452e6778958b4c96fc6af216322</x:v>
+      </x:c>
+      <x:c r="K132"/>
+      <x:c r="L132"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>BENLEAD111</x:v>
+      </x:c>
+      <x:c r="C133" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>Personal Leadership</x:v>
+      </x:c>
+      <x:c r="E133" t="str">
+        <x:v>Introduces leadership theory with an emphasis on self-awareness and personal development. Transformational, authentic and adaptive leadership are studied alongside Covey's seven habits, emotional intelligence, personality, values and goal-setting. Students analyze leadership cases and their group's assessment results, develop practical collaboration and conflict-resolution strategies, and construct a personal leadership plan with measurable goals and reflective evaluation.</x:v>
+      </x:c>
+      <x:c r="F133" t="str">
+        <x:v>Leadership studies; Organizational psychology</x:v>
+      </x:c>
+      <x:c r="G133" t="str">
+        <x:v>Transformational leadership; Authentic leadership; Adaptive and evolutionary perspectives on leadership; Covey's seven habits; Personal vision and values; Emotional intelligence; Personality and group dynamics; Goal-setting and prioritization; Conflict resolution and negotiation; Leading change and innovation</x:v>
+      </x:c>
+      <x:c r="H133" t="str">
+        <x:v>Leadership case analysis; Personality and emotional-intelligence self-assessment; Analysis of group assessment profiles; Reflective analysis; SMART goal-setting; Leadership simulations and negotiation role-play</x:v>
+      </x:c>
+      <x:c r="I133" t="str">
+        <x:v>BENLEAD111.pdf</x:v>
+      </x:c>
+      <x:c r="J133" t="str">
+        <x:v>79270c1b9cffd256d607db7a0f767ecc27804e884f34ef7389fb88bcf8c0bcea</x:v>
+      </x:c>
+      <x:c r="K133"/>
+      <x:c r="L133" t="str">
+        <x:v>Named personality and emotional-intelligence instruments are examples; the outline leaves the final approved tools to class instructions. The personal leadership plan is an ungraded developmental activity.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>BENLEAD311</x:v>
+      </x:c>
+      <x:c r="C134" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>The Psychology of Organisations, Management and Leadership</x:v>
+      </x:c>
+      <x:c r="E134" t="str">
+        <x:v>Examines organizational behaviour at individual, group and organizational levels. Personality, perception, motivation and workplace emotions connect to teamwork, leadership, power, negotiation, organizational structure, culture and change. Students apply research to organizational cases, propose a study with appropriate measures and ethical safeguards, and conduct a brief systematic literature review using PRISMA to develop transparent search, screening and synthesis procedures.</x:v>
+      </x:c>
+      <x:c r="F134" t="str">
+        <x:v>Organizational psychology; Organizational behaviour; Management; Leadership studies</x:v>
+      </x:c>
+      <x:c r="G134" t="str">
+        <x:v>Diversity and inclusion; Organizational structure; Workplace emotions, stress and health; Personality and individual differences; Perception and decision-making; Motivation; Group behaviour and work teams; Human resource practices; Communication; Conflict and negotiation; Leadership; Power and organizational politics; Job attitudes; Organizational culture and change</x:v>
+      </x:c>
+      <x:c r="H134" t="str">
+        <x:v>Research-informed organizational case analysis; Research design and operationalization; Demonstration of data-collection procedures; Systematic literature review; PRISMA search and screening documentation; Critical synthesis of research findings</x:v>
+      </x:c>
+      <x:c r="I134" t="str">
+        <x:v>BENLEAD311.pdf</x:v>
+      </x:c>
+      <x:c r="J134" t="str">
+        <x:v>f0abb4007547267ac6ce785c7b7f98d4da0c8d403414e27dcc86c40178575f4f</x:v>
+      </x:c>
+      <x:c r="K134"/>
+      <x:c r="L134" t="str">
+        <x:v>The research case assignment develops and demonstrates a research plan; it does not establish that students complete a full empirical study. PRISMA use supports a systematic review, not necessarily a quantitative meta-analysis.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>DISCOMP211</x:v>
+      </x:c>
+      <x:c r="C135" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>Networks and Operating Systems</x:v>
+      </x:c>
+      <x:c r="E135" t="str">
+        <x:v>Studies computer networks and operating systems as the infrastructure for communication and resource management. Internet protocols are examined through the application, transport, network and link layers. Operating-system study covers processes, threads, scheduling, concurrency, memory and persistent storage. Wireshark laboratories and investigative projects connect these concepts to observed packet behaviour, network properties and experimental examination of operating-system performance.</x:v>
+      </x:c>
+      <x:c r="F135" t="str">
+        <x:v>Computer science; Computer networking; Operating systems</x:v>
+      </x:c>
+      <x:c r="G135" t="str">
+        <x:v>Internet architecture; HTTP and DNS; UDP and TCP; IPv4 and IPv6; Network address translation; Network data and control planes; Ethernet and ARP; Processes and threads; CPU scheduling; Virtualization; Synchronization and deadlocks; Memory management; Storage and file systems</x:v>
+      </x:c>
+      <x:c r="H135" t="str">
+        <x:v>Network packet capture and analysis with Wireshark; Experimental investigation of network and operating-system behaviour; Hypothesis-based performance testing; Sensitivity analysis</x:v>
+      </x:c>
+      <x:c r="I135" t="str">
+        <x:v>DISCOMP211.pdf</x:v>
+      </x:c>
+      <x:c r="J135" t="str">
+        <x:v>3f55b5abce187a4f881dd0a5adbcbd1ad36b7ad53b79827dfe315d6f6d170bc6</x:v>
+      </x:c>
+      <x:c r="K135"/>
+      <x:c r="L135" t="str">
+        <x:v>Sensitivity analysis is specified as the highest project-performance level rather than a universal minimum requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>DISCOMP311</x:v>
+      </x:c>
+      <x:c r="C136" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>Algorithms and Data Structures</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>Develops algorithm design and analysis with particular attention to experimental performance. Students study asymptotic complexity, random-number generation, sorting, string algorithms and graph algorithms, including traversal, shortest paths and spanning trees. Laboratories and investigative projects require tracing algorithms, examining their associated data structures in software, and measuring performance; stronger projects also test improvements to the code.</x:v>
+      </x:c>
+      <x:c r="F136" t="str">
+        <x:v>Computer science; Algorithms and computational complexity</x:v>
+      </x:c>
+      <x:c r="G136" t="str">
+        <x:v>Algorithm design; Data structures; Maximum contiguous subsequence sum; Asymptotic time complexity; Random-number generation; Sorting and searching; String algorithms; Graph traversal; Breadth-first and depth-first search; Shortest paths; Minimum spanning trees; Topological sorting; Computational complexity</x:v>
+      </x:c>
+      <x:c r="H136" t="str">
+        <x:v>Asymptotic complexity analysis; Algorithm tracing; Experimental algorithm benchmarking; Investigation of software algorithms and data structures; Code optimization experiments</x:v>
+      </x:c>
+      <x:c r="I136" t="str">
+        <x:v>DISCOMP311.pdf</x:v>
+      </x:c>
+      <x:c r="J136" t="str">
+        <x:v>923d64ac6cf58d93516a005d26ceef0a39aceda609cf90e5bae0703d3c22f25b</x:v>
+      </x:c>
+      <x:c r="K136"/>
+      <x:c r="L136" t="str">
+        <x:v>Code-improvement experiments are an advanced project criterion; they are not required at every passing level.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>DISDATA111</x:v>
+      </x:c>
+      <x:c r="C137" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>Introduction to Data Science</x:v>
+      </x:c>
+      <x:c r="E137" t="str">
+        <x:v>Introduces data visualization, exploration and manipulation in R using tabular, textual and spatial data. Students learn the grammar of graphics, tidy-data principles, data import and joins, web scraping and functions. A group project integrates education expenditure and test-performance data, while an individual project answers a chosen research question through data preparation, analysis and informative visualization.</x:v>
+      </x:c>
+      <x:c r="F137" t="str">
+        <x:v>Data science; Data visualization</x:v>
+      </x:c>
+      <x:c r="G137" t="str">
+        <x:v>Grammar of graphics; Exploratory data analysis; Tidy data; Data transformation and integration; Data import; Relational joins; Dates and times; Web data; Functions; Text data; Geospatial data; Visualization design and interpretation</x:v>
+      </x:c>
+      <x:c r="H137" t="str">
+        <x:v>R programming with tidyverse; ggplot data visualization; Data cleaning and reshaping; Data joins; Web scraping; Text-data analysis; Geospatial data analysis; Exploratory research using existing datasets</x:v>
+      </x:c>
+      <x:c r="I137" t="str">
+        <x:v>DISDATA111.pdf</x:v>
+      </x:c>
+      <x:c r="J137" t="str">
+        <x:v>97cc4b6fd4327d83195f280b19c6e438ef8da845f1759c3b0fce0d3cd10a5391</x:v>
+      </x:c>
+      <x:c r="K137"/>
+      <x:c r="L137" t="str">
+        <x:v>The education-spending project is an application of data integration and visualization; it does not establish training in causal evaluation of education expenditure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B138" t="str">
+        <x:v>DISDATA211</x:v>
+      </x:c>
+      <x:c r="C138" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D138" t="str">
+        <x:v>Machine Learning</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>Introduces statistical learning for understanding data and predicting outcomes. Regression and classification lead into model assessment, resampling, regularization, nonlinear models, trees and support vector machines, followed by principal components and clustering. Students apply methods in R or Python, engineer predictors to improve linear-model performance, and undertake an independent prediction project that justifies model choices and evaluates results.</x:v>
+      </x:c>
+      <x:c r="F138" t="str">
+        <x:v>Data science; Machine learning; Statistics</x:v>
+      </x:c>
+      <x:c r="G138" t="str">
+        <x:v>Prediction and model accuracy; Linear regression; Logistic regression; Generative classification models; Classification performance; Cross-validation; Bootstrap; Subset selection; Shrinkage; High-dimensional data; Basis functions and splines; Generalized additive models; Decision trees; Support vector machines; Principal component analysis; Clustering; Feature engineering</x:v>
+      </x:c>
+      <x:c r="H138" t="str">
+        <x:v>Statistical modelling in R or Python; Linear and logistic regression; Cross-validation and bootstrap resampling; Ridge and LASSO regression; Spline and generalized additive modelling; Tree-based prediction; Support vector classification; Principal component analysis; Cluster analysis; Out-of-sample model evaluation</x:v>
+      </x:c>
+      <x:c r="I138" t="str">
+        <x:v>DISDATA211.pdf</x:v>
+      </x:c>
+      <x:c r="J138" t="str">
+        <x:v>b33f70fab99c19c025c12c69c831e525e2dabccba02d55f1c26c0f2eb4f6a34c</x:v>
+      </x:c>
+      <x:c r="K138"/>
+      <x:c r="L138" t="str">
+        <x:v>Independent prediction-project subjects are chosen by students; example datasets do not define common substantive course coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B139" t="str">
+        <x:v>DISDATA212</x:v>
+      </x:c>
+      <x:c r="C139" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D139" t="str">
+        <x:v>Image Processing and Computer Vision</x:v>
+      </x:c>
+      <x:c r="E139" t="str">
+        <x:v>Examines how digital images are represented, processed and interpreted to recognize structures and objects. Spatial and spectral representations, colour and image statistics support filtering, segmentation, curve and feature detection, tracking and object classification. Students use Python and OpenCV to implement image-processing techniques, investigate spectral representations, and build a recognition pipeline whose performance is benchmarked on previously unseen images.</x:v>
+      </x:c>
+      <x:c r="F139" t="str">
+        <x:v>Computer science; Computer vision; Digital image processing</x:v>
+      </x:c>
+      <x:c r="G139" t="str">
+        <x:v>Spatial and spectral image representations; Cameras and calibration; Colour models and quantization; Image histograms; Point operators; Linear and nonlinear filters; Edges and contours; Mathematical morphology; Image segmentation; Curve and corner detection; Feature detection and tracking; Object localization and classification; Recognition performance</x:v>
+      </x:c>
+      <x:c r="H139" t="str">
+        <x:v>Python and OpenCV programming; Image filtering; Histogram and point transformations; Morphological image processing; Hough transform; Image segmentation; Feature matching and tracking; Recognition-pipeline design; Benchmark evaluation on unseen images</x:v>
+      </x:c>
+      <x:c r="I139" t="str">
+        <x:v>DISDATA212.pdf</x:v>
+      </x:c>
+      <x:c r="J139" t="str">
+        <x:v>38b709f7287deb34d108867ea78b8b82b710a3e064bf8905a6376ead7f272633</x:v>
+      </x:c>
+      <x:c r="K139"/>
+      <x:c r="L139" t="str">
+        <x:v>Medical imaging and remote sensing are motivating application domains; the outline does not specify dedicated practical projects in either field.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B140" t="str">
+        <x:v>DISGATE101</x:v>
+      </x:c>
+      <x:c r="C140" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D140" t="str">
+        <x:v>Introduction to Programming</x:v>
+      </x:c>
+      <x:c r="E140" t="str">
+        <x:v>Introduces computational problem-solving through Python programming. Structured programming, functions and standard data structures lead into recursion, testing, debugging, exceptions and object-oriented design. Discrete-mathematical ideas accompany computational techniques such as guess-and-check and bisection. Students write, trace, explain and debug programs in regular exercises and two larger programming projects.</x:v>
+      </x:c>
+      <x:c r="F140" t="str">
+        <x:v>Computer science; Computer programming; Discrete mathematics</x:v>
+      </x:c>
+      <x:c r="G140" t="str">
+        <x:v>Strings and input/output; Branching and iteration; Binary numbers and floating-point approximation; Functions and recursion; Tuples, lists and dictionaries; Mutability and aliasing; Testing and debugging; Exceptions and assertions; Classes and inheritance; Regular expressions; Logic, sets and enumeration</x:v>
+      </x:c>
+      <x:c r="H140" t="str">
+        <x:v>Python programming; Structured and object-oriented program design; Code tracing; Software testing and debugging; Guess-and-check algorithms; Bisection search</x:v>
+      </x:c>
+      <x:c r="I140" t="str">
+        <x:v>DISGATE101.pdf</x:v>
+      </x:c>
+      <x:c r="J140" t="str">
+        <x:v>af757507863ade8967cd8159e6ddb25d5454aae7c78eda0ffb4cb39cfee5a7e5</x:v>
+      </x:c>
+      <x:c r="K140" t="str">
+        <x:v>The outline prints DISGATEI01, with a letter I, whereas the authoritative filename is DISGATE101.</x:v>
+      </x:c>
+      <x:c r="L140"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B141" t="str">
+        <x:v>DISGATE102</x:v>
+      </x:c>
+      <x:c r="C141" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>Calculus</x:v>
+      </x:c>
+      <x:c r="E141" t="str">
+        <x:v>Develops single-variable calculus and related mathematical tools for modelling scientific problems. Functions, limits and differentiation lead to optimization, Taylor series, complex numbers, integration and differential equations. Students solve problems analytically and with Mathematica, including numerical approximation. A project implements, analyzes and adapts a dynamic model, requiring interpretation of its behaviour and explanation of the computational results.</x:v>
+      </x:c>
+      <x:c r="F141" t="str">
+        <x:v>Mathematics; Calculus; Applied mathematics</x:v>
+      </x:c>
+      <x:c r="G141" t="str">
+        <x:v>Functions and limits; Continuity; Differentiation; Optimization; Taylor series; Complex numbers; Definite and indefinite integrals; Integration techniques; First-order differential equations; Population-growth and predator–prey models; Second-order linear differential equations; Dynamic models</x:v>
+      </x:c>
+      <x:c r="H141" t="str">
+        <x:v>Analytical differentiation and integration; Taylor approximation; Newton's method; Numerical integration; Euler's method; Analytical solution of differential equations; Computer algebra with Mathematica; Dynamic-model implementation and analysis</x:v>
+      </x:c>
+      <x:c r="I141" t="str">
+        <x:v>DISGATE102.pdf</x:v>
+      </x:c>
+      <x:c r="J141" t="str">
+        <x:v>9e44f5e73bd069fc73ad9c907d6e56693b87734d73cee092c33ffa14f45bac23</x:v>
+      </x:c>
+      <x:c r="K141"/>
+      <x:c r="L141"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B142" t="str">
+        <x:v>DISMATH211</x:v>
+      </x:c>
+      <x:c r="C142" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D142" t="str">
+        <x:v>Linear Algebra</x:v>
+      </x:c>
+      <x:c r="E142" t="str">
+        <x:v>Studies systems of linear equations, matrices and vector spaces, connecting algebraic structure to geometry and applications. Linear transformations, determinants, bases, eigenvalues and orthogonality support least-squares approximation, quadratic forms and singular value decomposition. Mathematica assignments apply the theory to computer graphics, dynamical systems, least-squares fitting and principal component analysis, alongside analytical solution of linear-algebra problems.</x:v>
+      </x:c>
+      <x:c r="F142" t="str">
+        <x:v>Mathematics; Linear algebra; Applied mathematics</x:v>
+      </x:c>
+      <x:c r="G142" t="str">
+        <x:v>Linear systems; Matrix algebra and invertibility; Determinants; Linear independence; Vector spaces and bases; Linear transformations; Eigenvalues and diagonalization; Difference equations and Markov chains; Inner products and orthogonality; Least squares; Symmetric matrices and quadratic forms; Constrained optimization; Singular value decomposition; Principal component analysis</x:v>
+      </x:c>
+      <x:c r="H142" t="str">
+        <x:v>Row reduction; Matrix factorization; Change of basis; Eigenvalue analysis; Gram–Schmidt orthogonalization; Orthogonal projection and least-squares fitting; Singular value decomposition; Principal component analysis; Computer algebra with Mathematica</x:v>
+      </x:c>
+      <x:c r="I142" t="str">
+        <x:v>DISMATH211.pdf</x:v>
+      </x:c>
+      <x:c r="J142" t="str">
+        <x:v>06f1513f4ad882b539af494a3deff34af584cd318d6b1f52ad05ce671b509bae</x:v>
+      </x:c>
+      <x:c r="K142"/>
+      <x:c r="L142"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>DISMATH212</x:v>
+      </x:c>
+      <x:c r="C143" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D143" t="str">
+        <x:v>Quantum Mechanics</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>Introduces quantum mechanics through Stern–Gerlach experiments, spin systems and the postulates of measurement. Wave functions and the Schrödinger equation lead to bound and scattering states, angular momentum, atomic structure and the harmonic oscillator. Perturbation and variational methods extend the analysis to approximate solutions and identical particles. A Mathematica project numerically determines bound states for a one-dimensional potential and evaluates the results.</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>Physics; Quantum mechanics</x:v>
+      </x:c>
+      <x:c r="G143" t="str">
+        <x:v>Spin and quantum measurement; State vectors and operators; Uncertainty principle; Wave functions and Schrödinger equation; Potential wells; Tunnelling and scattering; Angular momentum; Hydrogen atom; Harmonic oscillator; Perturbation theory; Variational principle; Identical particles and Pauli exclusion; Atomic and molecular structure; EPR paradox and Bell inequalities</x:v>
+      </x:c>
+      <x:c r="H143" t="str">
+        <x:v>State-vector and operator calculations; Eigenvalue analysis; Analytical solution of the Schrödinger equation; Perturbation approximation; Variational approximation; Numerical bound-state computation with Mathematica</x:v>
+      </x:c>
+      <x:c r="I143" t="str">
+        <x:v>DISMATH212.pdf</x:v>
+      </x:c>
+      <x:c r="J143" t="str">
+        <x:v>b9312562e9b7245bfb01bf142a707742c1829bd4201f75cde201d215997e45ac</x:v>
+      </x:c>
+      <x:c r="K143"/>
+      <x:c r="L143" t="str">
+        <x:v>Quantum spookiness is scheduled as a possible extra topic; the description also mentions quantum computing briefly without specifying substantive training in it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>DISMATH311</x:v>
+      </x:c>
+      <x:c r="C144" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D144" t="str">
+        <x:v>Abstract Algebra</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>Introduces axiomatic algebraic structures through a sustained study of groups, followed by symmetric groups, rings and fields. Students analyze homomorphisms, quotient structures, polynomial rings and field extensions, developing and adapting mathematical proofs throughout. A project applies the fundamental theorem of finite abelian groups to decompose a chosen group, using Mathematica and presenting the verified argument in a mathematical paper.</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>Mathematics; Abstract algebra; Group theory</x:v>
+      </x:c>
+      <x:c r="G144" t="str">
+        <x:v>Sets and mappings; Integer arithmetic; Mathematical induction; Groups and subgroups; Lagrange's theorem; Homomorphisms and normal subgroups; Quotient groups; Finite abelian groups; Cauchy and Sylow theorems; Symmetric and alternating groups; Rings, ideals and quotient rings; Polynomial rings and irreducibility; Fields and field extensions; Constructibility and splitting fields</x:v>
+      </x:c>
+      <x:c r="H144" t="str">
+        <x:v>Axiomatic mathematical reasoning; Proof construction and mathematical induction; Analysis of algebraic homomorphisms and quotient structures; Decomposition of finite abelian groups; Computer algebra with Mathematica</x:v>
+      </x:c>
+      <x:c r="I144" t="str">
+        <x:v>DISMATH311.pdf</x:v>
+      </x:c>
+      <x:c r="J144" t="str">
+        <x:v>cebbbef82b814ff8fcbfbd9b5baaa662a7498bf6f4629a3edf5cc1eabdf67648</x:v>
+      </x:c>
+      <x:c r="K144"/>
+      <x:c r="L144"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>ENSDELT111</x:v>
+      </x:c>
+      <x:c r="C145" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D145" t="str">
+        <x:v>Building with Nature</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>Examines how infrastructure and environmental planning can work with natural processes while supporting human needs and ecosystem health. Nature-based approaches are compared across sandy and muddy coasts, lakes, rivers, estuaries, cities and ports. Zeeland and Walcheren provide a regional setting for water-management history and coastal adaptation. Habitat connectivity, ecoducts and fish ladders extend the discussion to a group connectivity project.</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>Environmental science; Ecological engineering; Water management</x:v>
+      </x:c>
+      <x:c r="G145" t="str">
+        <x:v>Nature-based infrastructure; Coastal protection; Sandy and muddy coasts; Mangrove rehabilitation; Lowland lakes; River and estuary restoration; Delta cities; Habitat opportunities in ports; Walcheren water-management history; Ecosystem health; Habitat connectivity; Ecoducts and fish ladders</x:v>
+      </x:c>
+      <x:c r="H145"/>
+      <x:c r="I145" t="str">
+        <x:v>ENSDELT111.docx</x:v>
+      </x:c>
+      <x:c r="J145" t="str">
+        <x:v>859556b80e85b2489c0166fa739775251fd2eedabfa6d6d4248b6c2d37942942</x:v>
+      </x:c>
+      <x:c r="K145"/>
+      <x:c r="L145" t="str">
+        <x:v>The outline assigns a connectivity project and mentions fieldwork, but does not describe specific research, design or field-measurement procedures. Several later-session subjects remain unspecified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B146" t="str">
+        <x:v>ENSECOL111</x:v>
+      </x:c>
+      <x:c r="C146" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D146" t="str">
+        <x:v>The Living Planet: An Introduction to Biodiversity</x:v>
+      </x:c>
+      <x:c r="E146" t="str">
+        <x:v>Surveys biological diversity and phylogenetic relationships across the tree of life, from bacteria and archaea to protists, fungi, plants and animals. The course connects organismal diversity to ecosystem health and human concerns including food, climate, land use and well-being. Students identify organisms, measure biodiversity, and undertake a small research project with literature review, data collection, analysis and a research poster.</x:v>
+      </x:c>
+      <x:c r="F146" t="str">
+        <x:v>Biology; Biodiversity science; Ecology; Biological systematics</x:v>
+      </x:c>
+      <x:c r="G146" t="str">
+        <x:v>Tree of life and phylogeny; Viruses; Bacteria and archaea; Protists; Fungi; Seedless and seed plants; Invertebrates; Vertebrates and human diversity; Biodiversity measurement; Ecosystem health; Biodiversity and food security; Biodiversity and climate; Biodiversity and human well-being</x:v>
+      </x:c>
+      <x:c r="H146" t="str">
+        <x:v>Organism identification using identification apps; Rank-abundance diagrams; Species saturation curves; Biodiversity indices; Scientific literature searching; Small-scale empirical research with data collection and analysis</x:v>
+      </x:c>
+      <x:c r="I146" t="str">
+        <x:v>ENSECOL111.docx</x:v>
+      </x:c>
+      <x:c r="J146" t="str">
+        <x:v>2968dc7a6e96672770e4613484dad9fff052a99e47ad751ced8644f525097572</x:v>
+      </x:c>
+      <x:c r="K146"/>
+      <x:c r="L146" t="str">
+        <x:v>The small research project's particular subject and detailed protocol are supplied separately.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="A147" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B147" t="str">
+        <x:v>ENSECOL211</x:v>
+      </x:c>
+      <x:c r="C147" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D147" t="str">
+        <x:v>From Origins to Diversity: The Science of Evolution</x:v>
+      </x:c>
+      <x:c r="E147" t="str">
+        <x:v>Examines evolutionary theory from genes and populations to species diversification and the history of life. Genetics, natural selection, drift and adaptation underpin study of sexual reproduction, speciation, phylogeny and biogeography. Genomics, development, coevolution, radiation and extinction broaden the account across biological scales. Students use scientific literature to investigate and present the evolutionary history of a selected species.</x:v>
+      </x:c>
+      <x:c r="F147" t="str">
+        <x:v>Evolutionary biology; Population genetics; Phylogenetics</x:v>
+      </x:c>
+      <x:c r="G147" t="str">
+        <x:v>History and evidence of evolution; Molecular and Mendelian genetics; Natural selection and variation; Genetic drift; Molecular evolution; Multilocus and quantitative genetics; Adaptation and units of selection; Sexual reproduction; Species concepts and speciation; Phylogeny and classification; Evolutionary biogeography; Evolutionary genomics; Evolutionary developmental biology; Coevolution; Radiation and extinction</x:v>
+      </x:c>
+      <x:c r="H147" t="str">
+        <x:v>Literature-based reconstruction of a species' evolutionary history</x:v>
+      </x:c>
+      <x:c r="I147" t="str">
+        <x:v>ENSECOL211.docx</x:v>
+      </x:c>
+      <x:c r="J147" t="str">
+        <x:v>c115313aa536377b01d62b706dbea8c29725b972c40dbc82fbaa60ad03570ae0</x:v>
+      </x:c>
+      <x:c r="K147"/>
+      <x:c r="L147" t="str">
+        <x:v>The outline does not specify laboratory or computational protocols for evolutionary research; the assessed project investigates a species' evolutionary history.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B148" t="str">
+        <x:v>ENSECOL311</x:v>
+      </x:c>
+      <x:c r="C148" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D148" t="str">
+        <x:v>Marine Biology</x:v>
+      </x:c>
+      <x:c r="E148" t="str">
+        <x:v>Examines marine ecological processes, contrasting major ocean and coastal ecosystems and their responses to human activities. Physical and chemical oceanography support study of primary and secondary production, microbial ecology and habitats from estuaries and shores to deep seas, reefs and polar regions. Fisheries, aquaculture, acidification, sea-level rise and plastic pollution connect ecological knowledge to conservation and public communication through seminars and a multimedia outreach project.</x:v>
+      </x:c>
+      <x:c r="F148" t="str">
+        <x:v>Marine biology; Marine ecology; Oceanography</x:v>
+      </x:c>
+      <x:c r="G148" t="str">
+        <x:v>Physical and chemical oceanography; Marine primary and secondary production; Microbial ecology; Respiration and decomposition; Estuaries; Rocky and sandy shores; Pelagic ecosystems; Continental shelves and deep sea; Mangroves and seagrass; Coral reefs; Polar ecosystems; Fisheries and aquaculture; Ocean acidification; Sea-level rise; Marine plastic pollution; Marine conservation</x:v>
+      </x:c>
+      <x:c r="H148"/>
+      <x:c r="I148" t="str">
+        <x:v>ENSECOL311.pdf</x:v>
+      </x:c>
+      <x:c r="J148" t="str">
+        <x:v>7564a94542a0034103a02248038c30a493d14e8dac5dc99b4555d7e0ab23118e</x:v>
+      </x:c>
+      <x:c r="K148"/>
+      <x:c r="L148" t="str">
+        <x:v>The outline mentions possible fieldwork, laboratory visits and practicals subject to arrangements, but specifies no particular sampling or analytical techniques. The outreach project's medium is chosen by students.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B149" t="str">
+        <x:v>ENSENVI111</x:v>
+      </x:c>
+      <x:c r="C149" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D149" t="str">
+        <x:v>Dynamic Earth</x:v>
+      </x:c>
+      <x:c r="E149" t="str">
+        <x:v>Introduces Earth's surface and interior as interacting geological systems. Mineral and rock formation, deformation, stratigraphy and coastal processes connect to plate tectonics, seismicity, mantle and core structure, gravity, magnetism and heat flow. Practical work and Ardennes fieldwork develop observation and geological reconstruction: students identify materials, collect structural measurements, construct a cross-section and stratigraphic column, and explain the area's geological history.</x:v>
+      </x:c>
+      <x:c r="F149" t="str">
+        <x:v>Earth science; Geology; Geophysics</x:v>
+      </x:c>
+      <x:c r="G149" t="str">
+        <x:v>Earth formation and composition; Minerals and crystallization; Igneous, sedimentary and metamorphic rocks; Plate tectonics and Wilson cycle; Rock deformation; Stratigraphy; Coastal sedimentation, waves and currents; Seismic hazards; Seismic tomography; Mantle and core structure; Gravity and isostasy; Geomagnetism; Terrestrial heat flow; Climate–tectonic interactions</x:v>
+      </x:c>
+      <x:c r="H149" t="str">
+        <x:v>Mineral and rock identification; Geological field observation and structural measurement; Topographic and geological profiling; Stratigraphic-column construction; Geological-history reconstruction; Sand and coastal-feature analysis; Evaluation of geoscientific source evidence</x:v>
+      </x:c>
+      <x:c r="I149" t="str">
+        <x:v>ENSENVI111.pdf</x:v>
+      </x:c>
+      <x:c r="J149" t="str">
+        <x:v>8b32d33a43c4a992a3ae9b698df90125f746dcedf793a5a356da7a5a17ea6bf8</x:v>
+      </x:c>
+      <x:c r="K149" t="str">
+        <x:v>The cover prints ENVSCI111 and some instructions retain SCIEART101; the authoritative filename code is ENSENVI111.</x:v>
+      </x:c>
+      <x:c r="L149" t="str">
+        <x:v>SEM–EDS appears in the sand-analysis schedule, but the outline does not establish hands-on instrument training, so that technique is not claimed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B150" t="str">
+        <x:v>ENSENVI311</x:v>
+      </x:c>
+      <x:c r="C150" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D150" t="str">
+        <x:v>Environmental Biogeochemistry</x:v>
+      </x:c>
+      <x:c r="E150" t="str">
+        <x:v>Studies near-surface biogeochemical processes through interactions among water, minerals, soils and biological activity. Aqueous chemistry, redox, precipitation and dissolution underpin analysis of estuarine mixing, ore formation, clays, adsorption and biomineralization. Students use geochemical modelling and laboratory data to investigate contaminant mobility, remediation, wastewater treatment and resource recovery, developing a case study that evaluates environmental processes and possible interventions.</x:v>
+      </x:c>
+      <x:c r="F150" t="str">
+        <x:v>Biogeochemistry; Geochemistry; Environmental chemistry; Geology</x:v>
+      </x:c>
+      <x:c r="G150" t="str">
+        <x:v>Mineral–water interactions; Water composition and ionic strength; Chemical equilibrium; Carbonate chemistry; Estuarine mixing and flocculation; Redox and chemical speciation; Ore formation; Rare earth elements; Mineral stability and dissolution; Clays and adsorption; Biomineralization; Bioremediation; Wastewater treatment; Resource recovery</x:v>
+      </x:c>
+      <x:c r="H150" t="str">
+        <x:v>Geochemical equilibrium and thermodynamic modelling with Geochemist's Workbench and Visual MINTEQ; Electrolyte calculations; Piper and ternary diagrams; Pourbaix-diagram construction; Ore-grade determination; Adsorption practicals; Quantitative environmental case analysis</x:v>
+      </x:c>
+      <x:c r="I150" t="str">
+        <x:v>ENSENVI311.pdf</x:v>
+      </x:c>
+      <x:c r="J150" t="str">
+        <x:v>da943985fcfb0e41bdfc298f0e19e3c2559f38f2461bcfa9c65d059cc998b315</x:v>
+      </x:c>
+      <x:c r="K150" t="str">
+        <x:v>The cover identifies Environmental Biogeochemistry as ENSENVI111, whereas the filename and the body identify the advanced course as ENSENVI311.</x:v>
+      </x:c>
+      <x:c r="L150" t="str">
+        <x:v>The case-study subject and some assignment details are not fixed in the outline; modelling and practical work are described explicitly.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B151" t="str">
+        <x:v>ENSGATE101</x:v>
+      </x:c>
+      <x:c r="C151" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D151" t="str">
+        <x:v>Sustainability Essentials</x:v>
+      </x:c>
+      <x:c r="E151" t="str">
+        <x:v>Introduces sustainability through planetary boundaries and the mathematical and natural-science tools used to understand environmental change. Exponential growth and dynamic models connect to resilience, climate and heat exchange, ocean acidification, nutrient cycles and material behaviour. Students interpret graphs, solve simple differential equations and apply introductory chemistry and physics, then propose a response to a local sustainability problem within the planetary-boundaries framework.</x:v>
+      </x:c>
+      <x:c r="F151" t="str">
+        <x:v>Environmental science; Sustainability science; Applied mathematics; Physics; Chemistry</x:v>
+      </x:c>
+      <x:c r="G151" t="str">
+        <x:v>Planetary boundaries; Anthropocene and Great Acceleration; Exponential growth; Dynamic systems and resilience; Climate change; Energy, entropy and heat exchange; Ocean acidification; Chemical bonding and material structure; Nutrient cycles; Ozone depletion; Newtonian mechanics; Stress and strain; Wave propagation; Land-use change</x:v>
+      </x:c>
+      <x:c r="H151" t="str">
+        <x:v>Graph interpretation; Fermi estimation; Elementary differential-equation modelling; Logistic and Lotka–Volterra models; Basic chemical and thermodynamic analysis; Trigonometric wave modelling; Local sustainability problem analysis</x:v>
+      </x:c>
+      <x:c r="I151" t="str">
+        <x:v>ENSGATE101.pdf</x:v>
+      </x:c>
+      <x:c r="J151" t="str">
+        <x:v>9a9919a2fb0a476de8c86dd1049607d90dec7fef032dd8a7f6ddc5d40b87fa39</x:v>
+      </x:c>
+      <x:c r="K151" t="str">
+        <x:v>The cover, general-information code and running headers print ENSDELT101, while the course description and authoritative filename identify ENSGATE101. The learning outcomes name nitrogen and phosphorus cycles, while the scheduled nutrient-cycle lecture names sulfur and selenium.</x:v>
+      </x:c>
+      <x:c r="L151" t="str">
+        <x:v>The record retains the broader supported category of nutrient cycles. Some later coverage is provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="A152" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B152" t="str">
+        <x:v>ENSSUST111</x:v>
+      </x:c>
+      <x:c r="C152" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D152" t="str">
+        <x:v>Climate Change</x:v>
+      </x:c>
+      <x:c r="E152" t="str">
+        <x:v>Examines anthropogenic climate change through its physical drivers, ecological impacts and societal consequences. Greenhouse gases, feedbacks, sea-level rise and ocean acidification lead into agriculture, infrastructure, health, justice and governance. Mitigation and adaptation options include renewable energy, carbon removal and geoengineering. Students assess information sources, interview a stakeholder, communicate solutions through film and an infographic, and reflect on climate responsibility and justice.</x:v>
+      </x:c>
+      <x:c r="F152" t="str">
+        <x:v>Climate science; Environmental science; Sustainability studies; Environmental governance</x:v>
+      </x:c>
+      <x:c r="G152" t="str">
+        <x:v>Greenhouse gases; Climate feedbacks and tipping points; Ocean acidification; Sea-level rise; Biosphere impacts; Agriculture and food production; Climate and health; Transport and construction; Climate justice; Paris Agreement; Renewable energy; Carbon capture and sequestration; Geoengineering; Climate communication and misinformation; Climate anxiety; Mitigation and adaptation</x:v>
+      </x:c>
+      <x:c r="H152" t="str">
+        <x:v>Critical evaluation of climate-information sources; Stakeholder interviewing; Synthesis of climate-solution evidence; Structured reflection using What? So What? Now What?</x:v>
+      </x:c>
+      <x:c r="I152" t="str">
+        <x:v>ENSSUST111.pdf</x:v>
+      </x:c>
+      <x:c r="J152" t="str">
+        <x:v>39a65a91b186f1314dadfcab2aca2b527b632658f10fe179be351e0e6529c45c</x:v>
+      </x:c>
+      <x:c r="K152"/>
+      <x:c r="L152" t="str">
+        <x:v>Excursions introduce energy technologies but do not establish hands-on technical training in them.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="A153" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B153" t="str">
+        <x:v>ENSSUST112</x:v>
+      </x:c>
+      <x:c r="C153" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D153" t="str">
+        <x:v>Life Cycle Analysis &amp; Circular Economy</x:v>
+      </x:c>
+      <x:c r="E153" t="str">
+        <x:v>Develops life-cycle approaches to evaluating products, processes and services within a circular economy. Students examine environmental, social and health consequences from resource extraction to disposal or reuse, together with costs, revenues and management strategies. Three preliminary projects develop different parts or forms of life-cycle analysis, followed by a project that integrates the stages into a full product or process assessment.</x:v>
+      </x:c>
+      <x:c r="F153" t="str">
+        <x:v>Sustainability science; Industrial ecology; Life-cycle engineering and management</x:v>
+      </x:c>
+      <x:c r="G153" t="str">
+        <x:v>Circular economy; Product and process life cycles; Resource extraction and reuse; Environmental impacts; Social and health consequences; Life-cycle management strategies; Product-based and process-based assessment; Costs and revenues; Sustainable product and process planning</x:v>
+      </x:c>
+      <x:c r="H153" t="str">
+        <x:v>Life-cycle assessment; Life-cycle management strategy analysis; Environmental-impact estimation; Cost and revenue analysis; Integrated product or process assessment</x:v>
+      </x:c>
+      <x:c r="I153" t="str">
+        <x:v>ENSSUST112.pdf</x:v>
+      </x:c>
+      <x:c r="J153" t="str">
+        <x:v>d7b773839476eeadf64b9827ff273a32f64f40d06a85a16cfa842b82b9ea42b3</x:v>
+      </x:c>
+      <x:c r="K153"/>
+      <x:c r="L153" t="str">
+        <x:v>Detailed project instructions and assessment procedures are in a separate course manual not supplied here; no particular software or impact-assessment standard is specified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="A154" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B154" t="str">
+        <x:v>ENSSUST211</x:v>
+      </x:c>
+      <x:c r="C154" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D154" t="str">
+        <x:v>Energy and Sustainability</x:v>
+      </x:c>
+      <x:c r="E154" t="str">
+        <x:v>Studies renewable-energy resources, conversion technologies and their integration into sustainable energy systems. Solar, wind, hydro, geothermal and biomass resources are evaluated through physical principles, resource availability and generation potential. Storage, electricity grids and demand management connect individual technologies to system reliability. Quantitative exercises, a Polysun workshop, short experiments and local mini-grid work develop the ability to assess energy options in practical environmental and economic contexts.</x:v>
+      </x:c>
+      <x:c r="F154" t="str">
+        <x:v>Energy engineering; Renewable-energy systems; Sustainability science; Applied physics</x:v>
+      </x:c>
+      <x:c r="G154" t="str">
+        <x:v>Energy demand and renewable resources; Solar radiation and energy yield; Solar thermal and photovoltaic generation; Wind energy; Hydropower; Geothermal energy; Biomass, biogas and biofuels; Electricity grids; Energy storage; Batteries and pumped storage; Smart grids and system integration; Demand management; Mini-grids; Energy-system environmental and economic constraints</x:v>
+      </x:c>
+      <x:c r="H154" t="str">
+        <x:v>Renewable-energy resource and yield calculations; Polysun energy-system modelling; Hydropower sizing; Laboratory experimentation on renewable-energy systems; Energy-storage comparison; Mini-grid analysis and design</x:v>
+      </x:c>
+      <x:c r="I154" t="str">
+        <x:v>ENSSUST211.pdf</x:v>
+      </x:c>
+      <x:c r="J154" t="str">
+        <x:v>ea7285b4aa17ac3329371aff6731d153bada01111735dadfdade1670de323a4e</x:v>
+      </x:c>
+      <x:c r="K154" t="str">
+        <x:v>The project is variously described as sustainable electricity for a new Zeeland factory, a Zeeland mini-grid, and an assignment called Monkey Island; the supplied outline does not reconcile these descriptions.</x:v>
+      </x:c>
+      <x:c r="L154" t="str">
+        <x:v>The record describes the shared energy-system focus without assigning a definite project site. Short laboratory topics can include solar, wind, hydrogen storage or an approved related subject.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="A155" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B155" t="str">
+        <x:v>ENSSUST212</x:v>
+      </x:c>
+      <x:c r="C155" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D155" t="str">
+        <x:v>Transport Phenomena</x:v>
+      </x:c>
+      <x:c r="E155" t="str">
+        <x:v>Studies transport of momentum, energy and matter through a common framework of conservation laws and balances. Viscosity, thermal conductivity and diffusivity connect fluid mechanics, heat transfer and mass transfer to applications across engineering and the sciences. Students combine conceptual reasoning, mathematical derivation and numerical calculation to solve transport problems, and synthesize research papers on an individually selected application.</x:v>
+      </x:c>
+      <x:c r="F155" t="str">
+        <x:v>Chemical engineering; Applied physics; Transport phenomena</x:v>
+      </x:c>
+      <x:c r="G155" t="str">
+        <x:v>Momentum transport; Fluid mechanics; Energy transport and heat transfer; Mass transfer; Conservation laws; Transport balances; Viscosity; Thermal conductivity; Diffusivity; Scientific and engineering applications of transport</x:v>
+      </x:c>
+      <x:c r="H155" t="str">
+        <x:v>Conservation-balance modelling; Mathematical derivation of transport relations; Numerical transport calculations; Critical synthesis of research literature</x:v>
+      </x:c>
+      <x:c r="I155" t="str">
+        <x:v>ENSSUST212.pdf</x:v>
+      </x:c>
+      <x:c r="J155" t="str">
+        <x:v>3aed71ca5e8112a044167b155e38b7967e1aa49bfd0ef148b1aa684a82122065</x:v>
+      </x:c>
+      <x:c r="K155" t="str">
+        <x:v>The body and running headers retain ENGENER201, whereas the cover and authoritative filename identify ENSSUST212.</x:v>
+      </x:c>
+      <x:c r="L155" t="str">
+        <x:v>The outline provides no detailed sequence of transport techniques beyond the conservation and balance framework. Literature-study applications are chosen by individual students.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="A156" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B156" t="str">
+        <x:v>ENSSUST312</x:v>
+      </x:c>
+      <x:c r="C156" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D156" t="str">
+        <x:v>Future Materials / Interfacial Engineering</x:v>
+      </x:c>
+      <x:c r="E156" t="str">
+        <x:v>Examines the physical and chemical principles governing colloidal and interfacial systems. Materials are treated as dispersed or heterogeneous structures whose interfaces influence behaviour, linking physical chemistry to mechanics, thermodynamics and rheology. Students apply conceptual reasoning, derivations and numerical calculations to material problems, then integrate research literature on a selected application or special topic in interfacial engineering.</x:v>
+      </x:c>
+      <x:c r="F156" t="str">
+        <x:v>Materials science; Interfacial engineering; Colloid science; Physical chemistry</x:v>
+      </x:c>
+      <x:c r="G156" t="str">
+        <x:v>Colloidal dispersions; Interfaces in heterogeneous materials; Particle and domain length scales; Physical chemistry of colloidal systems; Thermodynamic and mechanical behaviour; Rheology; Engineering applications of interfacial systems</x:v>
+      </x:c>
+      <x:c r="H156" t="str">
+        <x:v>Mathematical and numerical analysis of interfacial systems; Critical synthesis of research literature</x:v>
+      </x:c>
+      <x:c r="I156" t="str">
+        <x:v>ENSSUST312.pdf</x:v>
+      </x:c>
+      <x:c r="J156" t="str">
+        <x:v>986f97a02f242b839a51dfb1bf78e9a8fe21af15e4a264619929eee8a6048356</x:v>
+      </x:c>
+      <x:c r="K156" t="str">
+        <x:v>Running headers retain ENGMATE301, whereas the cover, body title and authoritative filename identify ENSSUST312.</x:v>
+      </x:c>
+      <x:c r="L156" t="str">
+        <x:v>The schedule follows the interfacial-engineering textbook without specifying its chapter coverage. Example material types and students' individually chosen literature topics do not establish that every application is studied by all students.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="A157" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B157" t="str">
+        <x:v>GOSGATE101</x:v>
+      </x:c>
+      <x:c r="C157" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D157" t="str">
+        <x:v>Thinking Across Disciplines</x:v>
+      </x:c>
+      <x:c r="E157" t="str">
+        <x:v>Introduces philosophy, history, sociology, law and political science through family, kinship and community. Students examine reasoning and bias, historical family representations, agency and social structures, legal regulation of relationships, and political ideologies and values. Disciplinary workshops develop argument analysis, historical source interpretation and legal case briefing. A political-science memo compares party positions with citizens' family and gender values using manifesto and survey data.</x:v>
+      </x:c>
+      <x:c r="F157" t="str">
+        <x:v>Philosophy; History; Sociology; Law; Political science</x:v>
+      </x:c>
+      <x:c r="G157" t="str">
+        <x:v>Family, kinship and community; Logic and argumentation; Heuristics and cognitive biases; Historical demography and family life; American family representations and marginalization; Sociological imagination; Agency and social structure; Culture, social relations and inequality; Family law and human rights; Political ideologies; Gender values; Political representation and vote choice</x:v>
+      </x:c>
+      <x:c r="H157" t="str">
+        <x:v>Logical argument analysis; Historical analysis of primary and cultural sources; Sociological analysis of research articles; Legal database research; IRAC case briefing; Analysis of Comparative Manifesto Project and World Values Survey data; Interdisciplinary comparison</x:v>
+      </x:c>
+      <x:c r="I157" t="str">
+        <x:v>GOSGATE101.pdf</x:v>
+      </x:c>
+      <x:c r="J157" t="str">
+        <x:v>a93d03f409ab7df2cc902c9dea123fc3a7dcb5a08095f1bd5ef0e225014aa9fb</x:v>
+      </x:c>
+      <x:c r="K157"/>
+      <x:c r="L157"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="A158" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B158" t="str">
+        <x:v>GOSGATE102</x:v>
+      </x:c>
+      <x:c r="C158" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D158" t="str">
+        <x:v>Law, Society and Justice</x:v>
+      </x:c>
+      <x:c r="E158" t="str">
+        <x:v>Introduces legal, social and normative perspectives on law. Students compare legal systems and study principal fields of public and private law before examining interpretation, justice, social control, social change, race and gender. Case-law research, IRAC briefs, mock trials and a demand letter develop legal reasoning and practice. A small socio-legal project analyzes an issue within the theme of identity and community.</x:v>
+      </x:c>
+      <x:c r="F158" t="str">
+        <x:v>Law; Socio-legal studies; Legal philosophy</x:v>
+      </x:c>
+      <x:c r="G158" t="str">
+        <x:v>Common and civil law traditions; Constitutional and administrative law; Public international law; Human rights; Criminal law; Property, contract and tort law; Family law; Legal interpretation; Justice; Law and social control; Law and social change; Race and gender in law; Identity and community</x:v>
+      </x:c>
+      <x:c r="H158" t="str">
+        <x:v>Legal research; Case-law analysis; IRAC case briefing; Legal interpretation; Mock-trial advocacy; Demand-letter drafting</x:v>
+      </x:c>
+      <x:c r="I158" t="str">
+        <x:v>GOSGATE102.pdf</x:v>
+      </x:c>
+      <x:c r="J158" t="str">
+        <x:v>27fff0336111137dea384830fbc7d257e4a3a96b5e3dd935248de48f4f8b5b9e</x:v>
+      </x:c>
+      <x:c r="K158"/>
+      <x:c r="L158" t="str">
+        <x:v>The research project requires legal, social and normative analysis; the outline does not prescribe a particular empirical data-collection technique.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
+        <x:v>GOSHIST111</x:v>
+      </x:c>
+      <x:c r="C159" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D159" t="str">
+        <x:v>Modern History</x:v>
+      </x:c>
+      <x:c r="E159" t="str">
+        <x:v>Surveys economic, political and cultural developments from 1815 to the contemporary world, emphasizing their relationship to shifts in international power. Industrialization, nationalism and revolution lead into imperialism, world wars, economic crisis, the Cold War and decolonization. Students examine competing historical interpretations and significant contemporary legacies, developing a focused research question, evaluating sources and presenting an evidence-based historical essay.</x:v>
+      </x:c>
+      <x:c r="F159" t="str">
+        <x:v>History; Modern history; Economic history; International history</x:v>
+      </x:c>
+      <x:c r="G159" t="str">
+        <x:v>Industrialization; Nineteenth-century political ideologies and revolutions; Nationalism and nation-state formation; European imperialism; First World War; Russian Revolution; Great Depression; Fascism and dictatorship; Second World War; Cold War; Welfare states; Decolonization; European integration; Collapse of Soviet communism; Contemporary global power</x:v>
+      </x:c>
+      <x:c r="H159" t="str">
+        <x:v>Critical analysis of historical scholarship; Evaluation and triangulation of historical sources; Historical research-question development; Evidence-based historical argumentation</x:v>
+      </x:c>
+      <x:c r="I159" t="str">
+        <x:v>GOSHIST111.docx</x:v>
+      </x:c>
+      <x:c r="J159" t="str">
+        <x:v>683245d4adb0f51da2eb632a9dba7d961631826e29ca59910a978859ba595d62</x:v>
+      </x:c>
+      <x:c r="K159"/>
+      <x:c r="L159"/>
+    </x:row>
+    <x:row r="160">
+      <x:c r="A160" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B160" t="str">
+        <x:v>GOSHIST112</x:v>
+      </x:c>
+      <x:c r="C160" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D160" t="str">
+        <x:v>Histories of Gender: Repression and Resistance</x:v>
+      </x:c>
+      <x:c r="E160" t="str">
+        <x:v>Studies gendered histories and lives in North America from the nineteenth century to the present, centering storytelling and intersectionality. Queer and heteronormative narratives connect slavery, family, sexuality, health, incarceration and contemporary backlash to resistance and activism. Students interpret primary sources and scholarship, interview older queer people, contribute to the Walking with Pride activist artwork, and conduct an original research project in a chosen format.</x:v>
+      </x:c>
+      <x:c r="F160" t="str">
+        <x:v>History; Gender studies; Queer studies; Carceral studies</x:v>
+      </x:c>
+      <x:c r="G160" t="str">
+        <x:v>Gender and intersectionality; Body sovereignty; Heteronormativity and compulsory heterosexuality; Homonationalism; Rainbow capitalism; Masculinity and sexuality; Queer ageing and memory; Slavery and racialized gender histories; Family and socialization; Health and pathologization; Media bias and book bans; Incarceration; Queer activism and resistance</x:v>
+      </x:c>
+      <x:c r="H160" t="str">
+        <x:v>Historical primary-source research; Intersectional analysis; Oral-history interviewing; Critical interpretation of memoir and cultural representations; Arts-based research; Community-engaged activist art; Reflective analysis</x:v>
+      </x:c>
+      <x:c r="I160" t="str">
+        <x:v>GOSHIST112.docx</x:v>
+      </x:c>
+      <x:c r="J160" t="str">
+        <x:v>8b7562bcd41abf666e0457e7370026680e60a7598b656d92d1298ca3a5976bfb</x:v>
+      </x:c>
+      <x:c r="K160"/>
+      <x:c r="L160" t="str">
+        <x:v>Learning outcomes mention additional children's-story, future-scenario and international collaboration activities that are not clearly matched to the assessment schedule. The record centers the explicitly assigned interview, artwork and original research.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B161" t="str">
+        <x:v>GOSHIST211</x:v>
+      </x:c>
+      <x:c r="C161" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D161" t="str">
+        <x:v>History of Empires</x:v>
+      </x:c>
+      <x:c r="E161" t="str">
+        <x:v>Compares empires from antiquity to contemporary great powers through theories of imperial rise, dominance and decline. Cases span Persian, Roman, Chinese and Mongol empires, European overseas powers and modern global actors. Hard and soft power, imperialism and political organization provide recurring analytical questions. Students critically examine primary sources and historical scholarship and develop a researched argument on a particular empire or theoretical issue.</x:v>
+      </x:c>
+      <x:c r="F161" t="str">
+        <x:v>History; Imperial history; International history</x:v>
+      </x:c>
+      <x:c r="G161" t="str">
+        <x:v>Sources and characteristics of empire; Imperial rise and decline; Hard and soft power; Imperialism and colonial legacies; Persian, Roman and Chinese empires; Mongol and Ottoman empires; European overseas empires; Modern great powers; American and Soviet power; European Union; Contemporary China; Politics and future of empire</x:v>
+      </x:c>
+      <x:c r="H161" t="str">
+        <x:v>Comparative historical analysis; Primary-source analysis; Critical historiographical analysis; Evaluation of theories of imperial power</x:v>
+      </x:c>
+      <x:c r="I161" t="str">
+        <x:v>GOSHIST211.docx</x:v>
+      </x:c>
+      <x:c r="J161" t="str">
+        <x:v>6b0ce540628dd4f7d6b6b7457e90abe2ee822265a5e7b4fa12b9922786bddd33</x:v>
+      </x:c>
+      <x:c r="K161"/>
+      <x:c r="L161"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B162" t="str">
+        <x:v>GOSLAWJ111</x:v>
+      </x:c>
+      <x:c r="C162" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D162" t="str">
+        <x:v>Human Rights: Law &amp; Philosophy</x:v>
+      </x:c>
+      <x:c r="E162" t="str">
+        <x:v>Studies human rights through legal institutions, historical development and philosophical argument. Treaties, courts and monitoring mechanisms introduce positive human-rights law and the making of the Universal Declaration. Historical declarations, natural law and legal positivism frame debates about liberty, equality, duties, virtues and cultural universality. Students locate and analyze judicial decisions, examine the European Social Charter's monitoring system, and assess contemporary cases from legal and normative perspectives.</x:v>
+      </x:c>
+      <x:c r="F162" t="str">
+        <x:v>Human rights law; Legal philosophy; Intellectual history</x:v>
+      </x:c>
+      <x:c r="G162" t="str">
+        <x:v>Universal Declaration of Human Rights; Civil and political rights; Economic and social rights; European Convention on Human Rights; European Social Charter; UN treaty bodies; American and French rights declarations; Natural law; Legal positivism; Human rights and crisis; Rights, duties and virtues; Cultural critiques of universal rights</x:v>
+      </x:c>
+      <x:c r="H162" t="str">
+        <x:v>Judicial and treaty-body case-law research; Human-rights case analysis; Analysis of compliance-monitoring mechanisms; Historical interpretation of legal texts; Comparative philosophical argumentation</x:v>
+      </x:c>
+      <x:c r="I162" t="str">
+        <x:v>GOSLAWJ111.docx</x:v>
+      </x:c>
+      <x:c r="J162" t="str">
+        <x:v>10de832a1b07c565bb1f3968a550b116743bde965afe9000c879f22e53aa9c46</x:v>
+      </x:c>
+      <x:c r="K162"/>
+      <x:c r="L162" t="str">
+        <x:v>Some classical and medieval readings remain to be announced. The record does not infer that all proposed authors or optional court visits receive substantive treatment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B163" t="str">
+        <x:v>GOSLAWJ211</x:v>
+      </x:c>
+      <x:c r="C163" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D163" t="str">
+        <x:v>Criminal Law and Criminal Justice</x:v>
+      </x:c>
+      <x:c r="E163" t="str">
+        <x:v>Examines the principles and justification of criminal law, including punishment, criminalization, legality, criminal acts, causation and mental responsibility. Justifications, excuses, inchoate offences and participation extend analysis of liability. Students interpret legal texts and case decisions, advise a hypothetical client in a simulated legal-aid clinic, and conduct a small criminology project linking a research question to gathered or existing data.</x:v>
+      </x:c>
+      <x:c r="F163" t="str">
+        <x:v>Criminal law; Criminal justice; Criminology</x:v>
+      </x:c>
+      <x:c r="G163" t="str">
+        <x:v>Retributive and utilitarian punishment; Principles of criminalization; Legality and ultima ratio; Actus reus; Omissions and causation; Mens rea; Intent, recklessness and negligence; Justifications and excuses; Self-defence, necessity, duress and insanity; Preparation and attempt; Criminal participation; Crime and society</x:v>
+      </x:c>
+      <x:c r="H163" t="str">
+        <x:v>Criminal case-law analysis; Legal reasoning applied to hypothetical facts; Legal-advice memorandum drafting; Small-scale criminological research design; Collection or analysis of criminological data</x:v>
+      </x:c>
+      <x:c r="I163" t="str">
+        <x:v>GOSLAWJ211.pdf</x:v>
+      </x:c>
+      <x:c r="J163" t="str">
+        <x:v>f20e4d0421297f7c5e73c98f58028a06a8289d2586e72ae39498decde0adebaa</x:v>
+      </x:c>
+      <x:c r="K163"/>
+      <x:c r="L163" t="str">
+        <x:v>The criminology project's data source and specific collection or analysis technique are not prescribed in the outline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B164" t="str">
+        <x:v>GOSLAWJ311</x:v>
+      </x:c>
+      <x:c r="C164" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D164" t="str">
+        <x:v>Principles of Private Law</x:v>
+      </x:c>
+      <x:c r="E164" t="str">
+        <x:v>Studies property, tort and contract law comparatively, focusing on the principles underlying rights and obligations between persons. Cases from several legal systems connect possession, liability, agreement, fairness and remedies to wider social and policy pressures. Students prepare IRAC briefs and compare a common private-law issue across three jurisdictions. A simulated mediation develops negotiation and reasoned representation of a client's position.</x:v>
+      </x:c>
+      <x:c r="F164" t="str">
+        <x:v>Private law; Comparative law; Property law; Tort law; Contract law</x:v>
+      </x:c>
+      <x:c r="G164" t="str">
+        <x:v>Possession and ownership; Nuisance; Easements and servitudes; Necessity; Intentional torts; Negligence and duties to act; Privacy; Liability in equity; Offer and acceptance; Pre-contractual liability; Contractual mistake and fairness; Excuse; Specific performance and damages; Limits on recovery; Mediation</x:v>
+      </x:c>
+      <x:c r="H164" t="str">
+        <x:v>Case-law analysis; IRAC legal briefing; Functional comparative legal research; Application of legal principles to hypothetical facts; Mediation position-statement drafting; Simulated mediation and negotiation</x:v>
+      </x:c>
+      <x:c r="I164" t="str">
+        <x:v>GOSLAWJ311.pdf</x:v>
+      </x:c>
+      <x:c r="J164" t="str">
+        <x:v>747f5b37c4da867502c4ee41e483049a4fbdb712c33a62213e12aee6fb4d87d8</x:v>
+      </x:c>
+      <x:c r="K164" t="str">
+        <x:v>The assessment description includes unjust enrichment in the final exam, while the detailed schedule and final-exam entry specify contract law and remedies without a separate unjust-enrichment component.</x:v>
+      </x:c>
+      <x:c r="L164" t="str">
+        <x:v>The record follows the substantive schedule for common topic coverage; the research paper's private-law issue and three legal systems are individually selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B165" t="str">
+        <x:v>GOSPHIL111</x:v>
+      </x:c>
+      <x:c r="C165" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D165" t="str">
+        <x:v>Introduction to Western Philosophy</x:v>
+      </x:c>
+      <x:c r="E165" t="str">
+        <x:v>Introduces central philosophical questions through historical and contemporary texts. Knowledge, scepticism and causation connect to mind, consciousness and AI; ethical theories, freedom, personal identity, religion, time and life's meaning broaden the inquiry. Students closely read arguments, assess objections and construct focused philosophical essays. The predominantly Western selection also includes Buddhist perspectives on consciousness and the self.</x:v>
+      </x:c>
+      <x:c r="F165" t="str">
+        <x:v>Philosophy; Epistemology; Metaphysics; Ethics; Philosophy of mind</x:v>
+      </x:c>
+      <x:c r="G165" t="str">
+        <x:v>Knowledge and scepticism; Virtue and the good life; Consequentialist and Kantian ethics; Moral objectivity; God and religious argument; Idealism; Causation; Mind–body problem; Consciousness and AI; Freedom and responsibility; Personal identity and non-self; Existentialism; Gender and race; Time; Meaning of life</x:v>
+      </x:c>
+      <x:c r="H165" t="str">
+        <x:v>Close reading of philosophical texts; Conceptual analysis; Logical argument reconstruction and critique; Evaluation of objections; Construction of philosophical arguments</x:v>
+      </x:c>
+      <x:c r="I165" t="str">
+        <x:v>GOSPHIL111.pdf</x:v>
+      </x:c>
+      <x:c r="J165" t="str">
+        <x:v>d80de3778ea11b3d5267253b29897df194d763e0b1a7cb83eb734adf44b83148</x:v>
+      </x:c>
+      <x:c r="K165"/>
+      <x:c r="L165"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B166" t="str">
+        <x:v>GOSPHIL211</x:v>
+      </x:c>
+      <x:c r="C166" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D166" t="str">
+        <x:v>Wisdom of the East</x:v>
+      </x:c>
+      <x:c r="E166" t="str">
+        <x:v>Examines the philosophical and ethical dimensions of Hinduism, Buddhism, Confucianism, Taoism, Sikhism, Judaism, Christianity and Islam. Close engagement with sacred texts and comparative discussion explore relationships among humanity, the divine, religious ways of life and claims to universal truth. Conversion, veiling and relations with non-believers connect these traditions to modern secular contexts, while an individually chosen study applies religious ideas to a focused question.</x:v>
+      </x:c>
+      <x:c r="F166" t="str">
+        <x:v>Religious studies; Comparative religion; Philosophy of religion; Religious ethics</x:v>
+      </x:c>
+      <x:c r="G166" t="str">
+        <x:v>Religious worldviews and ways of life; Hinduism; Buddhism; Confucianism; Taoism; Sikhism; Judaism; Christianity; Islam; Humanity and divine order; Universal truth claims; Meaningful life; Religious conversion; Women's religious experiences; Veiling and seclusion; Religious traditions and secular modernity; Interfaith relations</x:v>
+      </x:c>
+      <x:c r="H166" t="str">
+        <x:v>Close reading of sacred texts; Comparative analysis of religious philosophies; Philosophical interpretation; Application of religious-ethical concepts to a selected case</x:v>
+      </x:c>
+      <x:c r="I166" t="str">
+        <x:v>GOSPHIL211.docx</x:v>
+      </x:c>
+      <x:c r="J166" t="str">
+        <x:v>8de1591185258a16484af89a26c1a608bc63453617edc449bd7ed1a01875c1be</x:v>
+      </x:c>
+      <x:c r="K166"/>
+      <x:c r="L166" t="str">
+        <x:v>Illustrative presentation topics are options rather than common course coverage; supplementary primary-text excerpts are selected during the course.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B167" t="str">
+        <x:v>GOSPHIL311</x:v>
+      </x:c>
+      <x:c r="C167" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D167" t="str">
+        <x:v>Philosophy of Emotion</x:v>
+      </x:c>
+      <x:c r="E167" t="str">
+        <x:v>Examines what emotions are and how they shape knowledge, decision-making, ethics, social life and politics. Feeling, cognitive and perceptual theories are compared with historical, phenomenological and contemporary accounts. Love, fear, grief, moods and political anger provide focused cases, alongside emotions in art and their changing relation to time. Students analyze texts and emotional vignettes and develop an independent philosophical paper or a project combining argument with creative work.</x:v>
+      </x:c>
+      <x:c r="F167" t="str">
+        <x:v>Philosophy of emotion; Philosophy of mind; Ethics; Political philosophy; Aesthetics</x:v>
+      </x:c>
+      <x:c r="G167" t="str">
+        <x:v>Feeling, cognitive and perceptual theories of emotion; Ancient Greek and Indian accounts of emotion; Epistemic emotions; Emotion and decision-making; Love; Fear and existential anxiety; Mood and grief; Moral emotions; Gender and emotion; Political love and anger; Racial injustice; Temporality of emotion; Emotion and artistic expression</x:v>
+      </x:c>
+      <x:c r="H167" t="str">
+        <x:v>Close philosophical reading; Conceptual and argumentative analysis; Phenomenological description of emotional experience; Critical comparison of emotion theories</x:v>
+      </x:c>
+      <x:c r="I167" t="str">
+        <x:v>GOSPHIL311.pdf</x:v>
+      </x:c>
+      <x:c r="J167" t="str">
+        <x:v>c654450123712a69b68ec3176b4c06115227856bc6433e75a9835fdf4164becd</x:v>
+      </x:c>
+      <x:c r="K167"/>
+      <x:c r="L167" t="str">
+        <x:v>The learning-outcomes table includes dedicated disgust and cognitive-science blocks that are not clearly matched in the detailed schedule. The profile and topics follow the scheduled course; creative work is an alternative final-project format.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B168" t="str">
+        <x:v>GOSPOLI111</x:v>
+      </x:c>
+      <x:c r="C168" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D168" t="str">
+        <x:v>Introduction to Political Philosophy</x:v>
+      </x:c>
+      <x:c r="E168" t="str">
+        <x:v>Examines influential Western accounts of human nature, society and political authority from classical antiquity to contemporary thought. Students compare justifications for political power and the historical problems those theories address, connecting past arguments to present political questions. Primary-text interpretation and a researched essay develop the ability to identify assumptions, assess normative claims and explain the continuing influence of political ideas.</x:v>
+      </x:c>
+      <x:c r="F168" t="str">
+        <x:v>Political philosophy; Political theory; History of political thought</x:v>
+      </x:c>
+      <x:c r="G168" t="str">
+        <x:v>Political authority and legitimacy; Human nature and society; Classical citizenship and democracy; Religion and politics; Political realism; Social contract and rights; Enlightenment; Conservatism; Liberalism and utilitarianism; Nationalism; Socialism and communism; Fascism and totalitarianism; Justice and welfare state; Neoliberalism; Multicultural society</x:v>
+      </x:c>
+      <x:c r="H168" t="str">
+        <x:v>Close analysis of political-philosophical texts; Assumption analysis; Historical contextualization of political ideas; Comparative normative argumentation; Application of political theory to contemporary questions</x:v>
+      </x:c>
+      <x:c r="I168" t="str">
+        <x:v>GOSPOLI111.docx</x:v>
+      </x:c>
+      <x:c r="J168" t="str">
+        <x:v>4d2310883ea5582a3bf21760b9a70a07ae8e2da48e62aacfcaa812a10b2cbe64</x:v>
+      </x:c>
+      <x:c r="K168"/>
+      <x:c r="L168"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B169" t="str">
+        <x:v>GOSPOLI112</x:v>
+      </x:c>
+      <x:c r="C169" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D169" t="str">
+        <x:v>Foundations of Comparative Politics</x:v>
+      </x:c>
+      <x:c r="E169" t="str">
+        <x:v>Introduces theory-driven comparison of political systems, emphasizing democracy, authoritarianism and institutional change. State–society relations, political culture, executives, legislatures, courts, parties, participation and policy provide a framework for examining contemporary democratic challenges. Students analyze democracy data, compare conventional and AI-assisted literature searches, and conduct a small qualitative or quantitative research project that answers a theoretically grounded question with empirical evidence.</x:v>
+      </x:c>
+      <x:c r="F169" t="str">
+        <x:v>Political science; Comparative politics; Political research methods</x:v>
+      </x:c>
+      <x:c r="G169" t="str">
+        <x:v>States, nations and civil society; Democratization; Authoritarianism and democratic backsliding; Political culture; Constitutions and courts; Executives and coalition government; Legislatures; Bureaucracies; Populism; Subnational government; Media and politics; Participation and polarization; Electoral and party systems; Interest groups; Public policy; Political economy</x:v>
+      </x:c>
+      <x:c r="H169" t="str">
+        <x:v>Comparative political analysis; Analysis of Varieties of Democracy data; Theory-driven qualitative or quantitative empirical research; Comparative evaluation of academic and AI-assisted literature searches; Election analysis</x:v>
+      </x:c>
+      <x:c r="I169" t="str">
+        <x:v>GOSPOLI112.pdf</x:v>
+      </x:c>
+      <x:c r="J169" t="str">
+        <x:v>c23ef0813e5da74903af4351bbc7c99788c90f29faa2a785c7f2938b0a5a4cea</x:v>
+      </x:c>
+      <x:c r="K169" t="str">
+        <x:v>The cover identifies GOSPOLI112, Fall 2025, while the following title and learning-outcomes table retain GOSPOLI211 and the inner title says Spring 2025. The authoritative key remains 2025h2/GOSPOLI112.</x:v>
+      </x:c>
+      <x:c r="L169" t="str">
+        <x:v>Research projects can use qualitative or quantitative approaches; the outline does not require every student to apply each method listed among the learning outcomes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B170" t="str">
+        <x:v>GOSPOLI311</x:v>
+      </x:c>
+      <x:c r="C170" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D170" t="str">
+        <x:v>European Union Politics</x:v>
+      </x:c>
+      <x:c r="E170" t="str">
+        <x:v>Examines EU integration, institutions, actors and decision-making, connecting public opinion, party politics and policy implementation to legitimacy and effectiveness. The second part investigates interest representation and the relative access of business and other groups. Students trace a legislative dossier, classify organizations and code parliamentary amendments, using original institutional information to analyze interactions between interest groups and EU policymakers.</x:v>
+      </x:c>
+      <x:c r="F170" t="str">
+        <x:v>Political science; European Union studies; Public policy</x:v>
+      </x:c>
+      <x:c r="G170" t="str">
+        <x:v>European integration; EU institutions; Legislative decision-making; Public opinion; Political parties and European Parliament; Interest representation; Agenda setting; Crisis policymaking; Policy implementation; Input and output legitimacy; Interest-group access; Business lobbying; Legislative amendments</x:v>
+      </x:c>
+      <x:c r="H170" t="str">
+        <x:v>EU policy-document research; Legislative process tracing; Classification of interest organizations; Coding of parliamentary amendments; Analysis of transparency-register and access data; Comparative analysis of EU news coverage</x:v>
+      </x:c>
+      <x:c r="I170" t="str">
+        <x:v>GOSPOLI311.pdf</x:v>
+      </x:c>
+      <x:c r="J170" t="str">
+        <x:v>fe6e69caa4993df1da7417c063185c9e640686b53b02f5c3c9fdcce838a4051e</x:v>
+      </x:c>
+      <x:c r="K170"/>
+      <x:c r="L170" t="str">
+        <x:v>The legislative dossier is selected during the course; the European Commission may be included alongside the Parliament. The outline does not establish a quantitative causal estimate of lobbying influence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B171" t="str">
+        <x:v>GOSSOCI111</x:v>
+      </x:c>
+      <x:c r="C171" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D171" t="str">
+        <x:v>INTRODUCTION TO SOCIOLOGY</x:v>
+      </x:c>
+      <x:c r="E171" t="str">
+        <x:v>Introduces sociological ways of explaining social life through classical and contemporary perspectives. Agency, social structure, solidarity and inequality connect to gender, race, crime, networks, resources and digital society. The course critically situates the classical canon within colonial and imperial histories and includes marginalized perspectives. Students formulate a sociological research question, build a theoretical framework from literature, and propose and evaluate two ways to investigate it.</x:v>
+      </x:c>
+      <x:c r="F171" t="str">
+        <x:v>Sociology; Social theory; Sociological research methods</x:v>
+      </x:c>
+      <x:c r="G171" t="str">
+        <x:v>Sociological imagination; Agency and social structure; Norms, roles and institutions; Classical sociology and colonialism; Solidarity; Gender and race; Crime; Groups and social networks; Stratification and mobility; Resources and inequality; Digital society; Alienation and commodity fetishism; Emotional labour</x:v>
+      </x:c>
+      <x:c r="H171" t="str">
+        <x:v>Sociological theory application; Critical analysis of social-scientific literature; Research-question development; Comparative research-method design; Assessment of access, positionality and research ethics</x:v>
+      </x:c>
+      <x:c r="I171" t="str">
+        <x:v>GOSSOCI111.pdf</x:v>
+      </x:c>
+      <x:c r="J171" t="str">
+        <x:v>42726f0181cb84e4971da9c5eafc6b1e2b9d77fcaa7e64cd79fc698c2185ff03</x:v>
+      </x:c>
+      <x:c r="K171"/>
+      <x:c r="L171" t="str">
+        <x:v>The final paper proposes two research methods and examines their limitations; it does not require students to complete the proposed interviews, ethnography or other data collection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B172" t="str">
+        <x:v>GOSSOCI311</x:v>
+      </x:c>
+      <x:c r="C172" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D172" t="str">
+        <x:v>NEW ISSUES IN CONTEMPORARY SOCIOLOGY</x:v>
+      </x:c>
+      <x:c r="E172" t="str">
+        <x:v>Examines civil society through critical, civil-sphere and decolonial theories. Social capital, trust, hegemony, public communication, solidarity and civil repair are studied through global cases and competing accounts of inclusion and exclusion. Students directly engage with a civil society organization, document observations, and connect empirical material to at least two theoretical perspectives. An individual paper also analyzes how the researcher's positionality shapes interpretation.</x:v>
+      </x:c>
+      <x:c r="F172" t="str">
+        <x:v>Sociology; Social theory; Political sociology; Cultural sociology</x:v>
+      </x:c>
+      <x:c r="G172" t="str">
+        <x:v>Civil society; Social trust and social capital; Hegemony; Critical theory; Public sphere and communicative power; Feminist critiques of participation; Solidarity and social cohesion; Social performance and drama; Civil-sphere codes and institutions; Exclusion and civil repair; Latin American civil society; Migrant solidarity; Decolonial critique; Researcher positionality</x:v>
+      </x:c>
+      <x:c r="H172" t="str">
+        <x:v>Community-engaged organizational research; Field observation and documentation; Application and comparison of sociological theories; Reflexive positionality analysis</x:v>
+      </x:c>
+      <x:c r="I172" t="str">
+        <x:v>GOSSOCI311.docx</x:v>
+      </x:c>
+      <x:c r="J172" t="str">
+        <x:v>ee1901ca5ed4dc2944b55242b207f688410ded852de1e9e14e92c8185c4144f7</x:v>
+      </x:c>
+      <x:c r="K172" t="str">
+        <x:v>The cover and course description identify GOSSOCI311, while an inner heading retains GOSSOCI301.</x:v>
+      </x:c>
+      <x:c r="L172" t="str">
+        <x:v>Groups choose at least two feasible forms of engagement. Interviews, volunteering and activity design are options, so no single one is claimed as compulsory for all students.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B173" t="str">
+        <x:v>GOSSOCI312</x:v>
+      </x:c>
+      <x:c r="C173" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D173" t="str">
+        <x:v>Anthropology of Religion</x:v>
+      </x:c>
+      <x:c r="E173" t="str">
+        <x:v>Examines religion as an anthropological category through classical theories, contemporary critiques and ethnographic inquiry. Ritual, symbolism, mediation, materiality, secularism, purity, authority, belonging and migration connect religious practices to wider cultural relations. Students conduct participant observation in person or online and an ethnographic interview, attending to consent, positionality and fieldwork ethics. A literature-based research paper develops a focused anthropological argument about religion.</x:v>
+      </x:c>
+      <x:c r="F173" t="str">
+        <x:v>Cultural anthropology; Anthropology of religion; Religious studies</x:v>
+      </x:c>
+      <x:c r="G173" t="str">
+        <x:v>Anthropological definitions of religion; Classical and contemporary religious theory; Ritual and symbolism; Religious mediation and materiality; Secularism; Purity, pollution and taboo; Religion and food; Religious worldmaking; Authority; Belief and belonging; Migration and diaspora; Heritage; Decolonizing religious studies; Ethnographic ethics and positionality</x:v>
+      </x:c>
+      <x:c r="H173" t="str">
+        <x:v>Participant observation; In-person or virtual ethnography; Ethnographic interviewing; Field-note writing; Interview transcription; Reflexive ethnographic reporting; Thick description; Anthropological literature analysis</x:v>
+      </x:c>
+      <x:c r="I173" t="str">
+        <x:v>GOSSOCI312.docx</x:v>
+      </x:c>
+      <x:c r="J173" t="str">
+        <x:v>a4316d9ce34c591f51cddfe2eb8e7bd7e71cad086b9f507623c7b96b7f55655b</x:v>
+      </x:c>
+      <x:c r="K173"/>
+      <x:c r="L173" t="str">
+        <x:v>The observation exercise offers in-person and virtual alternatives; it does not require both. The final paper analyzes published social-scientific literature rather than necessarily extending the student's own fieldwork.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B174" t="str">
+        <x:v>HCBBIOM311</x:v>
+      </x:c>
+      <x:c r="C174" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D174" t="str">
+        <x:v>Pharmacology</x:v>
+      </x:c>
+      <x:c r="E174" t="str">
+        <x:v>Studies how drugs act on molecular targets and how the body absorbs, distributes, metabolizes and eliminates them. Quantitative pharmacodynamics and pharmacokinetics connect receptor interactions to therapeutic action, adverse effects and drug development. Antimicrobial, inflammatory, respiratory and nervous-system applications extend the principles. Students calculate drug parameters, undertake virtual simulation assignments and analyze a psychoactive drug, including a proposed experiment addressing a research gap.</x:v>
+      </x:c>
+      <x:c r="F174" t="str">
+        <x:v>Pharmacology; Biomedical science; Neuropharmacology</x:v>
+      </x:c>
+      <x:c r="G174" t="str">
+        <x:v>Drug discovery and development; Drug–receptor interactions; Pharmacodynamics; Absorption, distribution, metabolism and elimination; Pharmacokinetics; Concentration–response relationships; Drug toxicity; Antimicrobial therapy; Inflammatory mediators; Respiratory treatment; Autonomic regulation; Psychoactive drugs; Immunopharmacology; Pharmacological ethics; Homeopathy evaluation</x:v>
+      </x:c>
+      <x:c r="H174" t="str">
+        <x:v>Quantitative pharmacodynamic and pharmacokinetic modelling; Calculation of concentration–response and time–concentration parameters; Virtual organ-bath simulation; Critical analysis of drug-mechanism literature; Hypothesis and experimental-proposal development</x:v>
+      </x:c>
+      <x:c r="I174" t="str">
+        <x:v>HCBBIOM311.pdf</x:v>
+      </x:c>
+      <x:c r="J174" t="str">
+        <x:v>f76e36b8bc1b199b55229c252d3da9f80ef1e3421920d4a607049f87cf825654</x:v>
+      </x:c>
+      <x:c r="K174"/>
+      <x:c r="L174" t="str">
+        <x:v>The organ-bath work is described as virtual practical work and simulation. The proposed neuropharmacological experiment is designed, not performed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B175" t="str">
+        <x:v>HCBCOGN111</x:v>
+      </x:c>
+      <x:c r="C175" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D175" t="str">
+        <x:v>Introduction to Cognitive Science</x:v>
+      </x:c>
+      <x:c r="E175" t="str">
+        <x:v>Introduces cognition through neural communication, brain anatomy and the methods used to investigate brain function. Sensation, perception, object recognition, action, memory and emotion are studied at behavioural, cellular and systems levels, followed by brain development and nature–nurture relationships. Students evaluate the possibilities and limitations of imaging and lesion evidence and critically analyze scientific articles; a paired memory assignment applies part of the course material.</x:v>
+      </x:c>
+      <x:c r="F175" t="str">
+        <x:v>Cognitive science; Cognitive neuroscience; Cognitive psychology</x:v>
+      </x:c>
+      <x:c r="G175" t="str">
+        <x:v>History of cognitive neuroscience; Mind–body problem; Neural signalling and synapses; Neuroanatomy; Brain-imaging and stimulation methods; Hemispheric lateralization; Somatosensation; Audition and vision; Object and face recognition; Motor control; Memory systems; Emotion and cognition; Brain development; Nature and nurture</x:v>
+      </x:c>
+      <x:c r="H175" t="str">
+        <x:v>Critical appraisal of cognitive-neuroscience research; Interpretation of evidence from brain-imaging and lesion studies</x:v>
+      </x:c>
+      <x:c r="I175" t="str">
+        <x:v>HCBCOGN111.pdf</x:v>
+      </x:c>
+      <x:c r="J175" t="str">
+        <x:v>83b9e4bece0f44559546ecee2857756ad0943efdc79ac52421859eea478baf7a</x:v>
+      </x:c>
+      <x:c r="K175" t="str">
+        <x:v>The first-page footer identifies HCBPSYC101 Introduction to Brain &amp; Behavior, whereas the title, later footers and authoritative filename identify HCBCOGN111 Introduction to Cognitive Science.</x:v>
+      </x:c>
+      <x:c r="L175" t="str">
+        <x:v>Imaging and stimulation techniques are introduced and compared, not taught as hands-on instrument operation. The paired memory assignment's protocol is provided separately and is not specified in this outline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B176" t="str">
+        <x:v>HCBCOGN311</x:v>
+      </x:c>
+      <x:c r="C176" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D176" t="str">
+        <x:v>Advanced Cognitive Science: Higher Order Functions</x:v>
+      </x:c>
+      <x:c r="E176" t="str">
+        <x:v>Examines higher cognitive functions through neurophysiology, neuroanatomy and current experimental evidence. Attention, memory, emotion, language, cognitive control, social cognition and consciousness connect to psychoactive drugs, pain and neuroethics. Students critically assess research and design a feasible experimental proposal, developing a research question, substantiated methods and ethical reasoning. Discussions of AI emotion and consciousness place selected cognitive questions in a contemporary context.</x:v>
+      </x:c>
+      <x:c r="F176" t="str">
+        <x:v>Cognitive neuroscience; Cognitive psychology; Neuropsychopharmacology</x:v>
+      </x:c>
+      <x:c r="G176" t="str">
+        <x:v>Psychoactive drug mechanisms and individual responses; Attention; Memory and amnesia; Long-term potentiation; Emotion and emotion regulation; Language; Cognitive control; Decision-making and planning; Social cognition; Pain; Consciousness; Neuroethics; AI and cognition</x:v>
+      </x:c>
+      <x:c r="H176" t="str">
+        <x:v>Critical evaluation of cognitive-neuroscience research; Experimental research design; Literature-based hypothesis development; Ethical analysis of proposed neuroscience research</x:v>
+      </x:c>
+      <x:c r="I176" t="str">
+        <x:v>HCBCOGN311.pdf</x:v>
+      </x:c>
+      <x:c r="J176" t="str">
+        <x:v>4139e4506f584deac13c10737e3a3551b5cc86e9ec9de75e30c18c9226ededc0</x:v>
+      </x:c>
+      <x:c r="K176" t="str">
+        <x:v>The first-page footer identifies HCBPSYC101 Introduction to Brain &amp; Behavior, whereas the title, later footers and authoritative filename identify HCBCOGN311 Advanced Cognitive Science: Higher Order Functions.</x:v>
+      </x:c>
+      <x:c r="L176" t="str">
+        <x:v>The assessed research output is an experimental proposal, report and presentation; the outline does not require students to execute the experiment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B177" t="str">
+        <x:v>HCBGATE101</x:v>
+      </x:c>
+      <x:c r="C177" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D177" t="str">
+        <x:v>Foundation of Life, Health &amp; Biomedical Science</x:v>
+      </x:c>
+      <x:c r="E177" t="str">
+        <x:v>Introduces the cellular and molecular foundations of life and their relevance to health and disease. Biological molecules, membranes, metabolism and cell communication lead into the cell cycle, heredity, gene expression, genomes and biotechnology. Selected applications examine outbreaks, cancer, lung disease and immunodeficiency. Students interpret published experiments and scientific literature and synthesize a biomedical question for a research presentation and mini-symposium.</x:v>
+      </x:c>
+      <x:c r="F177" t="str">
+        <x:v>Cell biology; Molecular biology; Biochemistry; Biomedical science</x:v>
+      </x:c>
+      <x:c r="G177" t="str">
+        <x:v>Biological macromolecules; Origin of life; Cell structure and membranes; Cellular communication; Enzymes and metabolism; Cellular energy pathways; Cell cycle and division; DNA and heredity; Protein synthesis; Gene mutation and regulation; Genomics; Recombinant DNA and biotechnology; Outbreak management; Cancer biology; Obstructive lung disease; Immunodeficiency</x:v>
+      </x:c>
+      <x:c r="H177" t="str">
+        <x:v>Critical interpretation of published biological experiments; Biomedical literature searching and synthesis; Analysis of molecular mechanisms</x:v>
+      </x:c>
+      <x:c r="I177" t="str">
+        <x:v>HCBGATE101.docx</x:v>
+      </x:c>
+      <x:c r="J177" t="str">
+        <x:v>8c91b11a15cd1c067c44c44ca41325d7ceb13500035451092ffe5f024430752d</x:v>
+      </x:c>
+      <x:c r="K177" t="str">
+        <x:v>The outline is labelled Fall 2025 and almost all schedule dates are in 2025, but the final mini-symposium entry is dated 18/12/2024. The authoritative semester is 2025h2.</x:v>
+      </x:c>
+      <x:c r="L177" t="str">
+        <x:v>Microscopy, electrophoresis, cloning and CRISPR appear as topics of student explanations of published research tools or experiments; no hands-on training in these techniques is established.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B178" t="str">
+        <x:v>HCBGATE102</x:v>
+      </x:c>
+      <x:c r="C178" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D178" t="str">
+        <x:v>Introduction to Brain &amp; Behavior</x:v>
+      </x:c>
+      <x:c r="E178" t="str">
+        <x:v>Introduces psychological and neuroscientific explanations of human behaviour. Neural signalling, brain anatomy and development are studied alongside learning, intelligence, personality, self-concept and social influences. Research methods and structural and functional imaging introduce how brain–behaviour relationships are investigated. Psychopathology, diagnostic classification, treatment approaches and clinical skills provide an introductory applied dimension, with case analysis and reflection on difficult concepts.</x:v>
+      </x:c>
+      <x:c r="F178" t="str">
+        <x:v>Psychology; Clinical psychology; Cognitive neuroscience</x:v>
+      </x:c>
+      <x:c r="G178" t="str">
+        <x:v>Psychological and neuroscientific perspectives; Neural communication; Brain anatomy and development; Habituation and sensitization; Classical, operant and social learning; Intelligence; Personality and self-concept; Social influence; Psychological research methods; Structural and functional brain imaging; Psychopathology; DSM-5-TR; Treatment of psychological disorders; Introductory clinical skills</x:v>
+      </x:c>
+      <x:c r="H178" t="str">
+        <x:v>Psychological case-study analysis; Critical interpretation of neuroscientific methods and findings</x:v>
+      </x:c>
+      <x:c r="I178" t="str">
+        <x:v>HCBGATE102.pdf</x:v>
+      </x:c>
+      <x:c r="J178" t="str">
+        <x:v>8ba0c8e8b7c6286f2c732506293ea2e6258eefcc691e841a37b7be4276f96698</x:v>
+      </x:c>
+      <x:c r="K178"/>
+      <x:c r="L178" t="str">
+        <x:v>Imaging, stimulation and computational techniques are introduced conceptually; the outline does not establish hands-on technical or clinical-assessment competence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="A179" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B179" t="str">
+        <x:v>HCBLIFE211</x:v>
+      </x:c>
+      <x:c r="C179" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D179" t="str">
+        <x:v>Molecular Cell Biology</x:v>
+      </x:c>
+      <x:c r="E179" t="str">
+        <x:v>Studies the molecular mechanisms underlying cellular structure, physiology and regulation, primarily in eukaryotes. Bioenergetics, proteins and membranes connect to genome replication, repair and gene expression, followed by trafficking, signalling, division, tissues, stem cells and cancer. Students evaluate research methods and reproducibility and investigate a drug's molecular target, therapeutic action, metabolism and adverse effects through primary literature, a paper and a research poster.</x:v>
+      </x:c>
+      <x:c r="F179" t="str">
+        <x:v>Molecular biology; Cell biology; Biochemistry</x:v>
+      </x:c>
+      <x:c r="G179" t="str">
+        <x:v>Cellular components and bioenergetics; Proteins and membranes; Cytoskeleton; DNA replication and repair; Genomes; Regulation of gene expression; Membrane transport and trafficking; Cell-signalling pathways; Cell division and fate; Tissue organization; Stem cells; Cancer; Molecular mechanisms of drug action</x:v>
+      </x:c>
+      <x:c r="H179" t="str">
+        <x:v>Critical analysis of primary molecular-biology literature; Evaluation of research-method limitations and reproducibility; Thermodynamic free-energy calculations; Molecular mechanism analysis</x:v>
+      </x:c>
+      <x:c r="I179" t="str">
+        <x:v>HCBLIFE211.pdf</x:v>
+      </x:c>
+      <x:c r="J179" t="str">
+        <x:v>9f344b6d90a7031554378b6e93fff5dd9e19d2b6fa6f9046925937a26c8c9c1e</x:v>
+      </x:c>
+      <x:c r="K179" t="str">
+        <x:v>The outline uses the dual identity SCILIFE201/HCBLIFE211; the authoritative filename code is HCBLIFE211. The final-exam chapter list differs from the preceding schedule's stem-cell and cancer chapters.</x:v>
+      </x:c>
+      <x:c r="L179" t="str">
+        <x:v>The record follows the named topics in the teaching schedule. Microscopy and other research technologies are studied critically; no hands-on laboratory technique is specified.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="A180" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B180" t="str">
+        <x:v>HCBLIFE212</x:v>
+      </x:c>
+      <x:c r="C180" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D180" t="str">
+        <x:v>Human Physiology</x:v>
+      </x:c>
+      <x:c r="E180" t="str">
+        <x:v>Studies normal adult human function through the integration of cellular processes and organ systems. Homeostasis, membrane dynamics and communication support nervous, endocrine, muscular, respiratory, cardiovascular, renal, digestive and reproductive physiology. Metabolism, exercise and growth connect functions across systems. Students investigate a selected physiological topic through scientific literature and develop a review paper through structured peer review, discussion and revision.</x:v>
+      </x:c>
+      <x:c r="F180" t="str">
+        <x:v>Human physiology; Systems physiology; Cell physiology</x:v>
+      </x:c>
+      <x:c r="G180" t="str">
+        <x:v>Homeostasis and control systems; Cell and tissue compartments; Membrane dynamics; Neural and endocrine communication; Muscles and motor control; Breathing and gas exchange; Blood and cardiovascular function; Blood-pressure regulation; Renal function; Fluid and electrolyte balance; Digestion; Metabolism and energy balance; Growth; Exercise; Reproduction and development</x:v>
+      </x:c>
+      <x:c r="H180" t="str">
+        <x:v>Physiological literature searching; Critical synthesis in a review paper; Structured scientific peer review</x:v>
+      </x:c>
+      <x:c r="I180" t="str">
+        <x:v>HCBLIFE212.pdf</x:v>
+      </x:c>
+      <x:c r="J180" t="str">
+        <x:v>fbb0d693101193c61ca13f8078015aab5c38ee78b1afb1cfcb1c22ab4c7e8e44</x:v>
+      </x:c>
+      <x:c r="K180"/>
+      <x:c r="L180" t="str">
+        <x:v>Disease examples illustrate normal function. The learning outcomes mention body-function measurement and a function-laboratory excursion, but no specific practical measurement protocol is supplied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="A181" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B181" t="str">
+        <x:v>HCBLIFE213</x:v>
+      </x:c>
+      <x:c r="C181" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D181" t="str">
+        <x:v>Biochemistry</x:v>
+      </x:c>
+      <x:c r="E181" t="str">
+        <x:v>Studies the chemistry of biological molecules and the reactions that sustain life. Protein structure and enzyme action lead into carbohydrates, lipids and the regulation of major metabolic pathways, including glycolysis, the citric acid cycle, oxidative phosphorylation and nitrogen metabolism. Students interpret biochemical mechanisms and investigate a disease whose molecular defect explains symptoms, diagnostic tests and treatment, communicating the analysis in a paper and poster.</x:v>
+      </x:c>
+      <x:c r="F181" t="str">
+        <x:v>Biochemistry; Biological chemistry; Metabolic biochemistry</x:v>
+      </x:c>
+      <x:c r="G181" t="str">
+        <x:v>Water and weak bonds; Amino acids and protein structure; Protein biochemistry techniques; Enzyme action, kinetics and regulation; Enzyme inhibitors; Haemoglobin; Carbohydrates and lipids; Metabolic regulation; Glycolysis and gluconeogenesis; Citric acid cycle; Oxidative phosphorylation; Glycogen metabolism; Pentose phosphate pathway; Fatty-acid metabolism; Urea cycle; Biochemical mechanisms of disease</x:v>
+      </x:c>
+      <x:c r="H181" t="str">
+        <x:v>Biochemical reaction and pathway analysis; Enzyme-kinetic interpretation; Critical analysis of primary biochemical literature; Mechanistic analysis of disease, diagnosis and treatment</x:v>
+      </x:c>
+      <x:c r="I181" t="str">
+        <x:v>HCBLIFE213.pdf</x:v>
+      </x:c>
+      <x:c r="J181" t="str">
+        <x:v>443b6f8eec4b83df35eecce45a67c64d2c27b6d8b8bf3be0a82049488ec353bd</x:v>
+      </x:c>
+      <x:c r="K181" t="str">
+        <x:v>The first text page uses SCICHEM202 2025-2 (HCBLIFE213); the authoritative filename code is HCBLIFE213. Some exam chapter ranges differ from the named topics in the preceding teaching schedule.</x:v>
+      </x:c>
+      <x:c r="L181" t="str">
+        <x:v>The title Biochemistry and Fall 2025 are visible in the cover image. Proteomics techniques are researched and explained in presentations; no hands-on laboratory technique is specified. The record follows the named teaching topics rather than inconsistent exam chapter references.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="A182" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B182" t="str">
+        <x:v>HCBPSYC211</x:v>
+      </x:c>
+      <x:c r="C182" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D182" t="str">
+        <x:v>Statistics &amp; Experimental Methods in Health &amp; Behavioral Sciences</x:v>
+      </x:c>
+      <x:c r="E182" t="str">
+        <x:v>Develops quantitative research design and statistical analysis for health and behavioural questions. Linear models connect correlation, multiple regression, group comparisons and covariate adjustment to repeated-measures and mixed designs, logistic regression and factor analysis. Students analyze real datasets in R, usually through R Commander, check assumptions, justify model selection and report results in APA format through a staged paper, a workshop and a research poster.</x:v>
+      </x:c>
+      <x:c r="F182" t="str">
+        <x:v>Statistics; Quantitative psychology; Health and behavioural research methods</x:v>
+      </x:c>
+      <x:c r="G182" t="str">
+        <x:v>Experimental, quasi-experimental and nonexperimental design; Statistical inference; Correlation; Multiple regression and dummy coding; Model assumptions; Mean comparisons; Nonparametric testing; ANOVA and ANCOVA; Factorial interactions; Repeated-measures and mixed designs; Logistic regression; Principal components and exploratory factor analysis; Scale reliability; Effect size and power; Statistical reporting</x:v>
+      </x:c>
+      <x:c r="H182" t="str">
+        <x:v>Statistical analysis in R and R Commander; Linear and logistic regression; Regression diagnostics; t-tests and nonparametric alternatives; ANOVA and ANCOVA; Repeated-measures and mixed-design analysis; Principal component analysis; Exploratory factor analysis; Cronbach's alpha; Quantitative model selection and APA reporting</x:v>
+      </x:c>
+      <x:c r="I182" t="str">
+        <x:v>HCBPSYC211.docx</x:v>
+      </x:c>
+      <x:c r="J182" t="str">
+        <x:v>52964b68c59177a2f99860495d340c628491424e78673c559b188626ee370400</x:v>
+      </x:c>
+      <x:c r="K182"/>
+      <x:c r="L182" t="str">
+        <x:v>R Commander is the principal interface; direct R coding is allowed and SPSS is optional. The assigned analyses use real datasets, including data from experimental studies; the outline does not establish that every student collects new experimental data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="A183" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B183" t="str">
+        <x:v>HCBPSYC311</x:v>
+      </x:c>
+      <x:c r="C183" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D183" t="str">
+        <x:v>Medical &amp; Health Psychology</x:v>
+      </x:c>
+      <x:c r="E183" t="str">
+        <x:v>Examines health and illness through interactions among biological, psychological and sociocultural factors. Health inequalities, behaviour and prevention lead into stress, symptoms, pain, medical consultation and treatment decisions. Chronic illness is considered from patients', families' and healthcare professionals' perspectives. Students analyze research, interventions and clinical cases, practice interviewing with attention to culture, and apply clinical-health formulation to understand support and quality of life in medical settings.</x:v>
+      </x:c>
+      <x:c r="F183" t="str">
+        <x:v>Health psychology; Medical psychology; Clinical health psychology</x:v>
+      </x:c>
+      <x:c r="G183" t="str">
+        <x:v>Biopsychosocial model; Health inequalities; Health-risk and protective behaviours; Behaviour-change models; Prevention; Stress and coping; Symptom perception; Somatic symptom disorders; Medical consultation; Shared decision-making; Doctor–patient communication; Pain; Chronic illness; Family and caregiver experiences; Quality of life; Cultural competence; Support for healthcare professionals</x:v>
+      </x:c>
+      <x:c r="H183" t="str">
+        <x:v>Psychological case-study analysis; Critical appraisal of health-psychology research and interventions; Clinical-health case formulation; Interviewing-skills practice; Cultural Formulation Interview analysis</x:v>
+      </x:c>
+      <x:c r="I183" t="str">
+        <x:v>HCBPSYC311.pdf</x:v>
+      </x:c>
+      <x:c r="J183" t="str">
+        <x:v>b2a319853aa4f0a3e7c8aad83fab2bcb95fdb7e4fec3e9d01a7a41aca21f460e</x:v>
+      </x:c>
+      <x:c r="K183"/>
+      <x:c r="L183" t="str">
+        <x:v>Interviewing is practiced in training sessions; the outline does not establish supervised clinical treatment of patients.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="A184" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B184" t="str">
+        <x:v>MCCCOMM111</x:v>
+      </x:c>
+      <x:c r="C184" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D184" t="str">
+        <x:v>The Art of Rhetorical Communication</x:v>
+      </x:c>
+      <x:c r="E184" t="str">
+        <x:v>Introduces classical rhetoric as both a historical tradition and a practical art of persuasion. Greek and Roman foundations extend into Christian, Renaissance and Enlightenment rhetoric. Students study invention, arrangement, style, memory and delivery, including rhetorical appeals, fallacies and figures of speech. Written exercises, dialectical debates and an individual speech develop reasoned, structured and audience-aware oral and written communication.</x:v>
+      </x:c>
+      <x:c r="F184" t="str">
+        <x:v>Rhetoric; Communication studies; Argumentation studies</x:v>
+      </x:c>
+      <x:c r="G184" t="str">
+        <x:v>History and theory of rhetoric; Deliberative, forensic and epideictic discourse; Invention; Arrangement; Rhetorical style; Memory and delivery; Logos, ethos and pathos; Fallacies; Tropes and schemes; Stasis theory; Enthymemes; Dialectical debate; Persuasive speech composition</x:v>
+      </x:c>
+      <x:c r="H184" t="str">
+        <x:v>Rhetorical discourse analysis; Argument invention and arrangement; Stasis analysis; Rhetorical figure analysis; Dialectical debating; Persuasive speechwriting and delivery</x:v>
+      </x:c>
+      <x:c r="I184" t="str">
+        <x:v>MCCCOMM111.pdf</x:v>
+      </x:c>
+      <x:c r="J184" t="str">
+        <x:v>6d0a5ab6af78754e7109b61d7122332ba66abbdeeebd5fe8c68fffa738205394</x:v>
+      </x:c>
+      <x:c r="K184" t="str">
+        <x:v>The outline is labelled Fall 2025 and predominantly scheduled in August–December, but two week-8 entries retain March dates. The authoritative semester remains 2025h2.</x:v>
+      </x:c>
+      <x:c r="L184"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="A185" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B185" t="str">
+        <x:v>MCCCOMM311</x:v>
+      </x:c>
+      <x:c r="C185" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D185" t="str">
+        <x:v>Persuasive Communication</x:v>
+      </x:c>
+      <x:c r="E185" t="str">
+        <x:v>Studies persuasion through communication theory, social psychology and ethical analysis, with a substantial community-engaged application. Framing, cognitive shortcuts, nudging and coactive persuasion inform the design of messages for science, society and sustainability. Students work with local organizations, including Delta Climate Centre projects, to address communication challenges and produce tailored materials. Structured reflection and speech coaching connect theoretical choices to professional and community practice.</x:v>
+      </x:c>
+      <x:c r="F185" t="str">
+        <x:v>Communication studies; Rhetoric; Social psychology; Applied ethics</x:v>
+      </x:c>
+      <x:c r="G185" t="str">
+        <x:v>Psychology of persuasion; Global perspectives on persuasion; Persuasion ethics; Coactive persuasion; Verbal and nonverbal communication; Message framing; Argumentation; Cognitive shortcuts; Nudging; Climate-transition communication; Audience-sensitive public messaging; Community-engaged communication</x:v>
+      </x:c>
+      <x:c r="H185" t="str">
+        <x:v>Persuasion-framework analysis; Ethical analysis of communication; Audience-oriented message framing; Applied communication-project design; Community-engaged communication consulting; Gibbs reflective-cycle analysis; Public-speaking coaching</x:v>
+      </x:c>
+      <x:c r="I185" t="str">
+        <x:v>MCCCOMM311.docx</x:v>
+      </x:c>
+      <x:c r="J185" t="str">
+        <x:v>24bfcf4a6e7c6b22e03e0a69d3f09178fda23cefc33cc746bd2eeb1772d4c6d3</x:v>
+      </x:c>
+      <x:c r="K185"/>
+      <x:c r="L185" t="str">
+        <x:v>The communication challenge and final medium depend on each client project. Advertising, campaigning, social movements and negotiation receive a selective synopsis rather than full separate training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="A186" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B186" t="str">
+        <x:v>MCCHEAM111</x:v>
+      </x:c>
+      <x:c r="C186" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D186" t="str">
+        <x:v>Introduction to Western Art History</x:v>
+      </x:c>
+      <x:c r="E186" t="str">
+        <x:v>Surveys Western art from late medieval and early Renaissance painting to modern and contemporary movements in Europe and the Americas. Selected works and artists are studied through composition, space, form, tone and colour, alongside historical and social contexts. Students analyze paintings and art-historical scholarship, research an artist collaboratively, and develop an individual visual analysis based on direct study of a museum painting.</x:v>
+      </x:c>
+      <x:c r="F186" t="str">
+        <x:v>Art history; Visual culture studies</x:v>
+      </x:c>
+      <x:c r="G186" t="str">
+        <x:v>Late medieval Italian painting; Northern and Italian Renaissance; Mannerism; Baroque and Rococo; Enlightenment and Romanticism; Realism and Impressionism; Post-Impressionism and Symbolism; Modernism and Cubism; Interwar art; Postwar and postmodern art; Composition, space, form, tone and colour; Art institutions and historical interpretation</x:v>
+      </x:c>
+      <x:c r="H186" t="str">
+        <x:v>Formal visual analysis of paintings; Historical contextualization of artworks; Critical analysis of art-historical scholarship; Direct observation of museum artworks</x:v>
+      </x:c>
+      <x:c r="I186" t="str">
+        <x:v>MCCHEAM111.docx</x:v>
+      </x:c>
+      <x:c r="J186" t="str">
+        <x:v>6639a72e35380de81d0eb42b55a8d8f5db67c6a64f31255d520684625421d494</x:v>
+      </x:c>
+      <x:c r="K186"/>
+      <x:c r="L186"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="A187" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B187" t="str">
+        <x:v>MCCHEAM311</x:v>
+      </x:c>
+      <x:c r="C187" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D187" t="str">
+        <x:v>The Global Artefact</x:v>
+      </x:c>
+      <x:c r="E187" t="str">
+        <x:v>Examines cultural heritage as a source of value, identity, ownership claims and conflict, with this edition focused on sharing heritage. Museum history, collecting, inclusion, education and legal protection connect to looting, trade and postcolonial interpretation. Students evaluate a museum display and work with primary-school children and local collections to research meaningful objects, find historical or cross-cultural parallels, and develop an accessible exhibition and individual research paper.</x:v>
+      </x:c>
+      <x:c r="F187" t="str">
+        <x:v>Heritage studies; Museum studies; Archaeology; Material culture studies</x:v>
+      </x:c>
+      <x:c r="G187" t="str">
+        <x:v>Museum history; Collecting and object value; Heritage and identity; Cultural rights and ownership; Universalism and nationalism; Inclusive curation; Museum visitor engagement; Heritage education; Illicit antiquities trade; Heritage protection in conflict; Restitution; Postcolonial heritage interpretation; Community claims to heritage; Object narratives</x:v>
+      </x:c>
+      <x:c r="H187" t="str">
+        <x:v>Object-based material-culture research; Comparative analysis of historical and cross-cultural objects; Collection and archival research; Interviews with object owners; Museum-display evaluation; Community-engaged exhibition and heritage-education design</x:v>
+      </x:c>
+      <x:c r="I187" t="str">
+        <x:v>MCCHEAM311.docx</x:v>
+      </x:c>
+      <x:c r="J187" t="str">
+        <x:v>e1cc43c26b77d9781b7a097ab750f8c676fce0bdb96af32f675f39661137ab61</x:v>
+      </x:c>
+      <x:c r="K187" t="str">
+        <x:v>The title and body identify MCCHEAM311 The Global Artefact, while an active running header retains MCCHEAM302. Another active header reads World Heritage in Local Places; the stated edition theme is Sharing Heritage.</x:v>
+      </x:c>
+      <x:c r="L187" t="str">
+        <x:v>Sharing Heritage is the edition theme. Project arrangements with the school remain partly provisional, and the exact objects depend on the participating children.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="A188" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B188" t="str">
+        <x:v>MCCHEAM312</x:v>
+      </x:c>
+      <x:c r="C188" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D188" t="str">
+        <x:v>Modern Art &amp; Modern Museums</x:v>
+      </x:c>
+      <x:c r="E188" t="str">
+        <x:v>Examines modern and contemporary art through debates about modernism, its margins and the institutions that frame artistic meaning. Avant-garde, abstraction, figuration, conceptual and postconceptual practices lead into installation, performance, video and global contemporary art. Museum and exhibition presentation provide a recurring perspective on public understanding. Students critically compare scholarship and develop an individually researched argument supported by an annotated bibliography and sustained art-historical inquiry.</x:v>
+      </x:c>
+      <x:c r="F188" t="str">
+        <x:v>Art history; Museum studies; Modern and contemporary art studies</x:v>
+      </x:c>
+      <x:c r="G188" t="str">
+        <x:v>Modernism and avant-garde; Modernism's margins; Cubism and abstraction; Modern architecture and design; Figuration; Mexican muralism; Abstract Expressionism; Minimalism; Pop Art; Postmodernism; Conceptual and postconceptual art; Photography, installation, performance and video; Global contemporary art; Art institutions and exhibitions; Art and capitalism</x:v>
+      </x:c>
+      <x:c r="H188" t="str">
+        <x:v>Critical art-historical analysis; Comparative analysis of art movements and interpretations; Scholarly source evaluation; Annotated research bibliography development; Independent art-historical research</x:v>
+      </x:c>
+      <x:c r="I188" t="str">
+        <x:v>MCCHEAM312.docx</x:v>
+      </x:c>
+      <x:c r="J188" t="str">
+        <x:v>26794bb432d4951f26f49334171789b465a2a31071ee95f95411447a7d64476e</x:v>
+      </x:c>
+      <x:c r="K188"/>
+      <x:c r="L188" t="str">
+        <x:v>The museum and exhibition focus concerns interpretation and presentation; the outline does not specify that students curate a full exhibition.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="A189" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B189" t="str">
+        <x:v>MCCLITR111</x:v>
+      </x:c>
+      <x:c r="C189" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D189" t="str">
+        <x:v>Introduction to Literary Studies</x:v>
+      </x:c>
+      <x:c r="E189" t="str">
+        <x:v>Introduces practical criticism and literary interpretation across fiction, creative nonfiction, poetry and drama, with a short introduction to film adaptation. Students examine literary value and the constructed character of texts through plot, character, setting, narration, symbolism, style, poetic form and dramatic structure. Close reading and engagement with critical sources support a presentation and argumentative essay applying the course's analytical vocabulary.</x:v>
+      </x:c>
+      <x:c r="F189" t="str">
+        <x:v>Literary studies; Literary criticism; Narratology</x:v>
+      </x:c>
+      <x:c r="G189" t="str">
+        <x:v>Literature and literary value; Fiction and formula; Plot and story; Character and setting; Point of view; Symbolism and allegory; Graphic fiction; Tone, humour and irony; Literary style; Creative nonfiction and memoir; Microfiction; Gothic and children's literature; Poetic imagery, sound and form; Tragic drama; Film adaptation</x:v>
+      </x:c>
+      <x:c r="H189" t="str">
+        <x:v>Close reading; Formalist literary analysis; Narrative analysis; Poetry and dramatic-structure analysis; Critical-source integration; Comparative analysis of literary and film narration</x:v>
+      </x:c>
+      <x:c r="I189" t="str">
+        <x:v>MCCLITR111.docx</x:v>
+      </x:c>
+      <x:c r="J189" t="str">
+        <x:v>8dbb22040038fdfc264389ef41e5806e093deeeba0c65eae12f64d0144684d3e</x:v>
+      </x:c>
+      <x:c r="K189" t="str">
+        <x:v>One midterm-break entry retains a 2023 date amid an otherwise Fall 2025 schedule. The authoritative semester remains 2025h2.</x:v>
+      </x:c>
+      <x:c r="L189" t="str">
+        <x:v>Film adaptation receives a brief introductory treatment, not comprehensive film-studies training.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="A190" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B190" t="str">
+        <x:v>MCCLITR211</x:v>
+      </x:c>
+      <x:c r="C190" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D190" t="str">
+        <x:v>World Myth and Literature</x:v>
+      </x:c>
+      <x:c r="E190" t="str">
+        <x:v>Compares ancient and medieval literary myths across cultures, emphasizing creation, power, gender, exchange and the movement of stories between forms. Greek, Roman, Near Eastern, Indian, African and Byzantine materials are interpreted through myth theory and literary analysis. Students investigate narrative patterns and networks, explain a theory through a graphic narrative, and creatively relocate an Ovidian metamorphosis to another cultural setting with scholarly justification.</x:v>
+      </x:c>
+      <x:c r="F190" t="str">
+        <x:v>Comparative literature; Classical studies; Mythology; Gender studies</x:v>
+      </x:c>
+      <x:c r="G190" t="str">
+        <x:v>Creation and divine-succession myths; Myth theory; Structuralism; Cosmic order; Honour and guilt; Gender and exchange; Women's agency and networks; Epic and tragedy; Cross-cultural narrative parallels; Oral and visual storytelling; Literary reception; Ovidian metamorphosis; Modern retellings of ancient myth</x:v>
+      </x:c>
+      <x:c r="H190" t="str">
+        <x:v>Comparative close reading; Theory-based myth analysis; Structuralist literary analysis; Interpretation of narrative networks; Primary- and secondary-source research; Cross-cultural adaptation and performance; Scholarly analysis of creative retelling</x:v>
+      </x:c>
+      <x:c r="I190" t="str">
+        <x:v>MCCLITR211.docx</x:v>
+      </x:c>
+      <x:c r="J190" t="str">
+        <x:v>a5192ac49c68a0c4bbbce6f1f2d7f6d418c77c5912b359a67063f36944bb37dd</x:v>
+      </x:c>
+      <x:c r="K190" t="str">
+        <x:v>The schedule heading retains ANTQ202, whereas the title and authoritative filename identify MCCLITR211.</x:v>
+      </x:c>
+      <x:c r="L190" t="str">
+        <x:v>Network theory is read and applied interpretively to narratives; the outline does not establish computational network-analysis training. Several possible research approaches are optional choices.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="A191" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B191" t="str">
+        <x:v>MCCLITR311</x:v>
+      </x:c>
+      <x:c r="C191" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D191" t="str">
+        <x:v>Film and Text – topics in theory and practice of film adaptation of literature</x:v>
+      </x:c>
+      <x:c r="E191" t="str">
+        <x:v>Examines how literary works become films through relations among narrative, media form, authorship and interpretation. Formal analysis of text and film establishes tools for studying cinematography, editing, sound and performance. Fidelity, medium specificity, intertextuality and auteurism guide comparisons of selected adaptations. Students develop a theory-based research project, using literary and film fragments to investigate an independently chosen adaptation question.</x:v>
+      </x:c>
+      <x:c r="F191" t="str">
+        <x:v>Adaptation studies; Film studies; Literary studies; Narratology</x:v>
+      </x:c>
+      <x:c r="G191" t="str">
+        <x:v>Literary and film narration; Cinematography; Mise-en-scène; Editing, continuity and montage; Sound and acting; Medium specificity; Fidelity debates; Intertextuality; Auteurism; Screenplay and authorship; Heritage adaptation; Adaptation markets; Interpretation and viewer participation</x:v>
+      </x:c>
+      <x:c r="H191" t="str">
+        <x:v>Formalist literary analysis; Close analysis of film sequences; Comparative text–film analysis; Intertextual analysis; Auteur analysis</x:v>
+      </x:c>
+      <x:c r="I191" t="str">
+        <x:v>MCCLITR311.docx</x:v>
+      </x:c>
+      <x:c r="J191" t="str">
+        <x:v>3d8c2e1b740e7929c213c34a25198fc90a8a103ef66e02c8a514d82ad54180ea</x:v>
+      </x:c>
+      <x:c r="K191"/>
+      <x:c r="L191" t="str">
+        <x:v>Later sessions list suggested final-presentation topics, such as Bollywood, opera and telenovelas. These choices are not treated as guaranteed common course coverage. The practical dimension is analytical research, not specified filmmaking production.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="A192" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B192" t="str">
+        <x:v>MCCMEDI111</x:v>
+      </x:c>
+      <x:c r="C192" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D192" t="str">
+        <x:v>Introduction to Film &amp; Media</x:v>
+      </x:c>
+      <x:c r="E192" t="str">
+        <x:v>Introduces film history, form and critical interpretation, with a shorter extension into wider media. Early cinema, Expressionism, montage, Hollywood and new waves provide material for analyzing narrative, cinematography, editing, sound and spectatorship. Media histories, convergence, power and diasporic cinema connect film to broader cultural and political contexts. Students apply theory to close readings and complete a focused research or creative-analytical project.</x:v>
+      </x:c>
+      <x:c r="F192" t="str">
+        <x:v>Film studies; Media studies; Visual culture studies</x:v>
+      </x:c>
+      <x:c r="G192" t="str">
+        <x:v>Early cinema; German Expressionism; Soviet montage; Hollywood cinema; European new waves; Film narrative and form; Cinematography, editing and sound; Spectatorship and the gaze; Gender and representation; Media histories; Convergence culture; Media power and politics; Global and diasporic cinema</x:v>
+      </x:c>
+      <x:c r="H192" t="str">
+        <x:v>Close analysis of film sequences; Formal film analysis; Historical and cultural contextualization; Theory-based media interpretation</x:v>
+      </x:c>
+      <x:c r="I192" t="str">
+        <x:v>MCCMEDI111.pdf</x:v>
+      </x:c>
+      <x:c r="J192" t="str">
+        <x:v>03e4960f2905cc4e770807b292d4d499632c8ef7f2ab5992d12c8ec2e16adeb7</x:v>
+      </x:c>
+      <x:c r="K192" t="str">
+        <x:v>The outline consistently prints MCCMED111, whereas the authoritative filename code is MCCMEDI111.</x:v>
+      </x:c>
+      <x:c r="L192" t="str">
+        <x:v>The course primarily develops film analysis; broader media receive introductory coverage. The final project can be a research essay or creative-analytical work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="A193" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B193" t="str">
+        <x:v>MCCMEDI112</x:v>
+      </x:c>
+      <x:c r="C193" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D193" t="str">
+        <x:v>Media Archaeology</x:v>
+      </x:c>
+      <x:c r="E193" t="str">
+        <x:v>Examines obsolete and pre-digital media as material and cultural evidence of how knowledge is produced, circulated and preserved. Media-archaeological theory and histories of print, electrical communication and audiovisual technologies connect physical form to communication, memory and experience. Students closely examine media objects and undertake independent research, using material analysis and historical interpretation to relate earlier technologies to contemporary media culture.</x:v>
+      </x:c>
+      <x:c r="F193" t="str">
+        <x:v>Media studies; Media archaeology; Media history; Material culture studies</x:v>
+      </x:c>
+      <x:c r="G193" t="str">
+        <x:v>Media materiality; Obsolescence; Knowledge production and preservation; Communication and memory; Media-archaeological theory; Histories of print and electrical communication; Sound recording and fidelity; Audiovisual media; Cassette culture; Portable listening; Historical and contemporary media relations</x:v>
+      </x:c>
+      <x:c r="H193" t="str">
+        <x:v>Material analysis of historical media objects; Media-archaeological interpretation; Historical and cultural contextualization</x:v>
+      </x:c>
+      <x:c r="I193" t="str">
+        <x:v>MCCMEDI112.pdf</x:v>
+      </x:c>
+      <x:c r="J193" t="str">
+        <x:v>2a1336fa049d69cdd24f3764eff2443949a6b486162af1e5830c8b723070d962</x:v>
+      </x:c>
+      <x:c r="K193" t="str">
+        <x:v>The outline consistently prints MCCMED112, whereas the authoritative filename code is MCCMEDI112.</x:v>
+      </x:c>
+      <x:c r="L193" t="str">
+        <x:v>Recording silence, examining cassette hiss and studying the Walkman are possible practical activities, not fixed exercises. The supplied schedule is preliminary and detailed project protocols are provided separately.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="A194" t="str">
+        <x:v>2025h2</x:v>
+      </x:c>
+      <x:c r="B194" t="str">
+        <x:v>MCCMEDI311</x:v>
+      </x:c>
+      <x:c r="C194" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D194" t="str">
+        <x:v>Media and Race: A Cultural History</x:v>
+      </x:c>
+      <x:c r="E194" t="str">
+        <x:v>Studies how media sustains and challenges racialized power in American history from the late nineteenth century to the present. Cultural narratives connect national identity, crime, health, exclusion, class, childhood and Indigenous experience to resistance and imagined futures. Students analyze primary cultural and archival sources alongside scholarship, develop a thesis-driven research paper, and produce a podcast examining contemporary social identities and inequalities.</x:v>
+      </x:c>
+      <x:c r="F194" t="str">
+        <x:v>Cultural history; Media studies; Race and ethnic studies; American studies</x:v>
+      </x:c>
+      <x:c r="G194" t="str">
+        <x:v>Race, whiteness and national identity; Media and systemic racism; Crime and punishment; Racial segregation; Medical racism; Afrofuturism and Indigenous futurisms; Inclusion and exclusion; Japanese American internment; Class and childhood; Work and politics; Tourism and white-saviour narratives; Indigenous identities; Storytelling and resistance</x:v>
+      </x:c>
+      <x:c r="H194" t="str">
+        <x:v>Historical primary-source analysis; Critical interpretation of film, photography, literature and music; Archival or cultural-text research; Analysis of futurist cultural works; Research-based podcast production</x:v>
+      </x:c>
+      <x:c r="I194" t="str">
+        <x:v>MCCMEDI311.docx</x:v>
+      </x:c>
+      <x:c r="J194" t="str">
+        <x:v>23f9d346f35e04cb8906167297bf8d323761465caf24e9963c551b7a52a1e702</x:v>
+      </x:c>
+      <x:c r="K194" t="str">
+        <x:v>The outline heading retains AH-Hist308, whereas the authoritative filename code is MCCMEDI311.</x:v>
+      </x:c>
+      <x:c r="L194" t="str">
+        <x:v>The paper can analyze a RIAS archival collection or a futurist cultural work; both paths are not compulsory. Specific podcast subjects and production formats are chosen by students.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Append two user-supplied Spring 2027 course outlines
</commit_message>
<xml_diff>
--- a/course-outline-database/UCR_Course_Outline_Database.xlsx
+++ b/course-outline-database/UCR_Course_Outline_Database.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="1" r:id="R775fb38698454fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="1" r:id="R95d7596415f84a00"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11767,6 +11767,78 @@
         <x:v>Specific cultural-presentation topics are not supplied. The textbook title refers to A2, but the outline does not explicitly establish an achieved CEFR level; none is assigned.</x:v>
       </x:c>
     </x:row>
+    <x:row r="198">
+      <x:c r="A198" t="str">
+        <x:v>2027h1</x:v>
+      </x:c>
+      <x:c r="B198" t="str">
+        <x:v>BENBUSI312</x:v>
+      </x:c>
+      <x:c r="C198" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D198" t="str">
+        <x:v>Money, Banking and Finance</x:v>
+      </x:c>
+      <x:c r="E198" t="str">
+        <x:v>Examines financial markets and institutions, including the pricing of bonds, stocks and derivatives, interest rates and their risk and term structure, commercial-bank balance sheets and performance, financial structure and regulation, banking fragility and financial crises, central banks, money creation and monetary policy. Students apply algebraic and graphical analysis to financial and monetary problems. In the Stanford Banking Game they manage a simulated bank, analyse performance in Excel dashboards, forecast financial statements, and make evidence-based decisions about loans, deposits, capital, liquidity and risk. A small research project extends a selected financial or monetary research article through additional literature, a case study or updated evidence.</x:v>
+      </x:c>
+      <x:c r="F198" t="str">
+        <x:v>Finance; Monetary economics; Banking</x:v>
+      </x:c>
+      <x:c r="G198" t="str">
+        <x:v>Financial markets and institutions; Bond, stock and derivative pricing; Interest-rate determination; Interest-rate risk and the term structure; Commercial-bank balance sheets and performance; Bank capital, liquidity and risk management; Financial structure and regulation; Banking fragility; Financial crises in advanced and emerging economies; Central banking; Money supply; Monetary-policy tools and conduct</x:v>
+      </x:c>
+      <x:c r="H198" t="str">
+        <x:v>Algebraic and graphical financial analysis; Balance-sheet analysis; Duration gap analysis; Bank-management simulation (Stanford Banking Game); Excel-based financial dashboard construction and performance analysis; Financial-statement forecasting; Research-article extension using literature comparison, case study or updated data</x:v>
+      </x:c>
+      <x:c r="I198" t="str">
+        <x:v>BENBUSI312.pdf</x:v>
+      </x:c>
+      <x:c r="J198" t="str">
+        <x:v>27c1aa64633a97a85da9de8ae2d19d0567b4fc4deb3373f82e4441c161ebefc9</x:v>
+      </x:c>
+      <x:c r="K198" t="str">
+        <x:v>User supplied this file as a Spring 2027 outline (2027h1). The cover identifies SSCECON209 Money, Banking and Finance, Spring 2022 (2022-1), dated 18 April 2022, and the schedule also uses 2022 dates. The supplied filename BENBUSI312.pdf and user-confirmed semester are retained as the authoritative key.</x:v>
+      </x:c>
+      <x:c r="L198"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="A199" t="str">
+        <x:v>2027h1</x:v>
+      </x:c>
+      <x:c r="B199" t="str">
+        <x:v>BENLEAD211</x:v>
+      </x:c>
+      <x:c r="C199" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D199" t="str">
+        <x:v>Leading Under Pressure: The Psychology of Emotion Regulation, Diversity and Leadership</x:v>
+      </x:c>
+      <x:c r="E199" t="str">
+        <x:v>Examines how emotion regulation, emotional intelligence, emotional expression and suppression, emotional labor, belonging, identity safety and psychological safety shape leadership and social interaction under conflict, exclusion and interpersonal uncertainty. It emphasises inclusive leadership and ethnic, cultural, sexual and gender minority experiences, with digital emotion regulation as a further strand. Students conduct a supervised quantitative survey project: formulating theory-driven hypotheses, selecting established psychological measures, designing and piloting a Qualtrics survey, recruiting participants ethically, collecting original data and preparing a clean dataset. Individual work applies descriptive statistics, reliability analysis, correlations, group comparisons and introductory multiple regression in SPSS or RStudio, and interprets findings and limitations in empirical reports and evidence-based leadership recommendations.</x:v>
+      </x:c>
+      <x:c r="F199" t="str">
+        <x:v>Leadership studies; Social psychology; Work and organizational psychology; Psychological measurement; Quantitative social research</x:v>
+      </x:c>
+      <x:c r="G199" t="str">
+        <x:v>Emotion regulation strategies; Emotional intelligence; Emotional expression and suppression; Emotional labor; Inclusive leadership; Belonging and identity safety; Psychological safety; Ethnic, cultural, sexual and gender minority experiences; Digital emotion regulation; Psychological measurement, reliability and validity; Ethical survey research in diverse populations; Interpretation and limitations of quantitative evidence; Evidence-based leadership recommendations</x:v>
+      </x:c>
+      <x:c r="H199" t="str">
+        <x:v>Theory-driven hypothesis formulation; Quantitative survey research; Established psychological measure selection and evaluation; Qualtrics survey construction and piloting; Ethical participant recruitment and original data collection; Codebook development, reverse coding and scale scoring; Data cleaning and missing-data documentation; Descriptive statistics; Reliability analysis; Correlation analysis; Group comparisons; Introductory multiple regression in SPSS or RStudio; APA-style empirical reporting</x:v>
+      </x:c>
+      <x:c r="I199" t="str">
+        <x:v>BENLEAD211.pdf</x:v>
+      </x:c>
+      <x:c r="J199" t="str">
+        <x:v>b371a30312e82f1f2b34c214f17c83aca9780d503b31f0d30cad0cd08e641d6f</x:v>
+      </x:c>
+      <x:c r="K199"/>
+      <x:c r="L199" t="str">
+        <x:v>The supplied document is a Spring 2027 course proposal; it states that an extended outline in the required UCR format will follow. Collaboration with local institutions and employee recruitment remain subject to formal agreement, ethical approval, feasibility and voluntary participation. Exploratory factor analysis is optional and conditional on the research question, sample size and student preparation; it is not included as a required method.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>